<commit_message>
Integrated Index fix changes and run testing
</commit_message>
<xml_diff>
--- a/tests/regression_test/results/master_results.xlsx
+++ b/tests/regression_test/results/master_results.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17340" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AllVersions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="AllVersions" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:R23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -430,6 +430,11 @@
           <t>TOC HiL</t>
         </is>
       </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Index Fixes</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -487,6 +492,31 @@
           <t>data-science</t>
         </is>
       </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>algorithms</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>cybersec</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>data-science</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -544,6 +574,31 @@
           <t>data-science</t>
         </is>
       </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>algorithms</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>cybersec</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>data-science</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -601,6 +656,31 @@
           <t>multi-metric</t>
         </is>
       </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -658,6 +738,31 @@
           <t>2025-10-11T15:43:07.024072</t>
         </is>
       </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>2025-10-11T19:16:34.393385</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>2025-10-11T18:14:29.155825</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>2025-10-11T18:14:29.138669</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2025-10-11T18:14:29.168733</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>2025-10-11T18:14:29.180316</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -695,6 +800,21 @@
       <c r="L6" t="n">
         <v>1.5</v>
       </c>
+      <c r="N6" t="n">
+        <v>-53.7</v>
+      </c>
+      <c r="O6" t="n">
+        <v>-35.9</v>
+      </c>
+      <c r="P6" t="n">
+        <v>62</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>-88.7</v>
+      </c>
+      <c r="R6" t="n">
+        <v>-2.8</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -732,6 +852,21 @@
       <c r="L7" t="n">
         <v>0</v>
       </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
+        <v>2</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>1</v>
+      </c>
+      <c r="R7" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -769,6 +904,21 @@
       <c r="L8" t="n">
         <v>0</v>
       </c>
+      <c r="N8" t="n">
+        <v>2</v>
+      </c>
+      <c r="O8" t="n">
+        <v>4</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>7</v>
+      </c>
+      <c r="R8" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -806,6 +956,21 @@
       <c r="L9" t="n">
         <v>-1</v>
       </c>
+      <c r="N9" t="n">
+        <v>-1</v>
+      </c>
+      <c r="O9" t="n">
+        <v>-1</v>
+      </c>
+      <c r="P9" t="n">
+        <v>-1</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>-1</v>
+      </c>
+      <c r="R9" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -843,6 +1008,21 @@
       <c r="L10" t="n">
         <v>106</v>
       </c>
+      <c r="N10" t="n">
+        <v>233</v>
+      </c>
+      <c r="O10" t="n">
+        <v>49</v>
+      </c>
+      <c r="P10" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>101</v>
+      </c>
+      <c r="R10" t="n">
+        <v>106</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -880,6 +1060,21 @@
       <c r="L11" t="n">
         <v>92</v>
       </c>
+      <c r="N11" t="n">
+        <v>195</v>
+      </c>
+      <c r="O11" t="n">
+        <v>27</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>12</v>
+      </c>
+      <c r="R11" t="n">
+        <v>88</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -917,6 +1112,21 @@
       <c r="L12" t="n">
         <v>13</v>
       </c>
+      <c r="N12" t="n">
+        <v>14</v>
+      </c>
+      <c r="O12" t="n">
+        <v>22</v>
+      </c>
+      <c r="P12" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>21</v>
+      </c>
+      <c r="R12" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -954,6 +1164,21 @@
       <c r="L13" t="n">
         <v>16</v>
       </c>
+      <c r="N13" t="n">
+        <v>4</v>
+      </c>
+      <c r="O13" t="n">
+        <v>12</v>
+      </c>
+      <c r="P13" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>12</v>
+      </c>
+      <c r="R13" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -991,6 +1216,21 @@
       <c r="L14" t="n">
         <v>105</v>
       </c>
+      <c r="N14" t="n">
+        <v>97</v>
+      </c>
+      <c r="O14" t="n">
+        <v>200</v>
+      </c>
+      <c r="P14" t="n">
+        <v>126</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>80</v>
+      </c>
+      <c r="R14" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1028,6 +1268,21 @@
       <c r="L15" t="n">
         <v>182</v>
       </c>
+      <c r="N15" t="n">
+        <v>207</v>
+      </c>
+      <c r="O15" t="n">
+        <v>350</v>
+      </c>
+      <c r="P15" t="n">
+        <v>131</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>171</v>
+      </c>
+      <c r="R15" t="n">
+        <v>179</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1065,6 +1320,21 @@
       <c r="L16" t="n">
         <v>179</v>
       </c>
+      <c r="N16" t="n">
+        <v>108</v>
+      </c>
+      <c r="O16" t="n">
+        <v>126</v>
+      </c>
+      <c r="P16" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>169</v>
+      </c>
+      <c r="R16" t="n">
+        <v>179</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1102,6 +1372,21 @@
       <c r="L17" t="n">
         <v>195</v>
       </c>
+      <c r="N17" t="n">
+        <v>100</v>
+      </c>
+      <c r="O17" t="n">
+        <v>122</v>
+      </c>
+      <c r="P17" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>267</v>
+      </c>
+      <c r="R17" t="n">
+        <v>197</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1139,6 +1424,21 @@
       <c r="L18" t="n">
         <v>178</v>
       </c>
+      <c r="N18" t="n">
+        <v>56</v>
+      </c>
+      <c r="O18" t="n">
+        <v>251</v>
+      </c>
+      <c r="P18" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>93</v>
+      </c>
+      <c r="R18" t="n">
+        <v>178</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1176,6 +1476,21 @@
       <c r="L19" t="n">
         <v>164</v>
       </c>
+      <c r="N19" t="n">
+        <v>142</v>
+      </c>
+      <c r="O19" t="n">
+        <v>191</v>
+      </c>
+      <c r="P19" t="n">
+        <v>48</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>153</v>
+      </c>
+      <c r="R19" t="n">
+        <v>159</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1213,6 +1528,21 @@
       <c r="L20" t="n">
         <v>74</v>
       </c>
+      <c r="N20" t="n">
+        <v>71</v>
+      </c>
+      <c r="O20" t="n">
+        <v>32</v>
+      </c>
+      <c r="P20" t="n">
+        <v>32</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>49</v>
+      </c>
+      <c r="R20" t="n">
+        <v>74</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1250,6 +1580,21 @@
       <c r="L21" t="n">
         <v>1</v>
       </c>
+      <c r="N21" t="n">
+        <v>16</v>
+      </c>
+      <c r="O21" t="n">
+        <v>9</v>
+      </c>
+      <c r="P21" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>21</v>
+      </c>
+      <c r="R21" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1287,6 +1632,21 @@
       <c r="L22" t="n">
         <v>-1</v>
       </c>
+      <c r="N22" t="n">
+        <v>-1</v>
+      </c>
+      <c r="O22" t="n">
+        <v>-1</v>
+      </c>
+      <c r="P22" t="n">
+        <v>-1</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>-1</v>
+      </c>
+      <c r="R22" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1324,11 +1684,27 @@
       <c r="L23" t="n">
         <v>862</v>
       </c>
+      <c r="N23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" t="n">
+        <v>529</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>6</v>
+      </c>
+      <c r="R23" t="n">
+        <v>862</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="H1:L1"/>
     <mergeCell ref="B1:F1"/>
+    <mergeCell ref="N1:R1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Excel sheets show colors
</commit_message>
<xml_diff>
--- a/tests/regression_test/results/master_results.xlsx
+++ b/tests/regression_test/results/master_results.xlsx
@@ -25,12 +25,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -45,12 +57,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -740,7 +754,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2025-10-11T19:16:34.393385</t>
+          <t>2025-10-12T21:40:36.187519</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -785,34 +799,34 @@
       <c r="F6" t="n">
         <v>-65.59999999999999</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" s="3" t="n">
         <v>-50.4</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I6" s="3" t="n">
         <v>-31.4</v>
       </c>
-      <c r="J6" t="n">
+      <c r="J6" s="3" t="n">
         <v>63.5</v>
       </c>
-      <c r="K6" t="n">
+      <c r="K6" s="4" t="n">
         <v>-268.2</v>
       </c>
-      <c r="L6" t="n">
+      <c r="L6" s="3" t="n">
         <v>1.5</v>
       </c>
-      <c r="N6" t="n">
+      <c r="N6" s="4" t="n">
         <v>-53.7</v>
       </c>
-      <c r="O6" t="n">
+      <c r="O6" s="4" t="n">
         <v>-35.9</v>
       </c>
-      <c r="P6" t="n">
+      <c r="P6" s="4" t="n">
         <v>62</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="Q6" s="3" t="n">
         <v>-88.7</v>
       </c>
-      <c r="R6" t="n">
+      <c r="R6" s="4" t="n">
         <v>-2.8</v>
       </c>
     </row>
@@ -837,34 +851,34 @@
       <c r="F7" t="n">
         <v>113</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="I7" t="n">
+      <c r="I7" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="J7" t="n">
+      <c r="J7" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="K7" t="n">
+      <c r="K7" s="4" t="n">
         <v>349</v>
       </c>
-      <c r="L7" t="n">
+      <c r="L7" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="N7" t="n">
+      <c r="N7" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="O7" t="n">
+      <c r="O7" s="3" t="n">
         <v>2</v>
       </c>
       <c r="P7" t="n">
         <v>0</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="Q7" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="R7" t="n">
+      <c r="R7" s="4" t="n">
         <v>2</v>
       </c>
     </row>
@@ -889,22 +903,22 @@
       <c r="F8" t="n">
         <v>121</v>
       </c>
-      <c r="H8" t="n">
+      <c r="H8" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="I8" t="n">
+      <c r="I8" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="J8" t="n">
+      <c r="J8" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="K8" t="n">
+      <c r="K8" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="L8" t="n">
+      <c r="L8" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="N8" t="n">
+      <c r="N8" s="3" t="n">
         <v>2</v>
       </c>
       <c r="O8" t="n">
@@ -913,10 +927,10 @@
       <c r="P8" t="n">
         <v>0</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="Q8" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="R8" t="n">
+      <c r="R8" s="4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -996,7 +1010,7 @@
       <c r="H10" t="n">
         <v>233</v>
       </c>
-      <c r="I10" t="n">
+      <c r="I10" s="4" t="n">
         <v>40</v>
       </c>
       <c r="J10" t="n">
@@ -1011,7 +1025,7 @@
       <c r="N10" t="n">
         <v>233</v>
       </c>
-      <c r="O10" t="n">
+      <c r="O10" s="3" t="n">
         <v>49</v>
       </c>
       <c r="P10" t="n">
@@ -1045,25 +1059,25 @@
       <c r="F11" t="n">
         <v>93</v>
       </c>
-      <c r="H11" t="n">
+      <c r="H11" s="3" t="n">
         <v>236</v>
       </c>
-      <c r="I11" t="n">
+      <c r="I11" s="4" t="n">
         <v>20</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
       </c>
-      <c r="K11" t="n">
+      <c r="K11" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="L11" t="n">
+      <c r="L11" s="4" t="n">
         <v>92</v>
       </c>
-      <c r="N11" t="n">
+      <c r="N11" s="4" t="n">
         <v>195</v>
       </c>
-      <c r="O11" t="n">
+      <c r="O11" s="3" t="n">
         <v>27</v>
       </c>
       <c r="P11" t="n">
@@ -1072,7 +1086,7 @@
       <c r="Q11" t="n">
         <v>12</v>
       </c>
-      <c r="R11" t="n">
+      <c r="R11" s="4" t="n">
         <v>88</v>
       </c>
     </row>
@@ -1149,10 +1163,10 @@
       <c r="F13" t="n">
         <v>16</v>
       </c>
-      <c r="H13" t="n">
+      <c r="H13" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="I13" t="n">
+      <c r="I13" s="4" t="n">
         <v>10</v>
       </c>
       <c r="J13" t="n">
@@ -1167,13 +1181,13 @@
       <c r="N13" t="n">
         <v>4</v>
       </c>
-      <c r="O13" t="n">
+      <c r="O13" s="3" t="n">
         <v>12</v>
       </c>
       <c r="P13" t="n">
         <v>2</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="Q13" s="3" t="n">
         <v>12</v>
       </c>
       <c r="R13" t="n">
@@ -1253,34 +1267,34 @@
       <c r="F15" t="n">
         <v>180</v>
       </c>
-      <c r="H15" t="n">
+      <c r="H15" s="3" t="n">
         <v>208</v>
       </c>
-      <c r="I15" t="n">
+      <c r="I15" s="3" t="n">
         <v>342</v>
       </c>
-      <c r="J15" t="n">
+      <c r="J15" s="4" t="n">
         <v>131</v>
       </c>
-      <c r="K15" t="n">
+      <c r="K15" s="4" t="n">
         <v>170</v>
       </c>
-      <c r="L15" t="n">
+      <c r="L15" s="3" t="n">
         <v>182</v>
       </c>
-      <c r="N15" t="n">
+      <c r="N15" s="4" t="n">
         <v>207</v>
       </c>
-      <c r="O15" t="n">
+      <c r="O15" s="3" t="n">
         <v>350</v>
       </c>
       <c r="P15" t="n">
         <v>131</v>
       </c>
-      <c r="Q15" t="n">
+      <c r="Q15" s="3" t="n">
         <v>171</v>
       </c>
-      <c r="R15" t="n">
+      <c r="R15" s="4" t="n">
         <v>179</v>
       </c>
     </row>
@@ -1357,10 +1371,10 @@
       <c r="F17" t="n">
         <v>195</v>
       </c>
-      <c r="H17" t="n">
+      <c r="H17" s="4" t="n">
         <v>109</v>
       </c>
-      <c r="I17" t="n">
+      <c r="I17" s="4" t="n">
         <v>123</v>
       </c>
       <c r="J17" t="n">
@@ -1372,19 +1386,19 @@
       <c r="L17" t="n">
         <v>195</v>
       </c>
-      <c r="N17" t="n">
+      <c r="N17" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="O17" t="n">
+      <c r="O17" s="4" t="n">
         <v>122</v>
       </c>
       <c r="P17" t="n">
         <v>15</v>
       </c>
-      <c r="Q17" t="n">
+      <c r="Q17" s="4" t="n">
         <v>267</v>
       </c>
-      <c r="R17" t="n">
+      <c r="R17" s="3" t="n">
         <v>197</v>
       </c>
     </row>
@@ -1461,34 +1475,34 @@
       <c r="F19" t="n">
         <v>159</v>
       </c>
-      <c r="H19" t="n">
+      <c r="H19" s="3" t="n">
         <v>178</v>
       </c>
-      <c r="I19" t="n">
+      <c r="I19" s="3" t="n">
         <v>194</v>
       </c>
-      <c r="J19" t="n">
+      <c r="J19" s="4" t="n">
         <v>48</v>
       </c>
-      <c r="K19" t="n">
+      <c r="K19" s="3" t="n">
         <v>154</v>
       </c>
-      <c r="L19" t="n">
+      <c r="L19" s="3" t="n">
         <v>164</v>
       </c>
-      <c r="N19" t="n">
+      <c r="N19" s="4" t="n">
         <v>142</v>
       </c>
-      <c r="O19" t="n">
+      <c r="O19" s="4" t="n">
         <v>191</v>
       </c>
       <c r="P19" t="n">
         <v>48</v>
       </c>
-      <c r="Q19" t="n">
+      <c r="Q19" s="4" t="n">
         <v>153</v>
       </c>
-      <c r="R19" t="n">
+      <c r="R19" s="4" t="n">
         <v>159</v>
       </c>
     </row>
@@ -1565,34 +1579,34 @@
       <c r="F21" t="n">
         <v>6</v>
       </c>
-      <c r="H21" t="n">
+      <c r="H21" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="I21" t="n">
+      <c r="I21" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="J21" t="n">
+      <c r="J21" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="K21" t="n">
+      <c r="K21" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="L21" t="n">
+      <c r="L21" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N21" t="n">
+      <c r="N21" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="O21" t="n">
+      <c r="O21" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="P21" t="n">
+      <c r="P21" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="Q21" t="n">
+      <c r="Q21" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="R21" t="n">
+      <c r="R21" s="3" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added average column to the excel sheet and updated excel
</commit_message>
<xml_diff>
--- a/tests/regression_test/results/master_results.xlsx
+++ b/tests/regression_test/results/master_results.xlsx
@@ -57,11 +57,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -430,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R23"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,12 +440,12 @@
           <t>original</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>TOC HiL</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Index Fixes</t>
         </is>
@@ -481,54 +482,69 @@
           <t>data-science</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>avg.</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>ai</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>algorithms</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>assembly</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>cybersec</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>data-science</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t>avg.</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
           <t>ai</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>algorithms</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>assembly</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>cybersec</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>data-science</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>avg.</t>
         </is>
       </c>
     </row>
@@ -563,52 +579,52 @@
           <t>data-science</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>ai</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>algorithms</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>assembly</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>cybersec</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>data-science</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>ai</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>algorithms</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>assembly</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>cybersec</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>data-science</t>
         </is>
@@ -645,52 +661,52 @@
           <t>multi-metric</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>multi-metric</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>multi-metric</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>multi-metric</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>multi-metric</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>multi-metric</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>multi-metric</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>multi-metric</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>multi-metric</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>multi-metric</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>multi-metric</t>
         </is>
@@ -704,7 +720,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2025-10-11T16:57:42.842778</t>
+          <t>2025-10-12T22:05:27.639126</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -727,52 +743,52 @@
           <t>2025-10-11T16:57:42.954007</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2025-10-11T15:43:07.037316</t>
-        </is>
-      </c>
       <c r="I5" t="inlineStr">
         <is>
+          <t>2025-10-12T22:03:24.930038</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
           <t>2025-10-11T15:43:07.047282</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>2025-10-11T15:43:07.060044</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>2025-10-11T15:43:07.067553</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>2025-10-11T15:43:07.024072</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>2025-10-12T21:40:36.187519</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>2025-10-12T22:19:55.496723</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>2025-10-11T18:14:29.155825</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>2025-10-11T18:14:29.138669</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>2025-10-11T18:14:29.168733</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>2025-10-11T18:14:29.180316</t>
         </is>
@@ -799,35 +815,44 @@
       <c r="F6" t="n">
         <v>-65.59999999999999</v>
       </c>
-      <c r="H6" s="3" t="n">
+      <c r="G6" t="n">
+        <v>-83.66000000000001</v>
+      </c>
+      <c r="I6" s="4" t="n">
         <v>-50.4</v>
       </c>
-      <c r="I6" s="3" t="n">
+      <c r="J6" s="4" t="n">
         <v>-31.4</v>
       </c>
-      <c r="J6" s="3" t="n">
+      <c r="K6" s="4" t="n">
         <v>63.5</v>
       </c>
-      <c r="K6" s="4" t="n">
+      <c r="L6" s="5" t="n">
         <v>-268.2</v>
       </c>
-      <c r="L6" s="3" t="n">
+      <c r="M6" s="4" t="n">
         <v>1.5</v>
       </c>
       <c r="N6" s="4" t="n">
+        <v>-57</v>
+      </c>
+      <c r="P6" s="5" t="n">
         <v>-53.7</v>
       </c>
-      <c r="O6" s="4" t="n">
+      <c r="Q6" s="5" t="n">
         <v>-35.9</v>
       </c>
-      <c r="P6" s="4" t="n">
+      <c r="R6" s="5" t="n">
         <v>62</v>
       </c>
-      <c r="Q6" s="3" t="n">
+      <c r="S6" s="4" t="n">
         <v>-88.7</v>
       </c>
-      <c r="R6" s="4" t="n">
+      <c r="T6" s="5" t="n">
         <v>-2.8</v>
+      </c>
+      <c r="U6" s="4" t="n">
+        <v>-23.82</v>
       </c>
     </row>
     <row r="7">
@@ -851,34 +876,34 @@
       <c r="F7" t="n">
         <v>113</v>
       </c>
-      <c r="H7" s="3" t="n">
+      <c r="I7" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I7" s="3" t="n">
+      <c r="J7" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="J7" s="3" t="n">
+      <c r="K7" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="K7" s="4" t="n">
+      <c r="L7" s="5" t="n">
         <v>349</v>
       </c>
-      <c r="L7" s="3" t="n">
+      <c r="M7" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="N7" s="3" t="n">
+      <c r="P7" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O7" s="3" t="n">
+      <c r="Q7" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="P7" t="n">
+      <c r="R7" t="n">
         <v>0</v>
       </c>
-      <c r="Q7" s="3" t="n">
+      <c r="S7" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R7" s="4" t="n">
+      <c r="T7" s="5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -903,34 +928,34 @@
       <c r="F8" t="n">
         <v>121</v>
       </c>
-      <c r="H8" s="3" t="n">
+      <c r="I8" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="I8" s="3" t="n">
+      <c r="J8" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="J8" s="3" t="n">
+      <c r="K8" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="K8" s="3" t="n">
+      <c r="L8" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="L8" s="3" t="n">
+      <c r="M8" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="N8" s="3" t="n">
+      <c r="P8" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="O8" t="n">
+      <c r="Q8" t="n">
         <v>4</v>
       </c>
-      <c r="P8" t="n">
+      <c r="R8" t="n">
         <v>0</v>
       </c>
-      <c r="Q8" s="3" t="n">
+      <c r="S8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="R8" s="4" t="n">
+      <c r="T8" s="5" t="n">
         <v>3</v>
       </c>
     </row>
@@ -955,9 +980,6 @@
       <c r="F9" t="n">
         <v>-1</v>
       </c>
-      <c r="H9" t="n">
-        <v>-1</v>
-      </c>
       <c r="I9" t="n">
         <v>-1</v>
       </c>
@@ -970,10 +992,7 @@
       <c r="L9" t="n">
         <v>-1</v>
       </c>
-      <c r="N9" t="n">
-        <v>-1</v>
-      </c>
-      <c r="O9" t="n">
+      <c r="M9" t="n">
         <v>-1</v>
       </c>
       <c r="P9" t="n">
@@ -983,6 +1002,12 @@
         <v>-1</v>
       </c>
       <c r="R9" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S9" t="n">
+        <v>-1</v>
+      </c>
+      <c r="T9" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -1007,34 +1032,34 @@
       <c r="F10" t="n">
         <v>106</v>
       </c>
-      <c r="H10" t="n">
+      <c r="I10" t="n">
         <v>233</v>
       </c>
-      <c r="I10" s="4" t="n">
+      <c r="J10" s="5" t="n">
         <v>40</v>
       </c>
-      <c r="J10" t="n">
+      <c r="K10" t="n">
         <v>3</v>
       </c>
-      <c r="K10" t="n">
+      <c r="L10" t="n">
         <v>101</v>
       </c>
-      <c r="L10" t="n">
+      <c r="M10" t="n">
         <v>106</v>
       </c>
-      <c r="N10" t="n">
+      <c r="P10" t="n">
         <v>233</v>
       </c>
-      <c r="O10" s="3" t="n">
+      <c r="Q10" s="4" t="n">
         <v>49</v>
       </c>
-      <c r="P10" t="n">
+      <c r="R10" t="n">
         <v>3</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="S10" t="n">
         <v>101</v>
       </c>
-      <c r="R10" t="n">
+      <c r="T10" t="n">
         <v>106</v>
       </c>
     </row>
@@ -1059,34 +1084,34 @@
       <c r="F11" t="n">
         <v>93</v>
       </c>
-      <c r="H11" s="3" t="n">
+      <c r="I11" s="4" t="n">
         <v>236</v>
       </c>
-      <c r="I11" s="4" t="n">
+      <c r="J11" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="J11" t="n">
+      <c r="K11" t="n">
         <v>0</v>
       </c>
-      <c r="K11" s="4" t="n">
+      <c r="L11" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="L11" s="4" t="n">
+      <c r="M11" s="5" t="n">
         <v>92</v>
       </c>
-      <c r="N11" s="4" t="n">
+      <c r="P11" s="5" t="n">
         <v>195</v>
       </c>
-      <c r="O11" s="3" t="n">
+      <c r="Q11" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="P11" t="n">
+      <c r="R11" t="n">
         <v>0</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="S11" t="n">
         <v>12</v>
       </c>
-      <c r="R11" s="4" t="n">
+      <c r="T11" s="5" t="n">
         <v>88</v>
       </c>
     </row>
@@ -1111,34 +1136,34 @@
       <c r="F12" t="n">
         <v>13</v>
       </c>
-      <c r="H12" t="n">
+      <c r="I12" t="n">
         <v>14</v>
       </c>
-      <c r="I12" t="n">
+      <c r="J12" t="n">
         <v>22</v>
       </c>
-      <c r="J12" t="n">
+      <c r="K12" t="n">
         <v>16</v>
       </c>
-      <c r="K12" t="n">
+      <c r="L12" t="n">
         <v>21</v>
       </c>
-      <c r="L12" t="n">
+      <c r="M12" t="n">
         <v>13</v>
       </c>
-      <c r="N12" t="n">
+      <c r="P12" t="n">
         <v>14</v>
       </c>
-      <c r="O12" t="n">
+      <c r="Q12" t="n">
         <v>22</v>
       </c>
-      <c r="P12" t="n">
+      <c r="R12" t="n">
         <v>16</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="S12" t="n">
         <v>21</v>
       </c>
-      <c r="R12" t="n">
+      <c r="T12" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1163,34 +1188,34 @@
       <c r="F13" t="n">
         <v>16</v>
       </c>
-      <c r="H13" s="3" t="n">
+      <c r="I13" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="I13" s="4" t="n">
+      <c r="J13" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="J13" t="n">
+      <c r="K13" t="n">
         <v>2</v>
       </c>
-      <c r="K13" t="n">
+      <c r="L13" t="n">
         <v>10</v>
       </c>
-      <c r="L13" t="n">
+      <c r="M13" t="n">
         <v>16</v>
       </c>
-      <c r="N13" t="n">
+      <c r="P13" t="n">
         <v>4</v>
       </c>
-      <c r="O13" s="3" t="n">
+      <c r="Q13" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="P13" t="n">
+      <c r="R13" t="n">
         <v>2</v>
       </c>
-      <c r="Q13" s="3" t="n">
+      <c r="S13" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="R13" t="n">
+      <c r="T13" t="n">
         <v>16</v>
       </c>
     </row>
@@ -1215,34 +1240,34 @@
       <c r="F14" t="n">
         <v>105</v>
       </c>
-      <c r="H14" t="n">
+      <c r="I14" t="n">
         <v>97</v>
       </c>
-      <c r="I14" t="n">
+      <c r="J14" t="n">
         <v>200</v>
       </c>
-      <c r="J14" t="n">
+      <c r="K14" t="n">
         <v>126</v>
       </c>
-      <c r="K14" t="n">
+      <c r="L14" t="n">
         <v>80</v>
       </c>
-      <c r="L14" t="n">
+      <c r="M14" t="n">
         <v>105</v>
       </c>
-      <c r="N14" t="n">
+      <c r="P14" t="n">
         <v>97</v>
       </c>
-      <c r="O14" t="n">
+      <c r="Q14" t="n">
         <v>200</v>
       </c>
-      <c r="P14" t="n">
+      <c r="R14" t="n">
         <v>126</v>
       </c>
-      <c r="Q14" t="n">
+      <c r="S14" t="n">
         <v>80</v>
       </c>
-      <c r="R14" t="n">
+      <c r="T14" t="n">
         <v>105</v>
       </c>
     </row>
@@ -1267,34 +1292,34 @@
       <c r="F15" t="n">
         <v>180</v>
       </c>
-      <c r="H15" s="3" t="n">
+      <c r="I15" s="4" t="n">
         <v>208</v>
       </c>
-      <c r="I15" s="3" t="n">
+      <c r="J15" s="4" t="n">
         <v>342</v>
       </c>
-      <c r="J15" s="4" t="n">
+      <c r="K15" s="5" t="n">
         <v>131</v>
       </c>
-      <c r="K15" s="4" t="n">
+      <c r="L15" s="5" t="n">
         <v>170</v>
       </c>
-      <c r="L15" s="3" t="n">
+      <c r="M15" s="4" t="n">
         <v>182</v>
       </c>
-      <c r="N15" s="4" t="n">
+      <c r="P15" s="5" t="n">
         <v>207</v>
       </c>
-      <c r="O15" s="3" t="n">
+      <c r="Q15" s="4" t="n">
         <v>350</v>
       </c>
-      <c r="P15" t="n">
+      <c r="R15" t="n">
         <v>131</v>
       </c>
-      <c r="Q15" s="3" t="n">
+      <c r="S15" s="4" t="n">
         <v>171</v>
       </c>
-      <c r="R15" s="4" t="n">
+      <c r="T15" s="5" t="n">
         <v>179</v>
       </c>
     </row>
@@ -1319,34 +1344,34 @@
       <c r="F16" t="n">
         <v>179</v>
       </c>
-      <c r="H16" t="n">
+      <c r="I16" t="n">
         <v>108</v>
       </c>
-      <c r="I16" t="n">
+      <c r="J16" t="n">
         <v>126</v>
       </c>
-      <c r="J16" t="n">
+      <c r="K16" t="n">
         <v>12</v>
       </c>
-      <c r="K16" t="n">
+      <c r="L16" t="n">
         <v>169</v>
       </c>
-      <c r="L16" t="n">
+      <c r="M16" t="n">
         <v>179</v>
       </c>
-      <c r="N16" t="n">
+      <c r="P16" t="n">
         <v>108</v>
       </c>
-      <c r="O16" t="n">
+      <c r="Q16" t="n">
         <v>126</v>
       </c>
-      <c r="P16" t="n">
+      <c r="R16" t="n">
         <v>12</v>
       </c>
-      <c r="Q16" t="n">
+      <c r="S16" t="n">
         <v>169</v>
       </c>
-      <c r="R16" t="n">
+      <c r="T16" t="n">
         <v>179</v>
       </c>
     </row>
@@ -1371,34 +1396,34 @@
       <c r="F17" t="n">
         <v>195</v>
       </c>
-      <c r="H17" s="4" t="n">
+      <c r="I17" s="5" t="n">
         <v>109</v>
       </c>
-      <c r="I17" s="4" t="n">
+      <c r="J17" s="5" t="n">
         <v>123</v>
       </c>
-      <c r="J17" t="n">
+      <c r="K17" t="n">
         <v>15</v>
       </c>
-      <c r="K17" t="n">
+      <c r="L17" t="n">
         <v>268</v>
       </c>
-      <c r="L17" t="n">
+      <c r="M17" t="n">
         <v>195</v>
       </c>
-      <c r="N17" s="4" t="n">
+      <c r="P17" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="O17" s="4" t="n">
+      <c r="Q17" s="5" t="n">
         <v>122</v>
       </c>
-      <c r="P17" t="n">
+      <c r="R17" t="n">
         <v>15</v>
       </c>
-      <c r="Q17" s="4" t="n">
+      <c r="S17" s="5" t="n">
         <v>267</v>
       </c>
-      <c r="R17" s="3" t="n">
+      <c r="T17" s="4" t="n">
         <v>197</v>
       </c>
     </row>
@@ -1423,34 +1448,34 @@
       <c r="F18" t="n">
         <v>178</v>
       </c>
-      <c r="H18" t="n">
+      <c r="I18" t="n">
         <v>56</v>
       </c>
-      <c r="I18" t="n">
+      <c r="J18" t="n">
         <v>251</v>
       </c>
-      <c r="J18" t="n">
+      <c r="K18" t="n">
         <v>16</v>
       </c>
-      <c r="K18" t="n">
+      <c r="L18" t="n">
         <v>93</v>
       </c>
-      <c r="L18" t="n">
+      <c r="M18" t="n">
         <v>178</v>
       </c>
-      <c r="N18" t="n">
+      <c r="P18" t="n">
         <v>56</v>
       </c>
-      <c r="O18" t="n">
+      <c r="Q18" t="n">
         <v>251</v>
       </c>
-      <c r="P18" t="n">
+      <c r="R18" t="n">
         <v>16</v>
       </c>
-      <c r="Q18" t="n">
+      <c r="S18" t="n">
         <v>93</v>
       </c>
-      <c r="R18" t="n">
+      <c r="T18" t="n">
         <v>178</v>
       </c>
     </row>
@@ -1475,34 +1500,34 @@
       <c r="F19" t="n">
         <v>159</v>
       </c>
-      <c r="H19" s="3" t="n">
+      <c r="I19" s="4" t="n">
         <v>178</v>
       </c>
-      <c r="I19" s="3" t="n">
+      <c r="J19" s="4" t="n">
         <v>194</v>
       </c>
-      <c r="J19" s="4" t="n">
+      <c r="K19" s="5" t="n">
         <v>48</v>
       </c>
-      <c r="K19" s="3" t="n">
+      <c r="L19" s="4" t="n">
         <v>154</v>
       </c>
-      <c r="L19" s="3" t="n">
+      <c r="M19" s="4" t="n">
         <v>164</v>
       </c>
-      <c r="N19" s="4" t="n">
+      <c r="P19" s="5" t="n">
         <v>142</v>
       </c>
-      <c r="O19" s="4" t="n">
+      <c r="Q19" s="5" t="n">
         <v>191</v>
       </c>
-      <c r="P19" t="n">
+      <c r="R19" t="n">
         <v>48</v>
       </c>
-      <c r="Q19" s="4" t="n">
+      <c r="S19" s="5" t="n">
         <v>153</v>
       </c>
-      <c r="R19" s="4" t="n">
+      <c r="T19" s="5" t="n">
         <v>159</v>
       </c>
     </row>
@@ -1527,34 +1552,34 @@
       <c r="F20" t="n">
         <v>74</v>
       </c>
-      <c r="H20" t="n">
+      <c r="I20" t="n">
         <v>71</v>
-      </c>
-      <c r="I20" t="n">
-        <v>32</v>
       </c>
       <c r="J20" t="n">
         <v>32</v>
       </c>
       <c r="K20" t="n">
+        <v>32</v>
+      </c>
+      <c r="L20" t="n">
         <v>49</v>
       </c>
-      <c r="L20" t="n">
+      <c r="M20" t="n">
         <v>74</v>
       </c>
-      <c r="N20" t="n">
+      <c r="P20" t="n">
         <v>71</v>
       </c>
-      <c r="O20" t="n">
+      <c r="Q20" t="n">
         <v>32</v>
       </c>
-      <c r="P20" t="n">
+      <c r="R20" t="n">
         <v>32</v>
       </c>
-      <c r="Q20" t="n">
+      <c r="S20" t="n">
         <v>49</v>
       </c>
-      <c r="R20" t="n">
+      <c r="T20" t="n">
         <v>74</v>
       </c>
     </row>
@@ -1579,34 +1604,34 @@
       <c r="F21" t="n">
         <v>6</v>
       </c>
-      <c r="H21" s="3" t="n">
+      <c r="I21" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="I21" s="3" t="n">
+      <c r="J21" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="J21" s="3" t="n">
+      <c r="K21" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="K21" s="4" t="n">
+      <c r="L21" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="L21" s="4" t="n">
+      <c r="M21" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="N21" s="4" t="n">
+      <c r="P21" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="O21" s="4" t="n">
+      <c r="Q21" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="P21" s="4" t="n">
+      <c r="R21" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="Q21" s="3" t="n">
+      <c r="S21" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="R21" s="3" t="n">
+      <c r="T21" s="4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1631,9 +1656,6 @@
       <c r="F22" t="n">
         <v>-1</v>
       </c>
-      <c r="H22" t="n">
-        <v>-1</v>
-      </c>
       <c r="I22" t="n">
         <v>-1</v>
       </c>
@@ -1646,10 +1668,7 @@
       <c r="L22" t="n">
         <v>-1</v>
       </c>
-      <c r="N22" t="n">
-        <v>-1</v>
-      </c>
-      <c r="O22" t="n">
+      <c r="M22" t="n">
         <v>-1</v>
       </c>
       <c r="P22" t="n">
@@ -1659,6 +1678,12 @@
         <v>-1</v>
       </c>
       <c r="R22" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S22" t="n">
+        <v>-1</v>
+      </c>
+      <c r="T22" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -1683,42 +1708,42 @@
       <c r="F23" t="n">
         <v>862</v>
       </c>
-      <c r="H23" t="n">
+      <c r="I23" t="n">
         <v>0</v>
       </c>
-      <c r="I23" t="n">
+      <c r="J23" t="n">
         <v>529</v>
       </c>
-      <c r="J23" t="n">
+      <c r="K23" t="n">
         <v>0</v>
       </c>
-      <c r="K23" t="n">
+      <c r="L23" t="n">
         <v>6</v>
       </c>
-      <c r="L23" t="n">
+      <c r="M23" t="n">
         <v>862</v>
-      </c>
-      <c r="N23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O23" t="n">
-        <v>529</v>
       </c>
       <c r="P23" t="n">
         <v>0</v>
       </c>
       <c r="Q23" t="n">
+        <v>529</v>
+      </c>
+      <c r="R23" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" t="n">
         <v>6</v>
       </c>
-      <c r="R23" t="n">
+      <c r="T23" t="n">
         <v>862</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="H1:L1"/>
+    <mergeCell ref="P1:U1"/>
+    <mergeCell ref="I1:N1"/>
     <mergeCell ref="B1:F1"/>
-    <mergeCell ref="N1:R1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test results from balance check
</commit_message>
<xml_diff>
--- a/tests/regression_test/results/master_results.xlsx
+++ b/tests/regression_test/results/master_results.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V23"/>
+  <dimension ref="A1:AB23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,6 +450,11 @@
           <t>Index Fixes</t>
         </is>
       </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>balance-checker</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -547,6 +552,36 @@
           <t>avg.</t>
         </is>
       </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>algorithms</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>cybersec</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>data-science</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>avg.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -629,6 +664,31 @@
           <t>data-science</t>
         </is>
       </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>algorithms</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>cybersec</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>data-science</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -711,6 +771,31 @@
           <t>multi-metric</t>
         </is>
       </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -793,6 +878,31 @@
           <t>2025-10-11T18:14:29.180316</t>
         </is>
       </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>2025-10-13T14:29:48.552114</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>2025-10-13T14:29:48.629250</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>2025-10-13T14:29:48.595294</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>2025-10-13T14:29:48.676909</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>2025-10-13T14:29:48.719281</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -854,6 +964,24 @@
       <c r="U6" s="4" t="n">
         <v>-23.82</v>
       </c>
+      <c r="W6" s="5" t="n">
+        <v>-60.2</v>
+      </c>
+      <c r="X6" s="5" t="n">
+        <v>-151.7</v>
+      </c>
+      <c r="Y6" s="5" t="n">
+        <v>-12.6</v>
+      </c>
+      <c r="Z6" s="5" t="n">
+        <v>-139.3</v>
+      </c>
+      <c r="AA6" s="5" t="n">
+        <v>-25.8</v>
+      </c>
+      <c r="AB6" s="5" t="n">
+        <v>-77.92</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -906,6 +1034,21 @@
       <c r="T7" s="5" t="n">
         <v>2</v>
       </c>
+      <c r="W7" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="X7" s="5" t="n">
+        <v>176</v>
+      </c>
+      <c r="Y7" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z7" s="5" t="n">
+        <v>82</v>
+      </c>
+      <c r="AA7" s="5" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -958,6 +1101,21 @@
       <c r="T8" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="W8" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="X8" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="Y8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z8" s="5" t="n">
+        <v>73</v>
+      </c>
+      <c r="AA8" s="5" t="n">
+        <v>93</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1010,6 +1168,21 @@
       <c r="T9" t="n">
         <v>-1</v>
       </c>
+      <c r="W9" t="n">
+        <v>-1</v>
+      </c>
+      <c r="X9" t="n">
+        <v>-1</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>-1</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1062,6 +1235,21 @@
       <c r="T10" t="n">
         <v>106</v>
       </c>
+      <c r="W10" t="n">
+        <v>233</v>
+      </c>
+      <c r="X10" s="4" t="n">
+        <v>57</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>101</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>106</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1114,6 +1302,21 @@
       <c r="T11" s="5" t="n">
         <v>88</v>
       </c>
+      <c r="W11" s="4" t="n">
+        <v>232</v>
+      </c>
+      <c r="X11" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z11" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="AA11" s="5" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1166,6 +1369,21 @@
       <c r="T12" t="n">
         <v>13</v>
       </c>
+      <c r="W12" t="n">
+        <v>14</v>
+      </c>
+      <c r="X12" t="n">
+        <v>22</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>16</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>21</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1218,6 +1436,21 @@
       <c r="T13" t="n">
         <v>16</v>
       </c>
+      <c r="W13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X13" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="Y13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z13" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="AA13" s="5" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1270,6 +1503,21 @@
       <c r="T14" t="n">
         <v>105</v>
       </c>
+      <c r="W14" t="n">
+        <v>97</v>
+      </c>
+      <c r="X14" t="n">
+        <v>200</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>126</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>80</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1322,6 +1570,21 @@
       <c r="T15" s="5" t="n">
         <v>179</v>
       </c>
+      <c r="W15" s="5" t="n">
+        <v>137</v>
+      </c>
+      <c r="X15" s="5" t="n">
+        <v>194</v>
+      </c>
+      <c r="Y15" s="5" t="n">
+        <v>89</v>
+      </c>
+      <c r="Z15" s="5" t="n">
+        <v>147</v>
+      </c>
+      <c r="AA15" s="5" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1374,6 +1637,21 @@
       <c r="T16" t="n">
         <v>179</v>
       </c>
+      <c r="W16" t="n">
+        <v>108</v>
+      </c>
+      <c r="X16" t="n">
+        <v>126</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>12</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>169</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>179</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1426,6 +1704,21 @@
       <c r="T17" s="4" t="n">
         <v>197</v>
       </c>
+      <c r="W17" s="4" t="n">
+        <v>203</v>
+      </c>
+      <c r="X17" s="4" t="n">
+        <v>310</v>
+      </c>
+      <c r="Y17" s="4" t="n">
+        <v>122</v>
+      </c>
+      <c r="Z17" s="4" t="n">
+        <v>335</v>
+      </c>
+      <c r="AA17" s="4" t="n">
+        <v>265</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1478,6 +1771,21 @@
       <c r="T18" t="n">
         <v>178</v>
       </c>
+      <c r="W18" t="n">
+        <v>56</v>
+      </c>
+      <c r="X18" t="n">
+        <v>251</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>16</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>93</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>178</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1530,6 +1838,21 @@
       <c r="T19" s="5" t="n">
         <v>159</v>
       </c>
+      <c r="W19" s="4" t="n">
+        <v>153</v>
+      </c>
+      <c r="X19" s="5" t="n">
+        <v>190</v>
+      </c>
+      <c r="Y19" s="4" t="n">
+        <v>66</v>
+      </c>
+      <c r="Z19" s="4" t="n">
+        <v>157</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>159</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1582,6 +1905,21 @@
       <c r="T20" t="n">
         <v>74</v>
       </c>
+      <c r="W20" t="n">
+        <v>71</v>
+      </c>
+      <c r="X20" t="n">
+        <v>32</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>32</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>49</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>74</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1634,6 +1972,21 @@
       <c r="T21" s="4" t="n">
         <v>3</v>
       </c>
+      <c r="W21" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="X21" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="Y21" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="Z21" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="AA21" s="4" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1686,6 +2039,21 @@
       <c r="T22" t="n">
         <v>-1</v>
       </c>
+      <c r="W22" t="n">
+        <v>-1</v>
+      </c>
+      <c r="X22" t="n">
+        <v>-1</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>-1</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1738,11 +2106,27 @@
       <c r="T23" t="n">
         <v>862</v>
       </c>
+      <c r="W23" t="n">
+        <v>0</v>
+      </c>
+      <c r="X23" s="5" t="n">
+        <v>528</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>862</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="P1:U1"/>
     <mergeCell ref="I1:N1"/>
+    <mergeCell ref="W1:AB1"/>
     <mergeCell ref="B1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
trying to analyse logs and fix based on biggest errors
</commit_message>
<xml_diff>
--- a/tests/regression_test/results/master_results.xlsx
+++ b/tests/regression_test/results/master_results.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW87"/>
+  <dimension ref="A1:BK87"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30.83203125" customWidth="1" style="4" min="1" max="1"/>
@@ -486,6 +486,16 @@
           <t>manual_images</t>
         </is>
       </c>
+      <c r="AY1" s="3" t="inlineStr">
+        <is>
+          <t>use-microtype</t>
+        </is>
+      </c>
+      <c r="BF1" s="3" t="inlineStr">
+        <is>
+          <t>nesting-depth</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -703,6 +713,66 @@
           <t>avg.</t>
         </is>
       </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>algorithms</t>
+        </is>
+      </c>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="BB2" t="inlineStr">
+        <is>
+          <t>cybersec</t>
+        </is>
+      </c>
+      <c r="BC2" t="inlineStr">
+        <is>
+          <t>data-science</t>
+        </is>
+      </c>
+      <c r="BD2" t="inlineStr">
+        <is>
+          <t>avg.</t>
+        </is>
+      </c>
+      <c r="BF2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="BG2" t="inlineStr">
+        <is>
+          <t>algorithms</t>
+        </is>
+      </c>
+      <c r="BH2" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="BI2" t="inlineStr">
+        <is>
+          <t>cybersec</t>
+        </is>
+      </c>
+      <c r="BJ2" t="inlineStr">
+        <is>
+          <t>data-science</t>
+        </is>
+      </c>
+      <c r="BK2" t="inlineStr">
+        <is>
+          <t>avg.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -885,6 +955,56 @@
           <t>data-science</t>
         </is>
       </c>
+      <c r="AY3" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="AZ3" t="inlineStr">
+        <is>
+          <t>algorithms</t>
+        </is>
+      </c>
+      <c r="BA3" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="BB3" t="inlineStr">
+        <is>
+          <t>cybersec</t>
+        </is>
+      </c>
+      <c r="BC3" t="inlineStr">
+        <is>
+          <t>data-science</t>
+        </is>
+      </c>
+      <c r="BF3" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="BG3" t="inlineStr">
+        <is>
+          <t>algorithms</t>
+        </is>
+      </c>
+      <c r="BH3" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="BI3" t="inlineStr">
+        <is>
+          <t>cybersec</t>
+        </is>
+      </c>
+      <c r="BJ3" t="inlineStr">
+        <is>
+          <t>data-science</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1067,6 +1187,56 @@
           <t>multi-metric</t>
         </is>
       </c>
+      <c r="AY4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="AZ4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="BA4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="BB4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="BC4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="BF4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="BG4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="BH4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="BI4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="BJ4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1249,6 +1419,56 @@
           <t>2025-10-24T23:26:57.639562</t>
         </is>
       </c>
+      <c r="AY5" t="inlineStr">
+        <is>
+          <t>2025-10-25T12:02:57.335066</t>
+        </is>
+      </c>
+      <c r="AZ5" t="inlineStr">
+        <is>
+          <t>2025-10-25T12:02:57.551118</t>
+        </is>
+      </c>
+      <c r="BA5" t="inlineStr">
+        <is>
+          <t>2025-10-25T12:02:57.493368</t>
+        </is>
+      </c>
+      <c r="BB5" t="inlineStr">
+        <is>
+          <t>2025-10-25T12:02:57.678508</t>
+        </is>
+      </c>
+      <c r="BC5" t="inlineStr">
+        <is>
+          <t>2025-10-25T12:02:57.750748</t>
+        </is>
+      </c>
+      <c r="BF5" t="inlineStr">
+        <is>
+          <t>2025-10-25T15:59:21.354930</t>
+        </is>
+      </c>
+      <c r="BG5" t="inlineStr">
+        <is>
+          <t>2025-10-25T15:59:21.585615</t>
+        </is>
+      </c>
+      <c r="BH5" t="inlineStr">
+        <is>
+          <t>2025-10-25T15:59:21.494610</t>
+        </is>
+      </c>
+      <c r="BI5" t="inlineStr">
+        <is>
+          <t>2025-10-25T15:59:21.692455</t>
+        </is>
+      </c>
+      <c r="BJ5" t="inlineStr">
+        <is>
+          <t>2025-10-25T15:59:21.762269</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1382,6 +1602,42 @@
       <c r="AW6" s="6" t="n">
         <v>-531.8599999999999</v>
       </c>
+      <c r="AY6" s="6" t="n">
+        <v>-585.4</v>
+      </c>
+      <c r="AZ6" s="6" t="n">
+        <v>-1059.3</v>
+      </c>
+      <c r="BA6" s="6" t="n">
+        <v>-256.3</v>
+      </c>
+      <c r="BB6" s="6" t="n">
+        <v>-908.8</v>
+      </c>
+      <c r="BC6" s="6" t="n">
+        <v>-397.7</v>
+      </c>
+      <c r="BD6" s="6" t="n">
+        <v>-641.5</v>
+      </c>
+      <c r="BF6" s="5" t="n">
+        <v>-526.2</v>
+      </c>
+      <c r="BG6" s="5" t="n">
+        <v>-1051.6</v>
+      </c>
+      <c r="BH6" s="5" t="n">
+        <v>-251.4</v>
+      </c>
+      <c r="BI6" s="5" t="n">
+        <v>-839.8</v>
+      </c>
+      <c r="BJ6" s="5" t="n">
+        <v>-322.6</v>
+      </c>
+      <c r="BK6" s="5" t="n">
+        <v>-598.3199999999999</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1494,6 +1750,36 @@
       <c r="AV7" t="n">
         <v>100</v>
       </c>
+      <c r="AY7" s="6" t="n">
+        <v>68.06999999999999</v>
+      </c>
+      <c r="AZ7" s="6" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="BA7" t="n">
+        <v>100</v>
+      </c>
+      <c r="BB7" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="BC7" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF7" s="5" t="n">
+        <v>87.11</v>
+      </c>
+      <c r="BG7" s="5" t="n">
+        <v>65.88</v>
+      </c>
+      <c r="BH7" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI7" t="n">
+        <v>100</v>
+      </c>
+      <c r="BJ7" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1606,6 +1892,36 @@
       <c r="AV8" s="6" t="n">
         <v>160</v>
       </c>
+      <c r="AY8" s="6" t="n">
+        <v>176.2891141472014</v>
+      </c>
+      <c r="AZ8" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="BA8" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="BB8" s="6" t="n">
+        <v>484</v>
+      </c>
+      <c r="BC8" s="6" t="n">
+        <v>301</v>
+      </c>
+      <c r="BF8" s="5" t="n">
+        <v>13.77568591436115</v>
+      </c>
+      <c r="BG8" s="5" t="n">
+        <v>7.58955676988464</v>
+      </c>
+      <c r="BH8" t="n">
+        <v>16</v>
+      </c>
+      <c r="BI8" s="5" t="n">
+        <v>358</v>
+      </c>
+      <c r="BJ8" s="5" t="n">
+        <v>163</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1718,6 +2034,36 @@
       <c r="AV9" s="6" t="n">
         <v>234</v>
       </c>
+      <c r="AY9" s="5" t="n">
+        <v>260.0264433671221</v>
+      </c>
+      <c r="AZ9" s="6" t="n">
+        <v>99.2</v>
+      </c>
+      <c r="BA9" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="BB9" s="6" t="n">
+        <v>152</v>
+      </c>
+      <c r="BC9" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="BF9" s="5" t="n">
+        <v>143.4967282745953</v>
+      </c>
+      <c r="BG9" s="5" t="n">
+        <v>15.17911353976928</v>
+      </c>
+      <c r="BH9" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="BI9" s="5" t="n">
+        <v>92</v>
+      </c>
+      <c r="BJ9" s="5" t="n">
+        <v>114</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1830,6 +2176,36 @@
       <c r="AV10" t="n">
         <v>106</v>
       </c>
+      <c r="AY10" t="n">
+        <v>233</v>
+      </c>
+      <c r="AZ10" t="n">
+        <v>906</v>
+      </c>
+      <c r="BA10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB10" t="n">
+        <v>101</v>
+      </c>
+      <c r="BC10" t="n">
+        <v>106</v>
+      </c>
+      <c r="BF10" t="n">
+        <v>233</v>
+      </c>
+      <c r="BG10" t="n">
+        <v>906</v>
+      </c>
+      <c r="BH10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BI10" t="n">
+        <v>101</v>
+      </c>
+      <c r="BJ10" t="n">
+        <v>106</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1942,6 +2318,36 @@
       <c r="AV11" t="n">
         <v>106</v>
       </c>
+      <c r="AY11" t="n">
+        <v>233</v>
+      </c>
+      <c r="AZ11" t="n">
+        <v>57</v>
+      </c>
+      <c r="BA11" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB11" t="n">
+        <v>101</v>
+      </c>
+      <c r="BC11" t="n">
+        <v>106</v>
+      </c>
+      <c r="BF11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG11" t="n">
+        <v>57</v>
+      </c>
+      <c r="BH11" t="n">
+        <v>3</v>
+      </c>
+      <c r="BI11" t="n">
+        <v>101</v>
+      </c>
+      <c r="BJ11" t="n">
+        <v>106</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2054,6 +2460,36 @@
       <c r="AV12" t="n">
         <v>92</v>
       </c>
+      <c r="AY12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ12" t="n">
+        <v>51</v>
+      </c>
+      <c r="BA12" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB12" t="n">
+        <v>101</v>
+      </c>
+      <c r="BC12" t="n">
+        <v>92</v>
+      </c>
+      <c r="BF12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG12" t="n">
+        <v>51</v>
+      </c>
+      <c r="BH12" t="n">
+        <v>3</v>
+      </c>
+      <c r="BI12" t="n">
+        <v>101</v>
+      </c>
+      <c r="BJ12" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2166,6 +2602,36 @@
       <c r="AV13" t="n">
         <v>0</v>
       </c>
+      <c r="AY13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ13" t="n">
+        <v>849</v>
+      </c>
+      <c r="BA13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF13" s="6" t="n">
+        <v>233</v>
+      </c>
+      <c r="BG13" t="n">
+        <v>849</v>
+      </c>
+      <c r="BH13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2278,6 +2744,36 @@
       <c r="AV14" t="n">
         <v>14</v>
       </c>
+      <c r="AY14" s="6" t="n">
+        <v>233</v>
+      </c>
+      <c r="AZ14" t="n">
+        <v>6</v>
+      </c>
+      <c r="BA14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC14" t="n">
+        <v>14</v>
+      </c>
+      <c r="BF14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG14" t="n">
+        <v>6</v>
+      </c>
+      <c r="BH14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI14" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ14" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2390,6 +2886,36 @@
       <c r="AV15" t="n">
         <v>13</v>
       </c>
+      <c r="AY15" t="n">
+        <v>14</v>
+      </c>
+      <c r="AZ15" t="n">
+        <v>22</v>
+      </c>
+      <c r="BA15" t="n">
+        <v>16</v>
+      </c>
+      <c r="BB15" t="n">
+        <v>21</v>
+      </c>
+      <c r="BC15" t="n">
+        <v>13</v>
+      </c>
+      <c r="BF15" t="n">
+        <v>14</v>
+      </c>
+      <c r="BG15" t="n">
+        <v>22</v>
+      </c>
+      <c r="BH15" t="n">
+        <v>16</v>
+      </c>
+      <c r="BI15" t="n">
+        <v>21</v>
+      </c>
+      <c r="BJ15" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2502,6 +3028,36 @@
       <c r="AV16" s="5" t="n">
         <v>17</v>
       </c>
+      <c r="AY16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2616,6 +3172,36 @@
       <c r="AV17" s="5" t="n">
         <v>-4</v>
       </c>
+      <c r="AY17" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="AZ17" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="BA17" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="BB17" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="BC17" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="BF17" t="n">
+        <v>14</v>
+      </c>
+      <c r="BG17" t="n">
+        <v>22</v>
+      </c>
+      <c r="BH17" t="n">
+        <v>16</v>
+      </c>
+      <c r="BI17" t="n">
+        <v>21</v>
+      </c>
+      <c r="BJ17" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2728,6 +3314,36 @@
       <c r="AV18" t="n">
         <v>105</v>
       </c>
+      <c r="AY18" t="n">
+        <v>97</v>
+      </c>
+      <c r="AZ18" t="n">
+        <v>200</v>
+      </c>
+      <c r="BA18" t="n">
+        <v>126</v>
+      </c>
+      <c r="BB18" t="n">
+        <v>80</v>
+      </c>
+      <c r="BC18" t="n">
+        <v>105</v>
+      </c>
+      <c r="BF18" t="n">
+        <v>97</v>
+      </c>
+      <c r="BG18" t="n">
+        <v>200</v>
+      </c>
+      <c r="BH18" t="n">
+        <v>126</v>
+      </c>
+      <c r="BI18" t="n">
+        <v>80</v>
+      </c>
+      <c r="BJ18" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2840,6 +3456,36 @@
       <c r="AV19" s="5" t="n">
         <v>178</v>
       </c>
+      <c r="AY19" s="6" t="n">
+        <v>129</v>
+      </c>
+      <c r="AZ19" s="6" t="n">
+        <v>223</v>
+      </c>
+      <c r="BA19" s="6" t="n">
+        <v>96</v>
+      </c>
+      <c r="BB19" s="6" t="n">
+        <v>146</v>
+      </c>
+      <c r="BC19" s="6" t="n">
+        <v>136</v>
+      </c>
+      <c r="BF19" t="n">
+        <v>129</v>
+      </c>
+      <c r="BG19" t="n">
+        <v>223</v>
+      </c>
+      <c r="BH19" t="n">
+        <v>96</v>
+      </c>
+      <c r="BI19" t="n">
+        <v>146</v>
+      </c>
+      <c r="BJ19" t="n">
+        <v>136</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2952,6 +3598,36 @@
       <c r="AV20" s="6" t="n">
         <v>-73</v>
       </c>
+      <c r="AY20" s="5" t="n">
+        <v>-32</v>
+      </c>
+      <c r="AZ20" s="5" t="n">
+        <v>-23</v>
+      </c>
+      <c r="BA20" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="BB20" s="5" t="n">
+        <v>-66</v>
+      </c>
+      <c r="BC20" s="5" t="n">
+        <v>-31</v>
+      </c>
+      <c r="BF20" t="n">
+        <v>-32</v>
+      </c>
+      <c r="BG20" t="n">
+        <v>-23</v>
+      </c>
+      <c r="BH20" t="n">
+        <v>30</v>
+      </c>
+      <c r="BI20" t="n">
+        <v>-66</v>
+      </c>
+      <c r="BJ20" t="n">
+        <v>-31</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3064,6 +3740,36 @@
       <c r="AV21" t="n">
         <v>179</v>
       </c>
+      <c r="AY21" t="n">
+        <v>108</v>
+      </c>
+      <c r="AZ21" t="n">
+        <v>126</v>
+      </c>
+      <c r="BA21" t="n">
+        <v>12</v>
+      </c>
+      <c r="BB21" t="n">
+        <v>169</v>
+      </c>
+      <c r="BC21" t="n">
+        <v>179</v>
+      </c>
+      <c r="BF21" t="n">
+        <v>108</v>
+      </c>
+      <c r="BG21" t="n">
+        <v>126</v>
+      </c>
+      <c r="BH21" t="n">
+        <v>12</v>
+      </c>
+      <c r="BI21" t="n">
+        <v>169</v>
+      </c>
+      <c r="BJ21" t="n">
+        <v>179</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3176,6 +3882,36 @@
       <c r="AV22" s="6" t="n">
         <v>195</v>
       </c>
+      <c r="AY22" s="5" t="n">
+        <v>190</v>
+      </c>
+      <c r="AZ22" s="5" t="n">
+        <v>314</v>
+      </c>
+      <c r="BA22" s="5" t="n">
+        <v>122</v>
+      </c>
+      <c r="BB22" s="5" t="n">
+        <v>349</v>
+      </c>
+      <c r="BC22" s="5" t="n">
+        <v>270</v>
+      </c>
+      <c r="BF22" t="n">
+        <v>190</v>
+      </c>
+      <c r="BG22" t="n">
+        <v>314</v>
+      </c>
+      <c r="BH22" t="n">
+        <v>122</v>
+      </c>
+      <c r="BI22" t="n">
+        <v>349</v>
+      </c>
+      <c r="BJ22" t="n">
+        <v>270</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3288,6 +4024,36 @@
       <c r="AV23" s="5" t="n">
         <v>-16</v>
       </c>
+      <c r="AY23" s="6" t="n">
+        <v>-82</v>
+      </c>
+      <c r="AZ23" s="6" t="n">
+        <v>-188</v>
+      </c>
+      <c r="BA23" s="6" t="n">
+        <v>-110</v>
+      </c>
+      <c r="BB23" s="6" t="n">
+        <v>-180</v>
+      </c>
+      <c r="BC23" s="6" t="n">
+        <v>-91</v>
+      </c>
+      <c r="BF23" t="n">
+        <v>-82</v>
+      </c>
+      <c r="BG23" t="n">
+        <v>-188</v>
+      </c>
+      <c r="BH23" t="n">
+        <v>-110</v>
+      </c>
+      <c r="BI23" t="n">
+        <v>-180</v>
+      </c>
+      <c r="BJ23" t="n">
+        <v>-91</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3400,6 +4166,36 @@
       <c r="AV24" t="n">
         <v>178</v>
       </c>
+      <c r="AY24" t="n">
+        <v>56</v>
+      </c>
+      <c r="AZ24" t="n">
+        <v>251</v>
+      </c>
+      <c r="BA24" t="n">
+        <v>16</v>
+      </c>
+      <c r="BB24" t="n">
+        <v>93</v>
+      </c>
+      <c r="BC24" t="n">
+        <v>178</v>
+      </c>
+      <c r="BF24" t="n">
+        <v>56</v>
+      </c>
+      <c r="BG24" t="n">
+        <v>251</v>
+      </c>
+      <c r="BH24" t="n">
+        <v>16</v>
+      </c>
+      <c r="BI24" t="n">
+        <v>93</v>
+      </c>
+      <c r="BJ24" t="n">
+        <v>178</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3512,6 +4308,36 @@
       <c r="AV25" s="5" t="n">
         <v>158</v>
       </c>
+      <c r="AY25" t="n">
+        <v>158</v>
+      </c>
+      <c r="AZ25" t="n">
+        <v>64</v>
+      </c>
+      <c r="BA25" t="n">
+        <v>67</v>
+      </c>
+      <c r="BB25" t="n">
+        <v>155</v>
+      </c>
+      <c r="BC25" t="n">
+        <v>158</v>
+      </c>
+      <c r="BF25" t="n">
+        <v>158</v>
+      </c>
+      <c r="BG25" t="n">
+        <v>64</v>
+      </c>
+      <c r="BH25" t="n">
+        <v>67</v>
+      </c>
+      <c r="BI25" t="n">
+        <v>155</v>
+      </c>
+      <c r="BJ25" t="n">
+        <v>158</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3624,6 +4450,36 @@
       <c r="AV26" t="n">
         <v>172</v>
       </c>
+      <c r="AY26" t="n">
+        <v>182</v>
+      </c>
+      <c r="AZ26" t="n">
+        <v>68</v>
+      </c>
+      <c r="BA26" t="n">
+        <v>67</v>
+      </c>
+      <c r="BB26" t="n">
+        <v>155</v>
+      </c>
+      <c r="BC26" t="n">
+        <v>172</v>
+      </c>
+      <c r="BF26" t="n">
+        <v>182</v>
+      </c>
+      <c r="BG26" t="n">
+        <v>68</v>
+      </c>
+      <c r="BH26" t="n">
+        <v>67</v>
+      </c>
+      <c r="BI26" t="n">
+        <v>155</v>
+      </c>
+      <c r="BJ26" t="n">
+        <v>172</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3736,6 +4592,36 @@
       <c r="AV27" s="6" t="n">
         <v>-152</v>
       </c>
+      <c r="AY27" t="n">
+        <v>-284</v>
+      </c>
+      <c r="AZ27" t="n">
+        <v>119</v>
+      </c>
+      <c r="BA27" t="n">
+        <v>-118</v>
+      </c>
+      <c r="BB27" t="n">
+        <v>-217</v>
+      </c>
+      <c r="BC27" t="n">
+        <v>-152</v>
+      </c>
+      <c r="BF27" t="n">
+        <v>-284</v>
+      </c>
+      <c r="BG27" t="n">
+        <v>119</v>
+      </c>
+      <c r="BH27" t="n">
+        <v>-118</v>
+      </c>
+      <c r="BI27" t="n">
+        <v>-217</v>
+      </c>
+      <c r="BJ27" t="n">
+        <v>-152</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3848,6 +4734,36 @@
       <c r="AV28" t="n">
         <v>74</v>
       </c>
+      <c r="AY28" t="n">
+        <v>71</v>
+      </c>
+      <c r="AZ28" t="n">
+        <v>32</v>
+      </c>
+      <c r="BA28" t="n">
+        <v>32</v>
+      </c>
+      <c r="BB28" t="n">
+        <v>49</v>
+      </c>
+      <c r="BC28" t="n">
+        <v>74</v>
+      </c>
+      <c r="BF28" t="n">
+        <v>71</v>
+      </c>
+      <c r="BG28" t="n">
+        <v>32</v>
+      </c>
+      <c r="BH28" t="n">
+        <v>32</v>
+      </c>
+      <c r="BI28" t="n">
+        <v>49</v>
+      </c>
+      <c r="BJ28" t="n">
+        <v>74</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3960,6 +4876,36 @@
       <c r="AV29" t="n">
         <v>0</v>
       </c>
+      <c r="AY29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4072,6 +5018,36 @@
       <c r="AV30" t="n">
         <v>74</v>
       </c>
+      <c r="AY30" t="n">
+        <v>71</v>
+      </c>
+      <c r="AZ30" t="n">
+        <v>32</v>
+      </c>
+      <c r="BA30" t="n">
+        <v>32</v>
+      </c>
+      <c r="BB30" t="n">
+        <v>49</v>
+      </c>
+      <c r="BC30" t="n">
+        <v>74</v>
+      </c>
+      <c r="BF30" t="n">
+        <v>71</v>
+      </c>
+      <c r="BG30" t="n">
+        <v>32</v>
+      </c>
+      <c r="BH30" t="n">
+        <v>32</v>
+      </c>
+      <c r="BI30" t="n">
+        <v>49</v>
+      </c>
+      <c r="BJ30" t="n">
+        <v>74</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4184,6 +5160,36 @@
       <c r="AV31" t="n">
         <v>1003</v>
       </c>
+      <c r="AY31" t="n">
+        <v>731</v>
+      </c>
+      <c r="AZ31" t="n">
+        <v>2651</v>
+      </c>
+      <c r="BA31" t="n">
+        <v>434</v>
+      </c>
+      <c r="BB31" t="n">
+        <v>1874</v>
+      </c>
+      <c r="BC31" t="n">
+        <v>1003</v>
+      </c>
+      <c r="BF31" t="n">
+        <v>731</v>
+      </c>
+      <c r="BG31" t="n">
+        <v>2651</v>
+      </c>
+      <c r="BH31" t="n">
+        <v>434</v>
+      </c>
+      <c r="BI31" t="n">
+        <v>1874</v>
+      </c>
+      <c r="BJ31" t="n">
+        <v>1003</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4296,6 +5302,36 @@
       <c r="AV32" t="n">
         <v>862</v>
       </c>
+      <c r="AY32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ32" t="n">
+        <v>528</v>
+      </c>
+      <c r="BA32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB32" t="n">
+        <v>6</v>
+      </c>
+      <c r="BC32" t="n">
+        <v>862</v>
+      </c>
+      <c r="BF32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG32" t="n">
+        <v>528</v>
+      </c>
+      <c r="BH32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI32" t="n">
+        <v>6</v>
+      </c>
+      <c r="BJ32" t="n">
+        <v>862</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4408,6 +5444,36 @@
       <c r="AV33" t="n">
         <v>141</v>
       </c>
+      <c r="AY33" t="n">
+        <v>731</v>
+      </c>
+      <c r="AZ33" t="n">
+        <v>2123</v>
+      </c>
+      <c r="BA33" t="n">
+        <v>434</v>
+      </c>
+      <c r="BB33" t="n">
+        <v>1868</v>
+      </c>
+      <c r="BC33" t="n">
+        <v>141</v>
+      </c>
+      <c r="BF33" t="n">
+        <v>731</v>
+      </c>
+      <c r="BG33" t="n">
+        <v>2123</v>
+      </c>
+      <c r="BH33" t="n">
+        <v>434</v>
+      </c>
+      <c r="BI33" t="n">
+        <v>1868</v>
+      </c>
+      <c r="BJ33" t="n">
+        <v>141</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4520,6 +5586,36 @@
       <c r="AV34" s="5" t="n">
         <v>566</v>
       </c>
+      <c r="AY34" t="n">
+        <v>611</v>
+      </c>
+      <c r="AZ34" t="n">
+        <v>519</v>
+      </c>
+      <c r="BA34" t="n">
+        <v>831</v>
+      </c>
+      <c r="BB34" t="n">
+        <v>807</v>
+      </c>
+      <c r="BC34" t="n">
+        <v>566</v>
+      </c>
+      <c r="BF34" t="n">
+        <v>611</v>
+      </c>
+      <c r="BG34" t="n">
+        <v>519</v>
+      </c>
+      <c r="BH34" t="n">
+        <v>831</v>
+      </c>
+      <c r="BI34" t="n">
+        <v>807</v>
+      </c>
+      <c r="BJ34" t="n">
+        <v>566</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4632,6 +5728,36 @@
       <c r="AV35" s="5" t="n">
         <v>538</v>
       </c>
+      <c r="AY35" t="n">
+        <v>604</v>
+      </c>
+      <c r="AZ35" t="n">
+        <v>511</v>
+      </c>
+      <c r="BA35" t="n">
+        <v>825</v>
+      </c>
+      <c r="BB35" t="n">
+        <v>784</v>
+      </c>
+      <c r="BC35" t="n">
+        <v>538</v>
+      </c>
+      <c r="BF35" t="n">
+        <v>604</v>
+      </c>
+      <c r="BG35" t="n">
+        <v>511</v>
+      </c>
+      <c r="BH35" t="n">
+        <v>825</v>
+      </c>
+      <c r="BI35" t="n">
+        <v>784</v>
+      </c>
+      <c r="BJ35" t="n">
+        <v>538</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4744,6 +5870,36 @@
       <c r="AV36" s="6" t="n">
         <v>28</v>
       </c>
+      <c r="AY36" t="n">
+        <v>7</v>
+      </c>
+      <c r="AZ36" t="n">
+        <v>8</v>
+      </c>
+      <c r="BA36" t="n">
+        <v>6</v>
+      </c>
+      <c r="BB36" t="n">
+        <v>23</v>
+      </c>
+      <c r="BC36" t="n">
+        <v>28</v>
+      </c>
+      <c r="BF36" t="n">
+        <v>7</v>
+      </c>
+      <c r="BG36" t="n">
+        <v>8</v>
+      </c>
+      <c r="BH36" t="n">
+        <v>6</v>
+      </c>
+      <c r="BI36" t="n">
+        <v>23</v>
+      </c>
+      <c r="BJ36" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4856,6 +6012,36 @@
       <c r="AV37" t="n">
         <v>1</v>
       </c>
+      <c r="AY37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ37" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA37" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB37" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC37" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF37" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG37" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH37" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI37" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ37" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4968,6 +6154,36 @@
       <c r="AV38" t="n">
         <v>1</v>
       </c>
+      <c r="AY38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ38" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA38" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB38" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC38" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF38" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG38" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH38" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI38" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ38" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5080,6 +6296,36 @@
       <c r="AV39" t="n">
         <v>0</v>
       </c>
+      <c r="AY39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ39" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA39" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB39" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC39" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF39" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG39" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH39" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI39" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ39" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5192,6 +6438,36 @@
       <c r="AV40" s="5" t="n">
         <v>158</v>
       </c>
+      <c r="AY40" t="n">
+        <v>158</v>
+      </c>
+      <c r="AZ40" t="n">
+        <v>64</v>
+      </c>
+      <c r="BA40" t="n">
+        <v>67</v>
+      </c>
+      <c r="BB40" t="n">
+        <v>155</v>
+      </c>
+      <c r="BC40" t="n">
+        <v>158</v>
+      </c>
+      <c r="BF40" t="n">
+        <v>158</v>
+      </c>
+      <c r="BG40" t="n">
+        <v>64</v>
+      </c>
+      <c r="BH40" t="n">
+        <v>67</v>
+      </c>
+      <c r="BI40" t="n">
+        <v>155</v>
+      </c>
+      <c r="BJ40" t="n">
+        <v>158</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -5304,6 +6580,36 @@
       <c r="AV41" s="5" t="n">
         <v>158</v>
       </c>
+      <c r="AY41" t="n">
+        <v>158</v>
+      </c>
+      <c r="AZ41" t="n">
+        <v>64</v>
+      </c>
+      <c r="BA41" t="n">
+        <v>67</v>
+      </c>
+      <c r="BB41" t="n">
+        <v>155</v>
+      </c>
+      <c r="BC41" t="n">
+        <v>158</v>
+      </c>
+      <c r="BF41" t="n">
+        <v>158</v>
+      </c>
+      <c r="BG41" t="n">
+        <v>64</v>
+      </c>
+      <c r="BH41" t="n">
+        <v>67</v>
+      </c>
+      <c r="BI41" t="n">
+        <v>155</v>
+      </c>
+      <c r="BJ41" t="n">
+        <v>158</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -5416,6 +6722,36 @@
       <c r="AV42" t="n">
         <v>0</v>
       </c>
+      <c r="AY42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ42" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -5528,6 +6864,36 @@
       <c r="AV43" t="n">
         <v>0</v>
       </c>
+      <c r="AY43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -5640,6 +7006,36 @@
       <c r="AV44" t="n">
         <v>0</v>
       </c>
+      <c r="AY44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ44" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA44" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB44" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC44" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF44" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG44" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH44" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI44" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ44" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -5752,6 +7148,36 @@
       <c r="AV45" t="n">
         <v>0</v>
       </c>
+      <c r="AY45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ45" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -5864,6 +7290,36 @@
       <c r="AV46" t="n">
         <v>43</v>
       </c>
+      <c r="AY46" t="n">
+        <v>102</v>
+      </c>
+      <c r="AZ46" t="n">
+        <v>69</v>
+      </c>
+      <c r="BA46" t="n">
+        <v>133</v>
+      </c>
+      <c r="BB46" t="n">
+        <v>119</v>
+      </c>
+      <c r="BC46" t="n">
+        <v>43</v>
+      </c>
+      <c r="BF46" t="n">
+        <v>102</v>
+      </c>
+      <c r="BG46" t="n">
+        <v>69</v>
+      </c>
+      <c r="BH46" t="n">
+        <v>133</v>
+      </c>
+      <c r="BI46" t="n">
+        <v>119</v>
+      </c>
+      <c r="BJ46" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5976,6 +7432,36 @@
       <c r="AV47" t="n">
         <v>43</v>
       </c>
+      <c r="AY47" t="n">
+        <v>102</v>
+      </c>
+      <c r="AZ47" t="n">
+        <v>69</v>
+      </c>
+      <c r="BA47" t="n">
+        <v>133</v>
+      </c>
+      <c r="BB47" t="n">
+        <v>119</v>
+      </c>
+      <c r="BC47" t="n">
+        <v>43</v>
+      </c>
+      <c r="BF47" t="n">
+        <v>102</v>
+      </c>
+      <c r="BG47" t="n">
+        <v>69</v>
+      </c>
+      <c r="BH47" t="n">
+        <v>133</v>
+      </c>
+      <c r="BI47" t="n">
+        <v>119</v>
+      </c>
+      <c r="BJ47" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -6088,6 +7574,36 @@
       <c r="AV48" t="n">
         <v>0</v>
       </c>
+      <c r="AY48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ48" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -6200,6 +7716,36 @@
       <c r="AV49" t="n">
         <v>244</v>
       </c>
+      <c r="AY49" t="n">
+        <v>28</v>
+      </c>
+      <c r="AZ49" t="n">
+        <v>114</v>
+      </c>
+      <c r="BA49" t="n">
+        <v>24</v>
+      </c>
+      <c r="BB49" t="n">
+        <v>265</v>
+      </c>
+      <c r="BC49" t="n">
+        <v>244</v>
+      </c>
+      <c r="BF49" t="n">
+        <v>28</v>
+      </c>
+      <c r="BG49" t="n">
+        <v>114</v>
+      </c>
+      <c r="BH49" t="n">
+        <v>24</v>
+      </c>
+      <c r="BI49" t="n">
+        <v>265</v>
+      </c>
+      <c r="BJ49" t="n">
+        <v>244</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -6312,6 +7858,36 @@
       <c r="AV50" s="6" t="n">
         <v>222</v>
       </c>
+      <c r="AY50" t="n">
+        <v>28</v>
+      </c>
+      <c r="AZ50" t="n">
+        <v>112</v>
+      </c>
+      <c r="BA50" t="n">
+        <v>24</v>
+      </c>
+      <c r="BB50" t="n">
+        <v>247</v>
+      </c>
+      <c r="BC50" t="n">
+        <v>222</v>
+      </c>
+      <c r="BF50" t="n">
+        <v>28</v>
+      </c>
+      <c r="BG50" t="n">
+        <v>112</v>
+      </c>
+      <c r="BH50" t="n">
+        <v>24</v>
+      </c>
+      <c r="BI50" t="n">
+        <v>247</v>
+      </c>
+      <c r="BJ50" t="n">
+        <v>222</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -6424,6 +8000,36 @@
       <c r="AV51" s="6" t="n">
         <v>22</v>
       </c>
+      <c r="AY51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ51" t="n">
+        <v>2</v>
+      </c>
+      <c r="BA51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB51" t="n">
+        <v>18</v>
+      </c>
+      <c r="BC51" t="n">
+        <v>22</v>
+      </c>
+      <c r="BF51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG51" t="n">
+        <v>2</v>
+      </c>
+      <c r="BH51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI51" t="n">
+        <v>18</v>
+      </c>
+      <c r="BJ51" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -6536,6 +8142,36 @@
       <c r="AV52" t="n">
         <v>1</v>
       </c>
+      <c r="AY52" t="n">
+        <v>9</v>
+      </c>
+      <c r="AZ52" t="n">
+        <v>2</v>
+      </c>
+      <c r="BA52" t="n">
+        <v>38</v>
+      </c>
+      <c r="BB52" t="n">
+        <v>105</v>
+      </c>
+      <c r="BC52" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF52" t="n">
+        <v>9</v>
+      </c>
+      <c r="BG52" t="n">
+        <v>2</v>
+      </c>
+      <c r="BH52" t="n">
+        <v>38</v>
+      </c>
+      <c r="BI52" t="n">
+        <v>105</v>
+      </c>
+      <c r="BJ52" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -6648,6 +8284,36 @@
       <c r="AV53" t="n">
         <v>1</v>
       </c>
+      <c r="AY53" t="n">
+        <v>8</v>
+      </c>
+      <c r="AZ53" t="n">
+        <v>2</v>
+      </c>
+      <c r="BA53" t="n">
+        <v>38</v>
+      </c>
+      <c r="BB53" t="n">
+        <v>103</v>
+      </c>
+      <c r="BC53" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF53" t="n">
+        <v>8</v>
+      </c>
+      <c r="BG53" t="n">
+        <v>2</v>
+      </c>
+      <c r="BH53" t="n">
+        <v>38</v>
+      </c>
+      <c r="BI53" t="n">
+        <v>103</v>
+      </c>
+      <c r="BJ53" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -6760,6 +8426,36 @@
       <c r="AV54" t="n">
         <v>0</v>
       </c>
+      <c r="AY54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ54" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA54" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB54" t="n">
+        <v>2</v>
+      </c>
+      <c r="BC54" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF54" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG54" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH54" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI54" t="n">
+        <v>2</v>
+      </c>
+      <c r="BJ54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -6872,6 +8568,36 @@
       <c r="AV55" t="n">
         <v>0</v>
       </c>
+      <c r="AY55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ55" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA55" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB55" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC55" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF55" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG55" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH55" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI55" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ55" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -6984,6 +8710,36 @@
       <c r="AV56" t="n">
         <v>0</v>
       </c>
+      <c r="AY56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ56" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA56" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB56" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC56" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF56" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG56" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH56" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI56" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ56" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -7096,6 +8852,36 @@
       <c r="AV57" t="n">
         <v>0</v>
       </c>
+      <c r="AY57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ57" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -7208,6 +8994,36 @@
       <c r="AV58" t="n">
         <v>4</v>
       </c>
+      <c r="AY58" t="n">
+        <v>68</v>
+      </c>
+      <c r="AZ58" t="n">
+        <v>165</v>
+      </c>
+      <c r="BA58" t="n">
+        <v>459</v>
+      </c>
+      <c r="BB58" t="n">
+        <v>38</v>
+      </c>
+      <c r="BC58" t="n">
+        <v>4</v>
+      </c>
+      <c r="BF58" t="n">
+        <v>68</v>
+      </c>
+      <c r="BG58" t="n">
+        <v>165</v>
+      </c>
+      <c r="BH58" t="n">
+        <v>459</v>
+      </c>
+      <c r="BI58" t="n">
+        <v>38</v>
+      </c>
+      <c r="BJ58" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -7320,6 +9136,36 @@
       <c r="AV59" t="n">
         <v>4</v>
       </c>
+      <c r="AY59" t="n">
+        <v>68</v>
+      </c>
+      <c r="AZ59" t="n">
+        <v>165</v>
+      </c>
+      <c r="BA59" t="n">
+        <v>459</v>
+      </c>
+      <c r="BB59" t="n">
+        <v>38</v>
+      </c>
+      <c r="BC59" t="n">
+        <v>4</v>
+      </c>
+      <c r="BF59" t="n">
+        <v>68</v>
+      </c>
+      <c r="BG59" t="n">
+        <v>165</v>
+      </c>
+      <c r="BH59" t="n">
+        <v>459</v>
+      </c>
+      <c r="BI59" t="n">
+        <v>38</v>
+      </c>
+      <c r="BJ59" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -7432,6 +9278,36 @@
       <c r="AV60" t="n">
         <v>0</v>
       </c>
+      <c r="AY60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ60" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA60" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB60" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC60" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF60" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG60" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH60" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI60" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -7544,6 +9420,36 @@
       <c r="AV61" t="n">
         <v>40</v>
       </c>
+      <c r="AY61" t="n">
+        <v>65</v>
+      </c>
+      <c r="AZ61" t="n">
+        <v>36</v>
+      </c>
+      <c r="BA61" t="n">
+        <v>102</v>
+      </c>
+      <c r="BB61" t="n">
+        <v>83</v>
+      </c>
+      <c r="BC61" t="n">
+        <v>40</v>
+      </c>
+      <c r="BF61" t="n">
+        <v>65</v>
+      </c>
+      <c r="BG61" t="n">
+        <v>36</v>
+      </c>
+      <c r="BH61" t="n">
+        <v>102</v>
+      </c>
+      <c r="BI61" t="n">
+        <v>83</v>
+      </c>
+      <c r="BJ61" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -7656,6 +9562,36 @@
       <c r="AV62" s="6" t="n">
         <v>34</v>
       </c>
+      <c r="AY62" t="n">
+        <v>59</v>
+      </c>
+      <c r="AZ62" t="n">
+        <v>30</v>
+      </c>
+      <c r="BA62" t="n">
+        <v>97</v>
+      </c>
+      <c r="BB62" t="n">
+        <v>80</v>
+      </c>
+      <c r="BC62" t="n">
+        <v>34</v>
+      </c>
+      <c r="BF62" t="n">
+        <v>59</v>
+      </c>
+      <c r="BG62" t="n">
+        <v>30</v>
+      </c>
+      <c r="BH62" t="n">
+        <v>97</v>
+      </c>
+      <c r="BI62" t="n">
+        <v>80</v>
+      </c>
+      <c r="BJ62" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -7768,6 +9704,36 @@
       <c r="AV63" s="6" t="n">
         <v>6</v>
       </c>
+      <c r="AY63" t="n">
+        <v>6</v>
+      </c>
+      <c r="AZ63" t="n">
+        <v>6</v>
+      </c>
+      <c r="BA63" t="n">
+        <v>5</v>
+      </c>
+      <c r="BB63" t="n">
+        <v>3</v>
+      </c>
+      <c r="BC63" t="n">
+        <v>6</v>
+      </c>
+      <c r="BF63" t="n">
+        <v>6</v>
+      </c>
+      <c r="BG63" t="n">
+        <v>6</v>
+      </c>
+      <c r="BH63" t="n">
+        <v>5</v>
+      </c>
+      <c r="BI63" t="n">
+        <v>3</v>
+      </c>
+      <c r="BJ63" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -7880,6 +9846,36 @@
       <c r="AV64" t="n">
         <v>0</v>
       </c>
+      <c r="AY64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ64" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA64" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB64" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC64" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF64" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG64" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH64" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI64" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -7992,6 +9988,36 @@
       <c r="AV65" t="n">
         <v>0</v>
       </c>
+      <c r="AY65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ65" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -8104,6 +10130,36 @@
       <c r="AV66" t="n">
         <v>0</v>
       </c>
+      <c r="AY66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ66" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -8216,6 +10272,36 @@
       <c r="AV67" t="n">
         <v>0</v>
       </c>
+      <c r="AY67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ67" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA67" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB67" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC67" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF67" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG67" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH67" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI67" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ67" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -8328,6 +10414,36 @@
       <c r="AV68" t="n">
         <v>0</v>
       </c>
+      <c r="AY68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ68" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -8440,6 +10556,36 @@
       <c r="AV69" t="n">
         <v>0</v>
       </c>
+      <c r="AY69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ69" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -8552,6 +10698,36 @@
       <c r="AV70" t="n">
         <v>0</v>
       </c>
+      <c r="AY70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ70" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -8664,6 +10840,36 @@
       <c r="AV71" t="n">
         <v>0</v>
       </c>
+      <c r="AY71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -8776,6 +10982,36 @@
       <c r="AV72" t="n">
         <v>0</v>
       </c>
+      <c r="AY72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ72" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -8888,6 +11124,36 @@
       <c r="AV73" t="n">
         <v>0</v>
       </c>
+      <c r="AY73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ73" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA73" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB73" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC73" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF73" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG73" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH73" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI73" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -9000,6 +11266,36 @@
       <c r="AV74" t="n">
         <v>0</v>
       </c>
+      <c r="AY74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ74" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA74" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB74" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC74" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF74" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG74" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH74" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI74" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -9112,6 +11408,36 @@
       <c r="AV75" t="n">
         <v>0</v>
       </c>
+      <c r="AY75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ75" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -9224,6 +11550,36 @@
       <c r="AV76" t="n">
         <v>0</v>
       </c>
+      <c r="AY76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ76" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -9336,6 +11692,36 @@
       <c r="AV77" t="n">
         <v>0</v>
       </c>
+      <c r="AY77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -9448,6 +11834,36 @@
       <c r="AV78" t="n">
         <v>0</v>
       </c>
+      <c r="AY78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ78" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -9560,6 +11976,36 @@
       <c r="AV79" t="n">
         <v>0</v>
       </c>
+      <c r="AY79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ79" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -9672,6 +12118,36 @@
       <c r="AV80" t="n">
         <v>0</v>
       </c>
+      <c r="AY80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ80" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -9784,6 +12260,36 @@
       <c r="AV81" t="n">
         <v>0</v>
       </c>
+      <c r="AY81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ81" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -9896,6 +12402,36 @@
       <c r="AV82" t="n">
         <v>0</v>
       </c>
+      <c r="AY82" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ82" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -10008,6 +12544,36 @@
       <c r="AV83" t="n">
         <v>0</v>
       </c>
+      <c r="AY83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ83" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -10120,6 +12686,36 @@
       <c r="AV84" t="n">
         <v>0</v>
       </c>
+      <c r="AY84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ84" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -10232,6 +12828,36 @@
       <c r="AV85" t="n">
         <v>0</v>
       </c>
+      <c r="AY85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -10344,6 +12970,36 @@
       <c r="AV86" t="n">
         <v>0</v>
       </c>
+      <c r="AY86" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ86" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA86" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB86" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC86" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF86" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG86" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH86" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI86" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -10456,16 +13112,48 @@
       <c r="AV87" t="n">
         <v>0</v>
       </c>
+      <c r="AY87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ87" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
     <mergeCell ref="AD1:AI1"/>
     <mergeCell ref="AR1:AW1"/>
     <mergeCell ref="P1:U1"/>
     <mergeCell ref="AK1:AP1"/>
     <mergeCell ref="W1:AB1"/>
     <mergeCell ref="B1:G1"/>
+    <mergeCell ref="AY1:BD1"/>
     <mergeCell ref="I1:N1"/>
+    <mergeCell ref="BF1:BK1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fixing bib and end itemize errors
</commit_message>
<xml_diff>
--- a/tests/regression_test/results/master_results.xlsx
+++ b/tests/regression_test/results/master_results.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BK96"/>
+  <dimension ref="A1:BY96"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="32.5" customWidth="1" style="4" min="1" max="1"/>
@@ -496,6 +496,16 @@
           <t>nesting-depth</t>
         </is>
       </c>
+      <c r="BM1" s="3" t="inlineStr">
+        <is>
+          <t>treating-unclosed</t>
+        </is>
+      </c>
+      <c r="BT1" s="3" t="inlineStr">
+        <is>
+          <t>fixing-bib</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -773,6 +783,66 @@
           <t>avg.</t>
         </is>
       </c>
+      <c r="BM2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="BN2" t="inlineStr">
+        <is>
+          <t>algorithms</t>
+        </is>
+      </c>
+      <c r="BO2" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="BP2" t="inlineStr">
+        <is>
+          <t>cybersec</t>
+        </is>
+      </c>
+      <c r="BQ2" t="inlineStr">
+        <is>
+          <t>data-science</t>
+        </is>
+      </c>
+      <c r="BR2" t="inlineStr">
+        <is>
+          <t>avg.</t>
+        </is>
+      </c>
+      <c r="BT2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="BU2" t="inlineStr">
+        <is>
+          <t>algorithms</t>
+        </is>
+      </c>
+      <c r="BV2" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="BW2" t="inlineStr">
+        <is>
+          <t>cybersec</t>
+        </is>
+      </c>
+      <c r="BX2" t="inlineStr">
+        <is>
+          <t>data-science</t>
+        </is>
+      </c>
+      <c r="BY2" t="inlineStr">
+        <is>
+          <t>avg.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -960,6 +1030,11 @@
           <t>ai</t>
         </is>
       </c>
+      <c r="AZ3" t="inlineStr">
+        <is>
+          <t>algorithms</t>
+        </is>
+      </c>
       <c r="BA3" t="inlineStr">
         <is>
           <t>assembly</t>
@@ -996,6 +1071,56 @@
         </is>
       </c>
       <c r="BJ3" t="inlineStr">
+        <is>
+          <t>data-science</t>
+        </is>
+      </c>
+      <c r="BM3" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="BN3" t="inlineStr">
+        <is>
+          <t>algorithms</t>
+        </is>
+      </c>
+      <c r="BO3" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="BP3" t="inlineStr">
+        <is>
+          <t>cybersec</t>
+        </is>
+      </c>
+      <c r="BQ3" t="inlineStr">
+        <is>
+          <t>data-science</t>
+        </is>
+      </c>
+      <c r="BT3" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="BU3" t="inlineStr">
+        <is>
+          <t>algorithms</t>
+        </is>
+      </c>
+      <c r="BV3" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="BW3" t="inlineStr">
+        <is>
+          <t>cybersec</t>
+        </is>
+      </c>
+      <c r="BX3" t="inlineStr">
         <is>
           <t>data-science</t>
         </is>
@@ -1187,6 +1312,11 @@
           <t>multi-metric</t>
         </is>
       </c>
+      <c r="AZ4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
       <c r="BA4" t="inlineStr">
         <is>
           <t>multi-metric</t>
@@ -1223,6 +1353,56 @@
         </is>
       </c>
       <c r="BJ4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="BM4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="BN4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="BO4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="BP4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="BQ4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="BT4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="BU4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="BV4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="BW4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="BX4" t="inlineStr">
         <is>
           <t>multi-metric</t>
         </is>
@@ -1411,22 +1591,27 @@
       </c>
       <c r="AY5" t="inlineStr">
         <is>
-          <t>2025-10-26T15:41:20.069223</t>
+          <t>2025-10-27T14:53:03.679475</t>
+        </is>
+      </c>
+      <c r="AZ5" t="inlineStr">
+        <is>
+          <t>2025-10-27T14:53:04.014736</t>
         </is>
       </c>
       <c r="BA5" t="inlineStr">
         <is>
-          <t>2025-10-26T15:41:20.244102</t>
+          <t>2025-10-27T14:53:03.892683</t>
         </is>
       </c>
       <c r="BB5" t="inlineStr">
         <is>
-          <t>2025-10-26T15:41:20.314569</t>
+          <t>2025-10-27T14:53:04.159801</t>
         </is>
       </c>
       <c r="BC5" t="inlineStr">
         <is>
-          <t>2025-10-26T15:41:20.398681</t>
+          <t>2025-10-27T14:53:04.258226</t>
         </is>
       </c>
       <c r="BF5" t="inlineStr">
@@ -1452,6 +1637,56 @@
       <c r="BJ5" t="inlineStr">
         <is>
           <t>2025-10-26T15:39:14.633442</t>
+        </is>
+      </c>
+      <c r="BM5" t="inlineStr">
+        <is>
+          <t>2025-10-28T11:44:05.539713</t>
+        </is>
+      </c>
+      <c r="BN5" t="inlineStr">
+        <is>
+          <t>2025-10-28T11:44:05.805317</t>
+        </is>
+      </c>
+      <c r="BO5" t="inlineStr">
+        <is>
+          <t>2025-10-28T11:44:05.683761</t>
+        </is>
+      </c>
+      <c r="BP5" t="inlineStr">
+        <is>
+          <t>2025-10-28T11:44:05.931348</t>
+        </is>
+      </c>
+      <c r="BQ5" t="inlineStr">
+        <is>
+          <t>2025-10-28T11:44:06.074306</t>
+        </is>
+      </c>
+      <c r="BT5" t="inlineStr">
+        <is>
+          <t>2025-10-28T12:25:13.208369</t>
+        </is>
+      </c>
+      <c r="BU5" t="inlineStr">
+        <is>
+          <t>2025-10-28T12:25:13.477210</t>
+        </is>
+      </c>
+      <c r="BV5" t="inlineStr">
+        <is>
+          <t>2025-10-28T12:25:13.373152</t>
+        </is>
+      </c>
+      <c r="BW5" t="inlineStr">
+        <is>
+          <t>2025-10-28T12:25:13.768400</t>
+        </is>
+      </c>
+      <c r="BX5" t="inlineStr">
+        <is>
+          <t>2025-10-28T12:25:13.846417</t>
         </is>
       </c>
     </row>
@@ -1590,6 +1825,9 @@
       <c r="AY6" s="6" t="n">
         <v>-565.4</v>
       </c>
+      <c r="AZ6" s="6" t="n">
+        <v>-1061.8</v>
+      </c>
       <c r="BA6" s="6" t="n">
         <v>-290.8</v>
       </c>
@@ -1600,12 +1838,12 @@
         <v>-376.2</v>
       </c>
       <c r="BD6" s="6" t="n">
-        <v>-537.925</v>
+        <v>-642.7</v>
       </c>
       <c r="BF6" s="5" t="n">
         <v>-506.2</v>
       </c>
-      <c r="BG6" t="n">
+      <c r="BG6" s="5" t="n">
         <v>-1054.1</v>
       </c>
       <c r="BH6" s="5" t="n">
@@ -1617,8 +1855,44 @@
       <c r="BJ6" s="5" t="n">
         <v>-301.1</v>
       </c>
-      <c r="BK6" s="6" t="n">
+      <c r="BK6" s="5" t="n">
         <v>-599.52</v>
+      </c>
+      <c r="BM6" s="5" t="n">
+        <v>-503.7</v>
+      </c>
+      <c r="BN6" s="5" t="n">
+        <v>-1049.5</v>
+      </c>
+      <c r="BO6" s="5" t="n">
+        <v>-278.9</v>
+      </c>
+      <c r="BP6" s="5" t="n">
+        <v>-669.8</v>
+      </c>
+      <c r="BQ6" s="5" t="n">
+        <v>-208.9</v>
+      </c>
+      <c r="BR6" s="5" t="n">
+        <v>-542.16</v>
+      </c>
+      <c r="BT6" s="5" t="n">
+        <v>-404.6</v>
+      </c>
+      <c r="BU6" s="5" t="n">
+        <v>-666.6</v>
+      </c>
+      <c r="BV6" t="n">
+        <v>-278.9</v>
+      </c>
+      <c r="BW6" t="n">
+        <v>-669.8</v>
+      </c>
+      <c r="BX6" t="n">
+        <v>-208.9</v>
+      </c>
+      <c r="BY6" s="5" t="n">
+        <v>-445.76</v>
       </c>
     </row>
     <row r="7">
@@ -1735,6 +2009,9 @@
       <c r="AY7" s="6" t="n">
         <v>68.06999999999999</v>
       </c>
+      <c r="AZ7" s="6" t="n">
+        <v>62.5</v>
+      </c>
       <c r="BA7" t="n">
         <v>100</v>
       </c>
@@ -1747,7 +2024,7 @@
       <c r="BF7" s="5" t="n">
         <v>87.11</v>
       </c>
-      <c r="BG7" t="n">
+      <c r="BG7" s="5" t="n">
         <v>65.88</v>
       </c>
       <c r="BH7" t="n">
@@ -1757,6 +2034,36 @@
         <v>100</v>
       </c>
       <c r="BJ7" t="n">
+        <v>100</v>
+      </c>
+      <c r="BM7" s="6" t="n">
+        <v>85.15000000000001</v>
+      </c>
+      <c r="BN7" s="6" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="BO7" t="n">
+        <v>100</v>
+      </c>
+      <c r="BP7" t="n">
+        <v>100</v>
+      </c>
+      <c r="BQ7" t="n">
+        <v>100</v>
+      </c>
+      <c r="BT7" s="5" t="n">
+        <v>85.43000000000001</v>
+      </c>
+      <c r="BU7" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="BV7" t="n">
+        <v>100</v>
+      </c>
+      <c r="BW7" t="n">
+        <v>100</v>
+      </c>
+      <c r="BX7" t="n">
         <v>100</v>
       </c>
     </row>
@@ -1874,6 +2181,9 @@
       <c r="AY8" s="6" t="n">
         <v>176.29</v>
       </c>
+      <c r="AZ8" s="6" t="n">
+        <v>16</v>
+      </c>
       <c r="BA8" s="6" t="n">
         <v>16</v>
       </c>
@@ -1886,7 +2196,7 @@
       <c r="BF8" s="5" t="n">
         <v>13.78</v>
       </c>
-      <c r="BG8" t="n">
+      <c r="BG8" s="5" t="n">
         <v>7.59</v>
       </c>
       <c r="BH8" t="n">
@@ -1897,6 +2207,36 @@
       </c>
       <c r="BJ8" s="5" t="n">
         <v>163</v>
+      </c>
+      <c r="BM8" s="6" t="n">
+        <v>16.44</v>
+      </c>
+      <c r="BN8" s="5" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="BO8" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="BP8" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="BQ8" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="BT8" s="5" t="n">
+        <v>16.39</v>
+      </c>
+      <c r="BU8" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="BV8" t="n">
+        <v>7</v>
+      </c>
+      <c r="BW8" t="n">
+        <v>19</v>
+      </c>
+      <c r="BX8" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -2013,6 +2353,9 @@
       <c r="AY9" s="5" t="n">
         <v>260.03</v>
       </c>
+      <c r="AZ9" s="6" t="n">
+        <v>99.2</v>
+      </c>
       <c r="BA9" s="6" t="n">
         <v>55</v>
       </c>
@@ -2025,7 +2368,7 @@
       <c r="BF9" s="5" t="n">
         <v>143.5</v>
       </c>
-      <c r="BG9" t="n">
+      <c r="BG9" s="5" t="n">
         <v>15.18</v>
       </c>
       <c r="BH9" s="5" t="n">
@@ -2036,6 +2379,36 @@
       </c>
       <c r="BJ9" s="5" t="n">
         <v>114</v>
+      </c>
+      <c r="BM9" s="6" t="n">
+        <v>146.8</v>
+      </c>
+      <c r="BN9" s="5" t="n">
+        <v>13.95</v>
+      </c>
+      <c r="BO9" t="n">
+        <v>6</v>
+      </c>
+      <c r="BP9" t="n">
+        <v>92</v>
+      </c>
+      <c r="BQ9" s="5" t="n">
+        <v>112</v>
+      </c>
+      <c r="BT9" s="6" t="n">
+        <v>344.14</v>
+      </c>
+      <c r="BU9" s="6" t="n">
+        <v>62.02</v>
+      </c>
+      <c r="BV9" t="n">
+        <v>6</v>
+      </c>
+      <c r="BW9" t="n">
+        <v>92</v>
+      </c>
+      <c r="BX9" t="n">
+        <v>112</v>
       </c>
     </row>
     <row r="10">
@@ -2152,6 +2525,9 @@
       <c r="AY10" t="n">
         <v>100</v>
       </c>
+      <c r="AZ10" t="n">
+        <v>6.29</v>
+      </c>
       <c r="BA10" t="n">
         <v>100</v>
       </c>
@@ -2174,6 +2550,36 @@
         <v>100</v>
       </c>
       <c r="BJ10" t="n">
+        <v>100</v>
+      </c>
+      <c r="BM10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN10" t="n">
+        <v>6.29</v>
+      </c>
+      <c r="BO10" t="n">
+        <v>100</v>
+      </c>
+      <c r="BP10" t="n">
+        <v>100</v>
+      </c>
+      <c r="BQ10" t="n">
+        <v>100</v>
+      </c>
+      <c r="BT10" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="BU10" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="BV10" t="n">
+        <v>100</v>
+      </c>
+      <c r="BW10" t="n">
+        <v>100</v>
+      </c>
+      <c r="BX10" t="n">
         <v>100</v>
       </c>
     </row>
@@ -2291,6 +2697,9 @@
       <c r="AY11" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="AZ11" t="n">
+        <v>89.47</v>
+      </c>
       <c r="BA11" t="n">
         <v>100</v>
       </c>
@@ -2313,6 +2722,36 @@
         <v>100</v>
       </c>
       <c r="BJ11" t="n">
+        <v>86.79000000000001</v>
+      </c>
+      <c r="BM11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN11" t="n">
+        <v>89.47</v>
+      </c>
+      <c r="BO11" t="n">
+        <v>100</v>
+      </c>
+      <c r="BP11" t="n">
+        <v>100</v>
+      </c>
+      <c r="BQ11" t="n">
+        <v>86.79000000000001</v>
+      </c>
+      <c r="BT11" s="5" t="n">
+        <v>99.56999999999999</v>
+      </c>
+      <c r="BU11" s="5" t="n">
+        <v>90.84</v>
+      </c>
+      <c r="BV11" t="n">
+        <v>100</v>
+      </c>
+      <c r="BW11" t="n">
+        <v>100</v>
+      </c>
+      <c r="BX11" t="n">
         <v>86.79000000000001</v>
       </c>
     </row>
@@ -2430,6 +2869,9 @@
       <c r="AY12" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="AZ12" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="BA12" s="6" t="n">
         <v>0</v>
       </c>
@@ -2452,6 +2894,36 @@
         <v>0</v>
       </c>
       <c r="BJ12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2569,6 +3041,9 @@
       <c r="AY13" s="6" t="n">
         <v>132.99</v>
       </c>
+      <c r="AZ13" s="6" t="n">
+        <v>111.5</v>
+      </c>
       <c r="BA13" s="6" t="n">
         <v>76.19</v>
       </c>
@@ -2591,6 +3066,36 @@
         <v>182.5</v>
       </c>
       <c r="BJ13" t="n">
+        <v>129.52</v>
+      </c>
+      <c r="BM13" t="n">
+        <v>132.99</v>
+      </c>
+      <c r="BN13" t="n">
+        <v>111.5</v>
+      </c>
+      <c r="BO13" t="n">
+        <v>76.19</v>
+      </c>
+      <c r="BP13" t="n">
+        <v>182.5</v>
+      </c>
+      <c r="BQ13" t="n">
+        <v>129.52</v>
+      </c>
+      <c r="BT13" t="n">
+        <v>132.99</v>
+      </c>
+      <c r="BU13" t="n">
+        <v>111.5</v>
+      </c>
+      <c r="BV13" t="n">
+        <v>76.19</v>
+      </c>
+      <c r="BW13" t="n">
+        <v>182.5</v>
+      </c>
+      <c r="BX13" t="n">
         <v>129.52</v>
       </c>
     </row>
@@ -2708,6 +3213,9 @@
       <c r="AY14" s="5" t="n">
         <v>175.93</v>
       </c>
+      <c r="AZ14" s="5" t="n">
+        <v>249.21</v>
+      </c>
       <c r="BA14" s="5" t="n">
         <v>1016.67</v>
       </c>
@@ -2730,6 +3238,36 @@
         <v>206.51</v>
       </c>
       <c r="BJ14" t="n">
+        <v>150.84</v>
+      </c>
+      <c r="BM14" t="n">
+        <v>175.93</v>
+      </c>
+      <c r="BN14" t="n">
+        <v>249.21</v>
+      </c>
+      <c r="BO14" t="n">
+        <v>1016.67</v>
+      </c>
+      <c r="BP14" t="n">
+        <v>206.51</v>
+      </c>
+      <c r="BQ14" t="n">
+        <v>150.84</v>
+      </c>
+      <c r="BT14" t="n">
+        <v>175.93</v>
+      </c>
+      <c r="BU14" t="n">
+        <v>249.21</v>
+      </c>
+      <c r="BV14" t="n">
+        <v>1016.67</v>
+      </c>
+      <c r="BW14" t="n">
+        <v>206.51</v>
+      </c>
+      <c r="BX14" t="n">
         <v>150.84</v>
       </c>
     </row>
@@ -2847,6 +3385,9 @@
       <c r="AY15" t="n">
         <v>607.14</v>
       </c>
+      <c r="AZ15" t="n">
+        <v>52.59</v>
+      </c>
       <c r="BA15" t="n">
         <v>837.5</v>
       </c>
@@ -2869,6 +3410,36 @@
         <v>333.33</v>
       </c>
       <c r="BJ15" t="n">
+        <v>185.39</v>
+      </c>
+      <c r="BM15" t="n">
+        <v>607.14</v>
+      </c>
+      <c r="BN15" t="n">
+        <v>52.59</v>
+      </c>
+      <c r="BO15" t="n">
+        <v>837.5</v>
+      </c>
+      <c r="BP15" s="5" t="n">
+        <v>334.41</v>
+      </c>
+      <c r="BQ15" t="n">
+        <v>185.39</v>
+      </c>
+      <c r="BT15" t="n">
+        <v>607.14</v>
+      </c>
+      <c r="BU15" t="n">
+        <v>52.59</v>
+      </c>
+      <c r="BV15" t="n">
+        <v>837.5</v>
+      </c>
+      <c r="BW15" t="n">
+        <v>334.41</v>
+      </c>
+      <c r="BX15" t="n">
         <v>185.39</v>
       </c>
     </row>
@@ -2986,6 +3557,9 @@
       <c r="AY16" t="n">
         <v>143.66</v>
       </c>
+      <c r="AZ16" t="n">
+        <v>215.62</v>
+      </c>
       <c r="BA16" t="n">
         <v>415.62</v>
       </c>
@@ -3008,6 +3582,36 @@
         <v>242.86</v>
       </c>
       <c r="BJ16" t="n">
+        <v>58.11</v>
+      </c>
+      <c r="BM16" t="n">
+        <v>143.66</v>
+      </c>
+      <c r="BN16" t="n">
+        <v>215.62</v>
+      </c>
+      <c r="BO16" t="n">
+        <v>415.62</v>
+      </c>
+      <c r="BP16" t="n">
+        <v>242.86</v>
+      </c>
+      <c r="BQ16" t="n">
+        <v>58.11</v>
+      </c>
+      <c r="BT16" t="n">
+        <v>143.66</v>
+      </c>
+      <c r="BU16" t="n">
+        <v>215.62</v>
+      </c>
+      <c r="BV16" t="n">
+        <v>415.62</v>
+      </c>
+      <c r="BW16" t="n">
+        <v>242.86</v>
+      </c>
+      <c r="BX16" t="n">
         <v>58.11</v>
       </c>
     </row>
@@ -3125,6 +3729,9 @@
       <c r="AY17" t="n">
         <v>0</v>
       </c>
+      <c r="AZ17" t="n">
+        <v>19.92</v>
+      </c>
       <c r="BA17" t="n">
         <v>0</v>
       </c>
@@ -3147,6 +3754,36 @@
         <v>0.32</v>
       </c>
       <c r="BJ17" t="n">
+        <v>85.94</v>
+      </c>
+      <c r="BM17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN17" t="n">
+        <v>19.92</v>
+      </c>
+      <c r="BO17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP17" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="BQ17" t="n">
+        <v>85.94</v>
+      </c>
+      <c r="BT17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU17" t="n">
+        <v>19.92</v>
+      </c>
+      <c r="BV17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW17" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="BX17" t="n">
         <v>85.94</v>
       </c>
     </row>
@@ -3156,7 +3793,7 @@
           <t>------------</t>
         </is>
       </c>
-      <c r="BC18" t="inlineStr"/>
+      <c r="BX18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3272,6 +3909,9 @@
       <c r="AY19" t="n">
         <v>233</v>
       </c>
+      <c r="AZ19" t="n">
+        <v>906</v>
+      </c>
       <c r="BA19" t="n">
         <v>3</v>
       </c>
@@ -3294,6 +3934,36 @@
         <v>101</v>
       </c>
       <c r="BJ19" t="n">
+        <v>106</v>
+      </c>
+      <c r="BM19" t="n">
+        <v>233</v>
+      </c>
+      <c r="BN19" t="n">
+        <v>906</v>
+      </c>
+      <c r="BO19" t="n">
+        <v>3</v>
+      </c>
+      <c r="BP19" t="n">
+        <v>101</v>
+      </c>
+      <c r="BQ19" t="n">
+        <v>106</v>
+      </c>
+      <c r="BT19" t="n">
+        <v>233</v>
+      </c>
+      <c r="BU19" t="n">
+        <v>906</v>
+      </c>
+      <c r="BV19" t="n">
+        <v>3</v>
+      </c>
+      <c r="BW19" t="n">
+        <v>101</v>
+      </c>
+      <c r="BX19" t="n">
         <v>106</v>
       </c>
     </row>
@@ -3411,6 +4081,9 @@
       <c r="AY20" t="n">
         <v>233</v>
       </c>
+      <c r="AZ20" t="n">
+        <v>57</v>
+      </c>
       <c r="BA20" t="n">
         <v>3</v>
       </c>
@@ -3433,6 +4106,36 @@
         <v>101</v>
       </c>
       <c r="BJ20" t="n">
+        <v>106</v>
+      </c>
+      <c r="BM20" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN20" t="n">
+        <v>57</v>
+      </c>
+      <c r="BO20" t="n">
+        <v>3</v>
+      </c>
+      <c r="BP20" t="n">
+        <v>101</v>
+      </c>
+      <c r="BQ20" t="n">
+        <v>106</v>
+      </c>
+      <c r="BT20" s="5" t="n">
+        <v>233</v>
+      </c>
+      <c r="BU20" s="5" t="n">
+        <v>906</v>
+      </c>
+      <c r="BV20" t="n">
+        <v>3</v>
+      </c>
+      <c r="BW20" t="n">
+        <v>101</v>
+      </c>
+      <c r="BX20" t="n">
         <v>106</v>
       </c>
     </row>
@@ -3550,6 +4253,9 @@
       <c r="AY21" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="AZ21" t="n">
+        <v>51</v>
+      </c>
       <c r="BA21" t="n">
         <v>3</v>
       </c>
@@ -3572,6 +4278,36 @@
         <v>101</v>
       </c>
       <c r="BJ21" t="n">
+        <v>92</v>
+      </c>
+      <c r="BM21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN21" t="n">
+        <v>51</v>
+      </c>
+      <c r="BO21" t="n">
+        <v>3</v>
+      </c>
+      <c r="BP21" t="n">
+        <v>101</v>
+      </c>
+      <c r="BQ21" t="n">
+        <v>92</v>
+      </c>
+      <c r="BT21" s="5" t="n">
+        <v>232</v>
+      </c>
+      <c r="BU21" s="5" t="n">
+        <v>823</v>
+      </c>
+      <c r="BV21" t="n">
+        <v>3</v>
+      </c>
+      <c r="BW21" t="n">
+        <v>101</v>
+      </c>
+      <c r="BX21" t="n">
         <v>92</v>
       </c>
     </row>
@@ -3689,6 +4425,9 @@
       <c r="AY22" t="n">
         <v>0</v>
       </c>
+      <c r="AZ22" t="n">
+        <v>849</v>
+      </c>
       <c r="BA22" t="n">
         <v>0</v>
       </c>
@@ -3711,6 +4450,36 @@
         <v>0</v>
       </c>
       <c r="BJ22" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM22" t="n">
+        <v>233</v>
+      </c>
+      <c r="BN22" t="n">
+        <v>849</v>
+      </c>
+      <c r="BO22" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP22" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ22" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV22" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW22" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3828,6 +4597,9 @@
       <c r="AY23" s="6" t="n">
         <v>233</v>
       </c>
+      <c r="AZ23" t="n">
+        <v>6</v>
+      </c>
       <c r="BA23" t="n">
         <v>0</v>
       </c>
@@ -3850,6 +4622,36 @@
         <v>0</v>
       </c>
       <c r="BJ23" t="n">
+        <v>14</v>
+      </c>
+      <c r="BM23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN23" t="n">
+        <v>6</v>
+      </c>
+      <c r="BO23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ23" t="n">
+        <v>14</v>
+      </c>
+      <c r="BT23" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU23" s="6" t="n">
+        <v>83</v>
+      </c>
+      <c r="BV23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW23" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX23" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3967,6 +4769,9 @@
       <c r="AY24" t="n">
         <v>14</v>
       </c>
+      <c r="AZ24" t="n">
+        <v>22</v>
+      </c>
       <c r="BA24" t="n">
         <v>16</v>
       </c>
@@ -3989,6 +4794,36 @@
         <v>21</v>
       </c>
       <c r="BJ24" t="n">
+        <v>13</v>
+      </c>
+      <c r="BM24" t="n">
+        <v>14</v>
+      </c>
+      <c r="BN24" t="n">
+        <v>22</v>
+      </c>
+      <c r="BO24" t="n">
+        <v>16</v>
+      </c>
+      <c r="BP24" t="n">
+        <v>21</v>
+      </c>
+      <c r="BQ24" t="n">
+        <v>13</v>
+      </c>
+      <c r="BT24" t="n">
+        <v>14</v>
+      </c>
+      <c r="BU24" t="n">
+        <v>22</v>
+      </c>
+      <c r="BV24" t="n">
+        <v>16</v>
+      </c>
+      <c r="BW24" t="n">
+        <v>21</v>
+      </c>
+      <c r="BX24" t="n">
         <v>13</v>
       </c>
     </row>
@@ -4106,6 +4941,9 @@
       <c r="AY25" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="AZ25" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="BA25" s="6" t="n">
         <v>0</v>
       </c>
@@ -4128,6 +4966,36 @@
         <v>0</v>
       </c>
       <c r="BJ25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4245,6 +5113,9 @@
       <c r="AY26" s="6" t="n">
         <v>14</v>
       </c>
+      <c r="AZ26" s="6" t="n">
+        <v>22</v>
+      </c>
       <c r="BA26" s="6" t="n">
         <v>16</v>
       </c>
@@ -4267,6 +5138,36 @@
         <v>21</v>
       </c>
       <c r="BJ26" t="n">
+        <v>13</v>
+      </c>
+      <c r="BM26" t="n">
+        <v>14</v>
+      </c>
+      <c r="BN26" t="n">
+        <v>22</v>
+      </c>
+      <c r="BO26" t="n">
+        <v>16</v>
+      </c>
+      <c r="BP26" t="n">
+        <v>21</v>
+      </c>
+      <c r="BQ26" t="n">
+        <v>13</v>
+      </c>
+      <c r="BT26" t="n">
+        <v>14</v>
+      </c>
+      <c r="BU26" t="n">
+        <v>22</v>
+      </c>
+      <c r="BV26" t="n">
+        <v>16</v>
+      </c>
+      <c r="BW26" t="n">
+        <v>21</v>
+      </c>
+      <c r="BX26" t="n">
         <v>13</v>
       </c>
     </row>
@@ -4384,6 +5285,9 @@
       <c r="AY27" t="n">
         <v>97</v>
       </c>
+      <c r="AZ27" t="n">
+        <v>200</v>
+      </c>
       <c r="BA27" t="n">
         <v>126</v>
       </c>
@@ -4406,6 +5310,36 @@
         <v>80</v>
       </c>
       <c r="BJ27" t="n">
+        <v>105</v>
+      </c>
+      <c r="BM27" t="n">
+        <v>97</v>
+      </c>
+      <c r="BN27" t="n">
+        <v>200</v>
+      </c>
+      <c r="BO27" t="n">
+        <v>126</v>
+      </c>
+      <c r="BP27" t="n">
+        <v>80</v>
+      </c>
+      <c r="BQ27" t="n">
+        <v>105</v>
+      </c>
+      <c r="BT27" t="n">
+        <v>97</v>
+      </c>
+      <c r="BU27" t="n">
+        <v>200</v>
+      </c>
+      <c r="BV27" t="n">
+        <v>126</v>
+      </c>
+      <c r="BW27" t="n">
+        <v>80</v>
+      </c>
+      <c r="BX27" t="n">
         <v>105</v>
       </c>
     </row>
@@ -4523,6 +5457,9 @@
       <c r="AY28" s="6" t="n">
         <v>129</v>
       </c>
+      <c r="AZ28" s="6" t="n">
+        <v>223</v>
+      </c>
       <c r="BA28" s="6" t="n">
         <v>96</v>
       </c>
@@ -4545,6 +5482,36 @@
         <v>146</v>
       </c>
       <c r="BJ28" t="n">
+        <v>136</v>
+      </c>
+      <c r="BM28" t="n">
+        <v>129</v>
+      </c>
+      <c r="BN28" t="n">
+        <v>223</v>
+      </c>
+      <c r="BO28" t="n">
+        <v>96</v>
+      </c>
+      <c r="BP28" t="n">
+        <v>146</v>
+      </c>
+      <c r="BQ28" t="n">
+        <v>136</v>
+      </c>
+      <c r="BT28" t="n">
+        <v>129</v>
+      </c>
+      <c r="BU28" t="n">
+        <v>223</v>
+      </c>
+      <c r="BV28" t="n">
+        <v>96</v>
+      </c>
+      <c r="BW28" t="n">
+        <v>146</v>
+      </c>
+      <c r="BX28" t="n">
         <v>136</v>
       </c>
     </row>
@@ -4662,6 +5629,9 @@
       <c r="AY29" s="5" t="n">
         <v>-32</v>
       </c>
+      <c r="AZ29" s="5" t="n">
+        <v>-23</v>
+      </c>
       <c r="BA29" s="5" t="n">
         <v>30</v>
       </c>
@@ -4684,6 +5654,36 @@
         <v>-66</v>
       </c>
       <c r="BJ29" t="n">
+        <v>-31</v>
+      </c>
+      <c r="BM29" t="n">
+        <v>-32</v>
+      </c>
+      <c r="BN29" t="n">
+        <v>-23</v>
+      </c>
+      <c r="BO29" t="n">
+        <v>30</v>
+      </c>
+      <c r="BP29" t="n">
+        <v>-66</v>
+      </c>
+      <c r="BQ29" t="n">
+        <v>-31</v>
+      </c>
+      <c r="BT29" t="n">
+        <v>-32</v>
+      </c>
+      <c r="BU29" t="n">
+        <v>-23</v>
+      </c>
+      <c r="BV29" t="n">
+        <v>30</v>
+      </c>
+      <c r="BW29" t="n">
+        <v>-66</v>
+      </c>
+      <c r="BX29" t="n">
         <v>-31</v>
       </c>
     </row>
@@ -4801,6 +5801,9 @@
       <c r="AY30" t="n">
         <v>108</v>
       </c>
+      <c r="AZ30" t="n">
+        <v>126</v>
+      </c>
       <c r="BA30" t="n">
         <v>12</v>
       </c>
@@ -4823,6 +5826,36 @@
         <v>169</v>
       </c>
       <c r="BJ30" t="n">
+        <v>179</v>
+      </c>
+      <c r="BM30" t="n">
+        <v>108</v>
+      </c>
+      <c r="BN30" t="n">
+        <v>126</v>
+      </c>
+      <c r="BO30" t="n">
+        <v>12</v>
+      </c>
+      <c r="BP30" t="n">
+        <v>169</v>
+      </c>
+      <c r="BQ30" t="n">
+        <v>179</v>
+      </c>
+      <c r="BT30" t="n">
+        <v>108</v>
+      </c>
+      <c r="BU30" t="n">
+        <v>126</v>
+      </c>
+      <c r="BV30" t="n">
+        <v>12</v>
+      </c>
+      <c r="BW30" t="n">
+        <v>169</v>
+      </c>
+      <c r="BX30" t="n">
         <v>179</v>
       </c>
     </row>
@@ -4940,6 +5973,9 @@
       <c r="AY31" s="5" t="n">
         <v>190</v>
       </c>
+      <c r="AZ31" s="5" t="n">
+        <v>314</v>
+      </c>
       <c r="BA31" s="5" t="n">
         <v>122</v>
       </c>
@@ -4962,6 +5998,36 @@
         <v>349</v>
       </c>
       <c r="BJ31" t="n">
+        <v>270</v>
+      </c>
+      <c r="BM31" t="n">
+        <v>190</v>
+      </c>
+      <c r="BN31" t="n">
+        <v>314</v>
+      </c>
+      <c r="BO31" t="n">
+        <v>122</v>
+      </c>
+      <c r="BP31" t="n">
+        <v>349</v>
+      </c>
+      <c r="BQ31" t="n">
+        <v>270</v>
+      </c>
+      <c r="BT31" t="n">
+        <v>190</v>
+      </c>
+      <c r="BU31" t="n">
+        <v>314</v>
+      </c>
+      <c r="BV31" t="n">
+        <v>122</v>
+      </c>
+      <c r="BW31" t="n">
+        <v>349</v>
+      </c>
+      <c r="BX31" t="n">
         <v>270</v>
       </c>
     </row>
@@ -5079,6 +6145,9 @@
       <c r="AY32" s="6" t="n">
         <v>-82</v>
       </c>
+      <c r="AZ32" s="6" t="n">
+        <v>-188</v>
+      </c>
       <c r="BA32" s="6" t="n">
         <v>-110</v>
       </c>
@@ -5101,6 +6170,36 @@
         <v>-180</v>
       </c>
       <c r="BJ32" t="n">
+        <v>-91</v>
+      </c>
+      <c r="BM32" t="n">
+        <v>-82</v>
+      </c>
+      <c r="BN32" t="n">
+        <v>-188</v>
+      </c>
+      <c r="BO32" t="n">
+        <v>-110</v>
+      </c>
+      <c r="BP32" t="n">
+        <v>-180</v>
+      </c>
+      <c r="BQ32" t="n">
+        <v>-91</v>
+      </c>
+      <c r="BT32" t="n">
+        <v>-82</v>
+      </c>
+      <c r="BU32" t="n">
+        <v>-188</v>
+      </c>
+      <c r="BV32" t="n">
+        <v>-110</v>
+      </c>
+      <c r="BW32" t="n">
+        <v>-180</v>
+      </c>
+      <c r="BX32" t="n">
         <v>-91</v>
       </c>
     </row>
@@ -5218,6 +6317,9 @@
       <c r="AY33" t="n">
         <v>56</v>
       </c>
+      <c r="AZ33" t="n">
+        <v>251</v>
+      </c>
       <c r="BA33" t="n">
         <v>16</v>
       </c>
@@ -5240,6 +6342,36 @@
         <v>93</v>
       </c>
       <c r="BJ33" t="n">
+        <v>178</v>
+      </c>
+      <c r="BM33" t="n">
+        <v>56</v>
+      </c>
+      <c r="BN33" t="n">
+        <v>251</v>
+      </c>
+      <c r="BO33" t="n">
+        <v>16</v>
+      </c>
+      <c r="BP33" t="n">
+        <v>93</v>
+      </c>
+      <c r="BQ33" t="n">
+        <v>178</v>
+      </c>
+      <c r="BT33" t="n">
+        <v>56</v>
+      </c>
+      <c r="BU33" t="n">
+        <v>251</v>
+      </c>
+      <c r="BV33" t="n">
+        <v>16</v>
+      </c>
+      <c r="BW33" t="n">
+        <v>93</v>
+      </c>
+      <c r="BX33" t="n">
         <v>178</v>
       </c>
     </row>
@@ -5357,6 +6489,9 @@
       <c r="AY34" t="n">
         <v>158</v>
       </c>
+      <c r="AZ34" t="n">
+        <v>64</v>
+      </c>
       <c r="BA34" t="n">
         <v>67</v>
       </c>
@@ -5379,6 +6514,36 @@
         <v>155</v>
       </c>
       <c r="BJ34" t="n">
+        <v>158</v>
+      </c>
+      <c r="BM34" t="n">
+        <v>158</v>
+      </c>
+      <c r="BN34" t="n">
+        <v>64</v>
+      </c>
+      <c r="BO34" t="n">
+        <v>67</v>
+      </c>
+      <c r="BP34" t="n">
+        <v>155</v>
+      </c>
+      <c r="BQ34" t="n">
+        <v>158</v>
+      </c>
+      <c r="BT34" t="n">
+        <v>158</v>
+      </c>
+      <c r="BU34" t="n">
+        <v>64</v>
+      </c>
+      <c r="BV34" t="n">
+        <v>67</v>
+      </c>
+      <c r="BW34" t="n">
+        <v>155</v>
+      </c>
+      <c r="BX34" t="n">
         <v>158</v>
       </c>
     </row>
@@ -5496,6 +6661,9 @@
       <c r="AY35" t="n">
         <v>182</v>
       </c>
+      <c r="AZ35" t="n">
+        <v>68</v>
+      </c>
       <c r="BA35" t="n">
         <v>67</v>
       </c>
@@ -5518,6 +6686,36 @@
         <v>155</v>
       </c>
       <c r="BJ35" t="n">
+        <v>172</v>
+      </c>
+      <c r="BM35" t="n">
+        <v>182</v>
+      </c>
+      <c r="BN35" t="n">
+        <v>68</v>
+      </c>
+      <c r="BO35" t="n">
+        <v>67</v>
+      </c>
+      <c r="BP35" s="5" t="n">
+        <v>156</v>
+      </c>
+      <c r="BQ35" t="n">
+        <v>172</v>
+      </c>
+      <c r="BT35" t="n">
+        <v>182</v>
+      </c>
+      <c r="BU35" t="n">
+        <v>68</v>
+      </c>
+      <c r="BV35" t="n">
+        <v>67</v>
+      </c>
+      <c r="BW35" t="n">
+        <v>156</v>
+      </c>
+      <c r="BX35" t="n">
         <v>172</v>
       </c>
     </row>
@@ -5635,6 +6833,9 @@
       <c r="AY36" t="n">
         <v>-284</v>
       </c>
+      <c r="AZ36" t="n">
+        <v>119</v>
+      </c>
       <c r="BA36" t="n">
         <v>-118</v>
       </c>
@@ -5657,6 +6858,36 @@
         <v>-217</v>
       </c>
       <c r="BJ36" t="n">
+        <v>-152</v>
+      </c>
+      <c r="BM36" t="n">
+        <v>-284</v>
+      </c>
+      <c r="BN36" t="n">
+        <v>119</v>
+      </c>
+      <c r="BO36" t="n">
+        <v>-118</v>
+      </c>
+      <c r="BP36" s="6" t="n">
+        <v>-218</v>
+      </c>
+      <c r="BQ36" t="n">
+        <v>-152</v>
+      </c>
+      <c r="BT36" t="n">
+        <v>-284</v>
+      </c>
+      <c r="BU36" t="n">
+        <v>119</v>
+      </c>
+      <c r="BV36" t="n">
+        <v>-118</v>
+      </c>
+      <c r="BW36" t="n">
+        <v>-218</v>
+      </c>
+      <c r="BX36" t="n">
         <v>-152</v>
       </c>
     </row>
@@ -5774,6 +7005,9 @@
       <c r="AY37" t="n">
         <v>71</v>
       </c>
+      <c r="AZ37" t="n">
+        <v>32</v>
+      </c>
       <c r="BA37" t="n">
         <v>32</v>
       </c>
@@ -5796,6 +7030,36 @@
         <v>49</v>
       </c>
       <c r="BJ37" t="n">
+        <v>74</v>
+      </c>
+      <c r="BM37" t="n">
+        <v>71</v>
+      </c>
+      <c r="BN37" t="n">
+        <v>32</v>
+      </c>
+      <c r="BO37" t="n">
+        <v>32</v>
+      </c>
+      <c r="BP37" t="n">
+        <v>49</v>
+      </c>
+      <c r="BQ37" t="n">
+        <v>74</v>
+      </c>
+      <c r="BT37" t="n">
+        <v>71</v>
+      </c>
+      <c r="BU37" t="n">
+        <v>32</v>
+      </c>
+      <c r="BV37" t="n">
+        <v>32</v>
+      </c>
+      <c r="BW37" t="n">
+        <v>49</v>
+      </c>
+      <c r="BX37" t="n">
         <v>74</v>
       </c>
     </row>
@@ -5913,6 +7177,9 @@
       <c r="AY38" t="n">
         <v>102</v>
       </c>
+      <c r="AZ38" t="n">
+        <v>69</v>
+      </c>
       <c r="BA38" t="n">
         <v>133</v>
       </c>
@@ -5935,6 +7202,36 @@
         <v>119</v>
       </c>
       <c r="BJ38" t="n">
+        <v>43</v>
+      </c>
+      <c r="BM38" t="n">
+        <v>102</v>
+      </c>
+      <c r="BN38" t="n">
+        <v>69</v>
+      </c>
+      <c r="BO38" t="n">
+        <v>133</v>
+      </c>
+      <c r="BP38" t="n">
+        <v>119</v>
+      </c>
+      <c r="BQ38" t="n">
+        <v>43</v>
+      </c>
+      <c r="BT38" t="n">
+        <v>102</v>
+      </c>
+      <c r="BU38" t="n">
+        <v>69</v>
+      </c>
+      <c r="BV38" t="n">
+        <v>133</v>
+      </c>
+      <c r="BW38" t="n">
+        <v>119</v>
+      </c>
+      <c r="BX38" t="n">
         <v>43</v>
       </c>
     </row>
@@ -6052,6 +7349,9 @@
       <c r="AY39" t="n">
         <v>-31</v>
       </c>
+      <c r="AZ39" t="n">
+        <v>-37</v>
+      </c>
       <c r="BA39" t="n">
         <v>-101</v>
       </c>
@@ -6074,6 +7374,36 @@
         <v>-70</v>
       </c>
       <c r="BJ39" t="n">
+        <v>31</v>
+      </c>
+      <c r="BM39" t="n">
+        <v>-31</v>
+      </c>
+      <c r="BN39" t="n">
+        <v>-37</v>
+      </c>
+      <c r="BO39" t="n">
+        <v>-101</v>
+      </c>
+      <c r="BP39" t="n">
+        <v>-70</v>
+      </c>
+      <c r="BQ39" t="n">
+        <v>31</v>
+      </c>
+      <c r="BT39" t="n">
+        <v>-31</v>
+      </c>
+      <c r="BU39" t="n">
+        <v>-37</v>
+      </c>
+      <c r="BV39" t="n">
+        <v>-101</v>
+      </c>
+      <c r="BW39" t="n">
+        <v>-70</v>
+      </c>
+      <c r="BX39" t="n">
         <v>31</v>
       </c>
     </row>
@@ -6191,6 +7521,9 @@
       <c r="AY40" t="n">
         <v>731</v>
       </c>
+      <c r="AZ40" t="n">
+        <v>2651</v>
+      </c>
       <c r="BA40" t="n">
         <v>434</v>
       </c>
@@ -6213,6 +7546,36 @@
         <v>1874</v>
       </c>
       <c r="BJ40" t="n">
+        <v>1003</v>
+      </c>
+      <c r="BM40" t="n">
+        <v>731</v>
+      </c>
+      <c r="BN40" t="n">
+        <v>2651</v>
+      </c>
+      <c r="BO40" t="n">
+        <v>434</v>
+      </c>
+      <c r="BP40" t="n">
+        <v>1874</v>
+      </c>
+      <c r="BQ40" t="n">
+        <v>1003</v>
+      </c>
+      <c r="BT40" t="n">
+        <v>731</v>
+      </c>
+      <c r="BU40" t="n">
+        <v>2651</v>
+      </c>
+      <c r="BV40" t="n">
+        <v>434</v>
+      </c>
+      <c r="BW40" t="n">
+        <v>1874</v>
+      </c>
+      <c r="BX40" t="n">
         <v>1003</v>
       </c>
     </row>
@@ -6330,6 +7693,9 @@
       <c r="AY41" t="n">
         <v>0</v>
       </c>
+      <c r="AZ41" t="n">
+        <v>528</v>
+      </c>
       <c r="BA41" t="n">
         <v>0</v>
       </c>
@@ -6352,6 +7718,36 @@
         <v>6</v>
       </c>
       <c r="BJ41" t="n">
+        <v>862</v>
+      </c>
+      <c r="BM41" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN41" t="n">
+        <v>528</v>
+      </c>
+      <c r="BO41" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP41" t="n">
+        <v>6</v>
+      </c>
+      <c r="BQ41" t="n">
+        <v>862</v>
+      </c>
+      <c r="BT41" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU41" t="n">
+        <v>528</v>
+      </c>
+      <c r="BV41" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW41" t="n">
+        <v>6</v>
+      </c>
+      <c r="BX41" t="n">
         <v>862</v>
       </c>
     </row>
@@ -6469,6 +7865,9 @@
       <c r="AY42" t="n">
         <v>731</v>
       </c>
+      <c r="AZ42" t="n">
+        <v>2123</v>
+      </c>
       <c r="BA42" t="n">
         <v>434</v>
       </c>
@@ -6491,6 +7890,36 @@
         <v>1868</v>
       </c>
       <c r="BJ42" t="n">
+        <v>141</v>
+      </c>
+      <c r="BM42" t="n">
+        <v>731</v>
+      </c>
+      <c r="BN42" t="n">
+        <v>2123</v>
+      </c>
+      <c r="BO42" t="n">
+        <v>434</v>
+      </c>
+      <c r="BP42" t="n">
+        <v>1868</v>
+      </c>
+      <c r="BQ42" t="n">
+        <v>141</v>
+      </c>
+      <c r="BT42" t="n">
+        <v>731</v>
+      </c>
+      <c r="BU42" t="n">
+        <v>2123</v>
+      </c>
+      <c r="BV42" t="n">
+        <v>434</v>
+      </c>
+      <c r="BW42" t="n">
+        <v>1868</v>
+      </c>
+      <c r="BX42" t="n">
         <v>141</v>
       </c>
     </row>
@@ -6608,6 +8037,9 @@
       <c r="AY43" t="n">
         <v>611</v>
       </c>
+      <c r="AZ43" t="n">
+        <v>519</v>
+      </c>
       <c r="BA43" t="n">
         <v>831</v>
       </c>
@@ -6630,6 +8062,36 @@
         <v>807</v>
       </c>
       <c r="BJ43" t="n">
+        <v>566</v>
+      </c>
+      <c r="BM43" t="n">
+        <v>611</v>
+      </c>
+      <c r="BN43" t="n">
+        <v>519</v>
+      </c>
+      <c r="BO43" t="n">
+        <v>831</v>
+      </c>
+      <c r="BP43" t="n">
+        <v>807</v>
+      </c>
+      <c r="BQ43" t="n">
+        <v>566</v>
+      </c>
+      <c r="BT43" t="n">
+        <v>611</v>
+      </c>
+      <c r="BU43" t="n">
+        <v>519</v>
+      </c>
+      <c r="BV43" t="n">
+        <v>831</v>
+      </c>
+      <c r="BW43" t="n">
+        <v>807</v>
+      </c>
+      <c r="BX43" t="n">
         <v>566</v>
       </c>
     </row>
@@ -6747,6 +8209,9 @@
       <c r="AY44" t="n">
         <v>604</v>
       </c>
+      <c r="AZ44" t="n">
+        <v>511</v>
+      </c>
       <c r="BA44" t="n">
         <v>825</v>
       </c>
@@ -6770,6 +8235,36 @@
       </c>
       <c r="BJ44" t="n">
         <v>538</v>
+      </c>
+      <c r="BM44" s="5" t="n">
+        <v>611</v>
+      </c>
+      <c r="BN44" s="5" t="n">
+        <v>519</v>
+      </c>
+      <c r="BO44" s="5" t="n">
+        <v>830</v>
+      </c>
+      <c r="BP44" s="5" t="n">
+        <v>807</v>
+      </c>
+      <c r="BQ44" s="5" t="n">
+        <v>566</v>
+      </c>
+      <c r="BT44" t="n">
+        <v>611</v>
+      </c>
+      <c r="BU44" t="n">
+        <v>519</v>
+      </c>
+      <c r="BV44" t="n">
+        <v>830</v>
+      </c>
+      <c r="BW44" t="n">
+        <v>807</v>
+      </c>
+      <c r="BX44" t="n">
+        <v>566</v>
       </c>
     </row>
     <row r="45">
@@ -6886,6 +8381,9 @@
       <c r="AY45" t="n">
         <v>7</v>
       </c>
+      <c r="AZ45" t="n">
+        <v>8</v>
+      </c>
       <c r="BA45" t="n">
         <v>6</v>
       </c>
@@ -6909,6 +8407,36 @@
       </c>
       <c r="BJ45" t="n">
         <v>28</v>
+      </c>
+      <c r="BM45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO45" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV45" t="n">
+        <v>1</v>
+      </c>
+      <c r="BW45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX45" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -7025,6 +8553,9 @@
       <c r="AY46" t="n">
         <v>1</v>
       </c>
+      <c r="AZ46" t="n">
+        <v>1</v>
+      </c>
       <c r="BA46" t="n">
         <v>1</v>
       </c>
@@ -7047,6 +8578,36 @@
         <v>1</v>
       </c>
       <c r="BJ46" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM46" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN46" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO46" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP46" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ46" t="n">
+        <v>1</v>
+      </c>
+      <c r="BT46" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU46" t="n">
+        <v>1</v>
+      </c>
+      <c r="BV46" t="n">
+        <v>1</v>
+      </c>
+      <c r="BW46" t="n">
+        <v>1</v>
+      </c>
+      <c r="BX46" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7164,6 +8725,9 @@
       <c r="AY47" t="n">
         <v>1</v>
       </c>
+      <c r="AZ47" t="n">
+        <v>1</v>
+      </c>
       <c r="BA47" t="n">
         <v>1</v>
       </c>
@@ -7186,6 +8750,36 @@
         <v>1</v>
       </c>
       <c r="BJ47" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM47" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN47" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO47" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP47" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ47" t="n">
+        <v>1</v>
+      </c>
+      <c r="BT47" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU47" t="n">
+        <v>1</v>
+      </c>
+      <c r="BV47" t="n">
+        <v>1</v>
+      </c>
+      <c r="BW47" t="n">
+        <v>1</v>
+      </c>
+      <c r="BX47" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7303,6 +8897,9 @@
       <c r="AY48" t="n">
         <v>0</v>
       </c>
+      <c r="AZ48" t="n">
+        <v>0</v>
+      </c>
       <c r="BA48" t="n">
         <v>0</v>
       </c>
@@ -7325,6 +8922,36 @@
         <v>0</v>
       </c>
       <c r="BJ48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX48" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7442,6 +9069,9 @@
       <c r="AY49" t="n">
         <v>158</v>
       </c>
+      <c r="AZ49" t="n">
+        <v>64</v>
+      </c>
       <c r="BA49" t="n">
         <v>67</v>
       </c>
@@ -7464,6 +9094,36 @@
         <v>155</v>
       </c>
       <c r="BJ49" t="n">
+        <v>158</v>
+      </c>
+      <c r="BM49" t="n">
+        <v>158</v>
+      </c>
+      <c r="BN49" t="n">
+        <v>64</v>
+      </c>
+      <c r="BO49" t="n">
+        <v>67</v>
+      </c>
+      <c r="BP49" t="n">
+        <v>155</v>
+      </c>
+      <c r="BQ49" t="n">
+        <v>158</v>
+      </c>
+      <c r="BT49" t="n">
+        <v>158</v>
+      </c>
+      <c r="BU49" t="n">
+        <v>64</v>
+      </c>
+      <c r="BV49" t="n">
+        <v>67</v>
+      </c>
+      <c r="BW49" t="n">
+        <v>155</v>
+      </c>
+      <c r="BX49" t="n">
         <v>158</v>
       </c>
     </row>
@@ -7581,6 +9241,9 @@
       <c r="AY50" t="n">
         <v>158</v>
       </c>
+      <c r="AZ50" t="n">
+        <v>64</v>
+      </c>
       <c r="BA50" t="n">
         <v>67</v>
       </c>
@@ -7603,6 +9266,36 @@
         <v>155</v>
       </c>
       <c r="BJ50" t="n">
+        <v>158</v>
+      </c>
+      <c r="BM50" t="n">
+        <v>158</v>
+      </c>
+      <c r="BN50" t="n">
+        <v>64</v>
+      </c>
+      <c r="BO50" t="n">
+        <v>67</v>
+      </c>
+      <c r="BP50" t="n">
+        <v>155</v>
+      </c>
+      <c r="BQ50" t="n">
+        <v>158</v>
+      </c>
+      <c r="BT50" t="n">
+        <v>158</v>
+      </c>
+      <c r="BU50" t="n">
+        <v>64</v>
+      </c>
+      <c r="BV50" t="n">
+        <v>67</v>
+      </c>
+      <c r="BW50" t="n">
+        <v>155</v>
+      </c>
+      <c r="BX50" t="n">
         <v>158</v>
       </c>
     </row>
@@ -7720,6 +9413,9 @@
       <c r="AY51" t="n">
         <v>0</v>
       </c>
+      <c r="AZ51" t="n">
+        <v>0</v>
+      </c>
       <c r="BA51" t="n">
         <v>0</v>
       </c>
@@ -7742,6 +9438,36 @@
         <v>0</v>
       </c>
       <c r="BJ51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX51" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7859,6 +9585,9 @@
       <c r="AY52" t="n">
         <v>0</v>
       </c>
+      <c r="AZ52" t="n">
+        <v>0</v>
+      </c>
       <c r="BA52" t="n">
         <v>0</v>
       </c>
@@ -7881,6 +9610,36 @@
         <v>0</v>
       </c>
       <c r="BJ52" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM52" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN52" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO52" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP52" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ52" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT52" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU52" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV52" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW52" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX52" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7998,6 +9757,9 @@
       <c r="AY53" t="n">
         <v>0</v>
       </c>
+      <c r="AZ53" t="n">
+        <v>0</v>
+      </c>
       <c r="BA53" t="n">
         <v>0</v>
       </c>
@@ -8020,6 +9782,36 @@
         <v>0</v>
       </c>
       <c r="BJ53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX53" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8137,6 +9929,9 @@
       <c r="AY54" t="n">
         <v>0</v>
       </c>
+      <c r="AZ54" t="n">
+        <v>0</v>
+      </c>
       <c r="BA54" t="n">
         <v>0</v>
       </c>
@@ -8159,6 +9954,36 @@
         <v>0</v>
       </c>
       <c r="BJ54" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM54" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN54" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO54" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP54" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ54" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT54" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU54" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV54" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW54" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX54" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8276,6 +10101,9 @@
       <c r="AY55" t="n">
         <v>102</v>
       </c>
+      <c r="AZ55" t="n">
+        <v>69</v>
+      </c>
       <c r="BA55" t="n">
         <v>133</v>
       </c>
@@ -8298,6 +10126,36 @@
         <v>119</v>
       </c>
       <c r="BJ55" t="n">
+        <v>43</v>
+      </c>
+      <c r="BM55" t="n">
+        <v>102</v>
+      </c>
+      <c r="BN55" t="n">
+        <v>69</v>
+      </c>
+      <c r="BO55" t="n">
+        <v>133</v>
+      </c>
+      <c r="BP55" t="n">
+        <v>119</v>
+      </c>
+      <c r="BQ55" t="n">
+        <v>43</v>
+      </c>
+      <c r="BT55" t="n">
+        <v>102</v>
+      </c>
+      <c r="BU55" t="n">
+        <v>69</v>
+      </c>
+      <c r="BV55" t="n">
+        <v>133</v>
+      </c>
+      <c r="BW55" t="n">
+        <v>119</v>
+      </c>
+      <c r="BX55" t="n">
         <v>43</v>
       </c>
     </row>
@@ -8415,6 +10273,9 @@
       <c r="AY56" t="n">
         <v>102</v>
       </c>
+      <c r="AZ56" t="n">
+        <v>69</v>
+      </c>
       <c r="BA56" t="n">
         <v>133</v>
       </c>
@@ -8437,6 +10298,36 @@
         <v>119</v>
       </c>
       <c r="BJ56" t="n">
+        <v>43</v>
+      </c>
+      <c r="BM56" t="n">
+        <v>102</v>
+      </c>
+      <c r="BN56" t="n">
+        <v>69</v>
+      </c>
+      <c r="BO56" t="n">
+        <v>133</v>
+      </c>
+      <c r="BP56" t="n">
+        <v>119</v>
+      </c>
+      <c r="BQ56" t="n">
+        <v>43</v>
+      </c>
+      <c r="BT56" t="n">
+        <v>102</v>
+      </c>
+      <c r="BU56" t="n">
+        <v>69</v>
+      </c>
+      <c r="BV56" t="n">
+        <v>133</v>
+      </c>
+      <c r="BW56" t="n">
+        <v>119</v>
+      </c>
+      <c r="BX56" t="n">
         <v>43</v>
       </c>
     </row>
@@ -8554,6 +10445,9 @@
       <c r="AY57" t="n">
         <v>0</v>
       </c>
+      <c r="AZ57" t="n">
+        <v>0</v>
+      </c>
       <c r="BA57" t="n">
         <v>0</v>
       </c>
@@ -8576,6 +10470,36 @@
         <v>0</v>
       </c>
       <c r="BJ57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX57" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8693,6 +10617,9 @@
       <c r="AY58" t="n">
         <v>28</v>
       </c>
+      <c r="AZ58" t="n">
+        <v>114</v>
+      </c>
       <c r="BA58" t="n">
         <v>24</v>
       </c>
@@ -8715,6 +10642,36 @@
         <v>265</v>
       </c>
       <c r="BJ58" t="n">
+        <v>244</v>
+      </c>
+      <c r="BM58" t="n">
+        <v>28</v>
+      </c>
+      <c r="BN58" t="n">
+        <v>114</v>
+      </c>
+      <c r="BO58" t="n">
+        <v>24</v>
+      </c>
+      <c r="BP58" t="n">
+        <v>265</v>
+      </c>
+      <c r="BQ58" t="n">
+        <v>244</v>
+      </c>
+      <c r="BT58" t="n">
+        <v>28</v>
+      </c>
+      <c r="BU58" t="n">
+        <v>114</v>
+      </c>
+      <c r="BV58" t="n">
+        <v>24</v>
+      </c>
+      <c r="BW58" t="n">
+        <v>265</v>
+      </c>
+      <c r="BX58" t="n">
         <v>244</v>
       </c>
     </row>
@@ -8832,6 +10789,9 @@
       <c r="AY59" t="n">
         <v>28</v>
       </c>
+      <c r="AZ59" t="n">
+        <v>112</v>
+      </c>
       <c r="BA59" t="n">
         <v>24</v>
       </c>
@@ -8855,6 +10815,36 @@
       </c>
       <c r="BJ59" t="n">
         <v>222</v>
+      </c>
+      <c r="BM59" t="n">
+        <v>28</v>
+      </c>
+      <c r="BN59" s="5" t="n">
+        <v>114</v>
+      </c>
+      <c r="BO59" t="n">
+        <v>24</v>
+      </c>
+      <c r="BP59" s="5" t="n">
+        <v>265</v>
+      </c>
+      <c r="BQ59" s="5" t="n">
+        <v>244</v>
+      </c>
+      <c r="BT59" t="n">
+        <v>28</v>
+      </c>
+      <c r="BU59" t="n">
+        <v>114</v>
+      </c>
+      <c r="BV59" t="n">
+        <v>24</v>
+      </c>
+      <c r="BW59" t="n">
+        <v>265</v>
+      </c>
+      <c r="BX59" t="n">
+        <v>244</v>
       </c>
     </row>
     <row r="60">
@@ -8971,6 +10961,9 @@
       <c r="AY60" t="n">
         <v>0</v>
       </c>
+      <c r="AZ60" t="n">
+        <v>2</v>
+      </c>
       <c r="BA60" t="n">
         <v>0</v>
       </c>
@@ -8994,6 +10987,36 @@
       </c>
       <c r="BJ60" t="n">
         <v>22</v>
+      </c>
+      <c r="BM60" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN60" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO60" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP60" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ60" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT60" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU60" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV60" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW60" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX60" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="61">
@@ -9110,6 +11133,9 @@
       <c r="AY61" t="n">
         <v>9</v>
       </c>
+      <c r="AZ61" t="n">
+        <v>2</v>
+      </c>
       <c r="BA61" t="n">
         <v>38</v>
       </c>
@@ -9132,6 +11158,36 @@
         <v>105</v>
       </c>
       <c r="BJ61" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM61" t="n">
+        <v>9</v>
+      </c>
+      <c r="BN61" t="n">
+        <v>2</v>
+      </c>
+      <c r="BO61" t="n">
+        <v>38</v>
+      </c>
+      <c r="BP61" t="n">
+        <v>105</v>
+      </c>
+      <c r="BQ61" t="n">
+        <v>1</v>
+      </c>
+      <c r="BT61" t="n">
+        <v>9</v>
+      </c>
+      <c r="BU61" t="n">
+        <v>2</v>
+      </c>
+      <c r="BV61" t="n">
+        <v>38</v>
+      </c>
+      <c r="BW61" t="n">
+        <v>105</v>
+      </c>
+      <c r="BX61" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9249,6 +11305,9 @@
       <c r="AY62" t="n">
         <v>8</v>
       </c>
+      <c r="AZ62" t="n">
+        <v>2</v>
+      </c>
       <c r="BA62" t="n">
         <v>38</v>
       </c>
@@ -9271,6 +11330,36 @@
         <v>103</v>
       </c>
       <c r="BJ62" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM62" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="BN62" t="n">
+        <v>2</v>
+      </c>
+      <c r="BO62" t="n">
+        <v>38</v>
+      </c>
+      <c r="BP62" s="5" t="n">
+        <v>105</v>
+      </c>
+      <c r="BQ62" t="n">
+        <v>1</v>
+      </c>
+      <c r="BT62" t="n">
+        <v>9</v>
+      </c>
+      <c r="BU62" t="n">
+        <v>2</v>
+      </c>
+      <c r="BV62" t="n">
+        <v>38</v>
+      </c>
+      <c r="BW62" t="n">
+        <v>105</v>
+      </c>
+      <c r="BX62" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9388,6 +11477,9 @@
       <c r="AY63" t="n">
         <v>1</v>
       </c>
+      <c r="AZ63" t="n">
+        <v>0</v>
+      </c>
       <c r="BA63" t="n">
         <v>0</v>
       </c>
@@ -9410,6 +11502,36 @@
         <v>2</v>
       </c>
       <c r="BJ63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM63" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP63" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX63" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9527,6 +11649,9 @@
       <c r="AY64" t="n">
         <v>0</v>
       </c>
+      <c r="AZ64" t="n">
+        <v>0</v>
+      </c>
       <c r="BA64" t="n">
         <v>0</v>
       </c>
@@ -9549,6 +11674,36 @@
         <v>0</v>
       </c>
       <c r="BJ64" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM64" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN64" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO64" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP64" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ64" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT64" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU64" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV64" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW64" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX64" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9666,6 +11821,9 @@
       <c r="AY65" t="n">
         <v>0</v>
       </c>
+      <c r="AZ65" t="n">
+        <v>0</v>
+      </c>
       <c r="BA65" t="n">
         <v>0</v>
       </c>
@@ -9688,6 +11846,36 @@
         <v>0</v>
       </c>
       <c r="BJ65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX65" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9805,6 +11993,9 @@
       <c r="AY66" t="n">
         <v>0</v>
       </c>
+      <c r="AZ66" t="n">
+        <v>0</v>
+      </c>
       <c r="BA66" t="n">
         <v>0</v>
       </c>
@@ -9827,6 +12018,36 @@
         <v>0</v>
       </c>
       <c r="BJ66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX66" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9944,6 +12165,9 @@
       <c r="AY67" t="n">
         <v>68</v>
       </c>
+      <c r="AZ67" t="n">
+        <v>165</v>
+      </c>
       <c r="BA67" t="n">
         <v>459</v>
       </c>
@@ -9966,6 +12190,36 @@
         <v>38</v>
       </c>
       <c r="BJ67" t="n">
+        <v>4</v>
+      </c>
+      <c r="BM67" t="n">
+        <v>68</v>
+      </c>
+      <c r="BN67" t="n">
+        <v>165</v>
+      </c>
+      <c r="BO67" t="n">
+        <v>459</v>
+      </c>
+      <c r="BP67" t="n">
+        <v>38</v>
+      </c>
+      <c r="BQ67" t="n">
+        <v>4</v>
+      </c>
+      <c r="BT67" t="n">
+        <v>68</v>
+      </c>
+      <c r="BU67" t="n">
+        <v>165</v>
+      </c>
+      <c r="BV67" t="n">
+        <v>459</v>
+      </c>
+      <c r="BW67" t="n">
+        <v>38</v>
+      </c>
+      <c r="BX67" t="n">
         <v>4</v>
       </c>
     </row>
@@ -10083,6 +12337,9 @@
       <c r="AY68" t="n">
         <v>68</v>
       </c>
+      <c r="AZ68" t="n">
+        <v>165</v>
+      </c>
       <c r="BA68" t="n">
         <v>459</v>
       </c>
@@ -10105,6 +12362,36 @@
         <v>38</v>
       </c>
       <c r="BJ68" t="n">
+        <v>4</v>
+      </c>
+      <c r="BM68" t="n">
+        <v>68</v>
+      </c>
+      <c r="BN68" t="n">
+        <v>165</v>
+      </c>
+      <c r="BO68" t="n">
+        <v>459</v>
+      </c>
+      <c r="BP68" t="n">
+        <v>38</v>
+      </c>
+      <c r="BQ68" t="n">
+        <v>4</v>
+      </c>
+      <c r="BT68" t="n">
+        <v>68</v>
+      </c>
+      <c r="BU68" t="n">
+        <v>165</v>
+      </c>
+      <c r="BV68" t="n">
+        <v>459</v>
+      </c>
+      <c r="BW68" t="n">
+        <v>38</v>
+      </c>
+      <c r="BX68" t="n">
         <v>4</v>
       </c>
     </row>
@@ -10222,6 +12509,9 @@
       <c r="AY69" t="n">
         <v>0</v>
       </c>
+      <c r="AZ69" t="n">
+        <v>0</v>
+      </c>
       <c r="BA69" t="n">
         <v>0</v>
       </c>
@@ -10244,6 +12534,36 @@
         <v>0</v>
       </c>
       <c r="BJ69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX69" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10361,6 +12681,9 @@
       <c r="AY70" t="n">
         <v>65</v>
       </c>
+      <c r="AZ70" t="n">
+        <v>36</v>
+      </c>
       <c r="BA70" t="n">
         <v>102</v>
       </c>
@@ -10383,6 +12706,36 @@
         <v>83</v>
       </c>
       <c r="BJ70" t="n">
+        <v>40</v>
+      </c>
+      <c r="BM70" t="n">
+        <v>65</v>
+      </c>
+      <c r="BN70" t="n">
+        <v>36</v>
+      </c>
+      <c r="BO70" t="n">
+        <v>102</v>
+      </c>
+      <c r="BP70" t="n">
+        <v>83</v>
+      </c>
+      <c r="BQ70" t="n">
+        <v>40</v>
+      </c>
+      <c r="BT70" t="n">
+        <v>65</v>
+      </c>
+      <c r="BU70" t="n">
+        <v>36</v>
+      </c>
+      <c r="BV70" t="n">
+        <v>102</v>
+      </c>
+      <c r="BW70" t="n">
+        <v>83</v>
+      </c>
+      <c r="BX70" t="n">
         <v>40</v>
       </c>
     </row>
@@ -10500,6 +12853,9 @@
       <c r="AY71" t="n">
         <v>59</v>
       </c>
+      <c r="AZ71" t="n">
+        <v>30</v>
+      </c>
       <c r="BA71" t="n">
         <v>97</v>
       </c>
@@ -10523,6 +12879,36 @@
       </c>
       <c r="BJ71" t="n">
         <v>34</v>
+      </c>
+      <c r="BM71" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="BN71" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="BO71" s="5" t="n">
+        <v>102</v>
+      </c>
+      <c r="BP71" s="5" t="n">
+        <v>83</v>
+      </c>
+      <c r="BQ71" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="BT71" t="n">
+        <v>65</v>
+      </c>
+      <c r="BU71" t="n">
+        <v>36</v>
+      </c>
+      <c r="BV71" t="n">
+        <v>102</v>
+      </c>
+      <c r="BW71" t="n">
+        <v>83</v>
+      </c>
+      <c r="BX71" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="72">
@@ -10639,6 +13025,9 @@
       <c r="AY72" t="n">
         <v>6</v>
       </c>
+      <c r="AZ72" t="n">
+        <v>6</v>
+      </c>
       <c r="BA72" t="n">
         <v>5</v>
       </c>
@@ -10662,6 +13051,36 @@
       </c>
       <c r="BJ72" t="n">
         <v>6</v>
+      </c>
+      <c r="BM72" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN72" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO72" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP72" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ72" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX72" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -10778,6 +13197,9 @@
       <c r="AY73" t="n">
         <v>0</v>
       </c>
+      <c r="AZ73" t="n">
+        <v>0</v>
+      </c>
       <c r="BA73" t="n">
         <v>0</v>
       </c>
@@ -10800,6 +13222,36 @@
         <v>0</v>
       </c>
       <c r="BJ73" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM73" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN73" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO73" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP73" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ73" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT73" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU73" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV73" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW73" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX73" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10917,6 +13369,9 @@
       <c r="AY74" t="n">
         <v>0</v>
       </c>
+      <c r="AZ74" t="n">
+        <v>0</v>
+      </c>
       <c r="BA74" t="n">
         <v>0</v>
       </c>
@@ -10939,6 +13394,36 @@
         <v>0</v>
       </c>
       <c r="BJ74" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM74" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN74" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO74" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP74" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ74" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT74" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU74" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV74" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW74" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX74" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11056,6 +13541,9 @@
       <c r="AY75" t="n">
         <v>0</v>
       </c>
+      <c r="AZ75" t="n">
+        <v>0</v>
+      </c>
       <c r="BA75" t="n">
         <v>0</v>
       </c>
@@ -11078,6 +13566,36 @@
         <v>0</v>
       </c>
       <c r="BJ75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX75" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11195,6 +13713,9 @@
       <c r="AY76" t="n">
         <v>0</v>
       </c>
+      <c r="AZ76" t="n">
+        <v>0</v>
+      </c>
       <c r="BA76" t="n">
         <v>0</v>
       </c>
@@ -11217,6 +13738,36 @@
         <v>0</v>
       </c>
       <c r="BJ76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW76" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX76" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11334,6 +13885,9 @@
       <c r="AY77" t="n">
         <v>0</v>
       </c>
+      <c r="AZ77" t="n">
+        <v>0</v>
+      </c>
       <c r="BA77" t="n">
         <v>0</v>
       </c>
@@ -11356,6 +13910,36 @@
         <v>0</v>
       </c>
       <c r="BJ77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW77" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX77" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11473,6 +14057,9 @@
       <c r="AY78" t="n">
         <v>0</v>
       </c>
+      <c r="AZ78" t="n">
+        <v>0</v>
+      </c>
       <c r="BA78" t="n">
         <v>0</v>
       </c>
@@ -11495,6 +14082,36 @@
         <v>0</v>
       </c>
       <c r="BJ78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW78" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX78" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11612,6 +14229,9 @@
       <c r="AY79" t="n">
         <v>0</v>
       </c>
+      <c r="AZ79" t="n">
+        <v>0</v>
+      </c>
       <c r="BA79" t="n">
         <v>0</v>
       </c>
@@ -11634,6 +14254,36 @@
         <v>0</v>
       </c>
       <c r="BJ79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW79" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX79" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11751,6 +14401,9 @@
       <c r="AY80" t="n">
         <v>0</v>
       </c>
+      <c r="AZ80" t="n">
+        <v>0</v>
+      </c>
       <c r="BA80" t="n">
         <v>0</v>
       </c>
@@ -11773,6 +14426,36 @@
         <v>0</v>
       </c>
       <c r="BJ80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW80" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX80" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11890,6 +14573,9 @@
       <c r="AY81" t="n">
         <v>0</v>
       </c>
+      <c r="AZ81" t="n">
+        <v>0</v>
+      </c>
       <c r="BA81" t="n">
         <v>0</v>
       </c>
@@ -11912,6 +14598,36 @@
         <v>0</v>
       </c>
       <c r="BJ81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW81" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX81" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12029,6 +14745,9 @@
       <c r="AY82" t="n">
         <v>0</v>
       </c>
+      <c r="AZ82" t="n">
+        <v>0</v>
+      </c>
       <c r="BA82" t="n">
         <v>0</v>
       </c>
@@ -12051,6 +14770,36 @@
         <v>0</v>
       </c>
       <c r="BJ82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW82" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX82" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12168,6 +14917,9 @@
       <c r="AY83" t="n">
         <v>0</v>
       </c>
+      <c r="AZ83" t="n">
+        <v>0</v>
+      </c>
       <c r="BA83" t="n">
         <v>0</v>
       </c>
@@ -12190,6 +14942,36 @@
         <v>0</v>
       </c>
       <c r="BJ83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW83" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX83" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12307,6 +15089,9 @@
       <c r="AY84" t="n">
         <v>0</v>
       </c>
+      <c r="AZ84" t="n">
+        <v>0</v>
+      </c>
       <c r="BA84" t="n">
         <v>0</v>
       </c>
@@ -12329,6 +15114,36 @@
         <v>0</v>
       </c>
       <c r="BJ84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW84" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX84" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12446,6 +15261,9 @@
       <c r="AY85" t="n">
         <v>0</v>
       </c>
+      <c r="AZ85" t="n">
+        <v>0</v>
+      </c>
       <c r="BA85" t="n">
         <v>0</v>
       </c>
@@ -12468,6 +15286,36 @@
         <v>0</v>
       </c>
       <c r="BJ85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW85" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX85" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12585,6 +15433,9 @@
       <c r="AY86" t="n">
         <v>0</v>
       </c>
+      <c r="AZ86" t="n">
+        <v>0</v>
+      </c>
       <c r="BA86" t="n">
         <v>0</v>
       </c>
@@ -12607,6 +15458,36 @@
         <v>0</v>
       </c>
       <c r="BJ86" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM86" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN86" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO86" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP86" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ86" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT86" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU86" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV86" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW86" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX86" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12724,6 +15605,9 @@
       <c r="AY87" t="n">
         <v>0</v>
       </c>
+      <c r="AZ87" t="n">
+        <v>0</v>
+      </c>
       <c r="BA87" t="n">
         <v>0</v>
       </c>
@@ -12746,6 +15630,36 @@
         <v>0</v>
       </c>
       <c r="BJ87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW87" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX87" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12863,6 +15777,9 @@
       <c r="AY88" t="n">
         <v>0</v>
       </c>
+      <c r="AZ88" t="n">
+        <v>0</v>
+      </c>
       <c r="BA88" t="n">
         <v>0</v>
       </c>
@@ -12885,6 +15802,36 @@
         <v>0</v>
       </c>
       <c r="BJ88" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM88" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN88" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO88" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP88" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ88" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT88" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU88" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV88" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW88" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX88" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13002,6 +15949,9 @@
       <c r="AY89" t="n">
         <v>0</v>
       </c>
+      <c r="AZ89" t="n">
+        <v>0</v>
+      </c>
       <c r="BA89" t="n">
         <v>0</v>
       </c>
@@ -13024,6 +15974,36 @@
         <v>0</v>
       </c>
       <c r="BJ89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW89" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX89" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13141,6 +16121,9 @@
       <c r="AY90" t="n">
         <v>0</v>
       </c>
+      <c r="AZ90" t="n">
+        <v>0</v>
+      </c>
       <c r="BA90" t="n">
         <v>0</v>
       </c>
@@ -13163,6 +16146,36 @@
         <v>0</v>
       </c>
       <c r="BJ90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW90" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX90" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13280,6 +16293,9 @@
       <c r="AY91" t="n">
         <v>0</v>
       </c>
+      <c r="AZ91" t="n">
+        <v>0</v>
+      </c>
       <c r="BA91" t="n">
         <v>0</v>
       </c>
@@ -13302,6 +16318,36 @@
         <v>0</v>
       </c>
       <c r="BJ91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX91" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13419,6 +16465,9 @@
       <c r="AY92" t="n">
         <v>0</v>
       </c>
+      <c r="AZ92" t="n">
+        <v>0</v>
+      </c>
       <c r="BA92" t="n">
         <v>0</v>
       </c>
@@ -13441,6 +16490,36 @@
         <v>0</v>
       </c>
       <c r="BJ92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW92" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX92" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13558,6 +16637,9 @@
       <c r="AY93" t="n">
         <v>0</v>
       </c>
+      <c r="AZ93" t="n">
+        <v>0</v>
+      </c>
       <c r="BA93" t="n">
         <v>0</v>
       </c>
@@ -13580,6 +16662,36 @@
         <v>0</v>
       </c>
       <c r="BJ93" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM93" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN93" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO93" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP93" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ93" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT93" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU93" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV93" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW93" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX93" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13697,6 +16809,9 @@
       <c r="AY94" t="n">
         <v>0</v>
       </c>
+      <c r="AZ94" t="n">
+        <v>0</v>
+      </c>
       <c r="BA94" t="n">
         <v>0</v>
       </c>
@@ -13719,6 +16834,36 @@
         <v>0</v>
       </c>
       <c r="BJ94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW94" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX94" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13836,6 +16981,9 @@
       <c r="AY95" t="n">
         <v>0</v>
       </c>
+      <c r="AZ95" t="n">
+        <v>0</v>
+      </c>
       <c r="BA95" t="n">
         <v>0</v>
       </c>
@@ -13858,6 +17006,36 @@
         <v>0</v>
       </c>
       <c r="BJ95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW95" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX95" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13975,6 +17153,9 @@
       <c r="AY96" t="n">
         <v>0</v>
       </c>
+      <c r="AZ96" t="n">
+        <v>0</v>
+      </c>
       <c r="BA96" t="n">
         <v>0</v>
       </c>
@@ -13997,15 +17178,47 @@
         <v>0</v>
       </c>
       <c r="BJ96" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM96" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN96" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO96" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP96" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ96" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT96" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU96" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV96" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW96" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX96" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="11">
     <mergeCell ref="AD1:AI1"/>
     <mergeCell ref="AR1:AW1"/>
     <mergeCell ref="P1:U1"/>
+    <mergeCell ref="BM1:BR1"/>
     <mergeCell ref="AK1:AP1"/>
+    <mergeCell ref="BT1:BY1"/>
     <mergeCell ref="W1:AB1"/>
     <mergeCell ref="AY1:BD1"/>
     <mergeCell ref="B1:G1"/>

</xml_diff>

<commit_message>
Image fix, new method pdf-extract-kit
</commit_message>
<xml_diff>
--- a/tests/regression_test/results/master_results.xlsx
+++ b/tests/regression_test/results/master_results.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CM121"/>
+  <dimension ref="A1:CT121"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30.33203125" customWidth="1" style="4" min="1" max="1"/>
@@ -517,6 +517,11 @@
           <t>Index fix</t>
         </is>
       </c>
+      <c r="CO1" s="3" t="inlineStr">
+        <is>
+          <t>img_fix</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -914,6 +919,36 @@
           <t>avg.</t>
         </is>
       </c>
+      <c r="CO2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="CP2" t="inlineStr">
+        <is>
+          <t>algorithms</t>
+        </is>
+      </c>
+      <c r="CQ2" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="CR2" t="inlineStr">
+        <is>
+          <t>cybersec</t>
+        </is>
+      </c>
+      <c r="CS2" t="inlineStr">
+        <is>
+          <t>data-science</t>
+        </is>
+      </c>
+      <c r="CT2" t="inlineStr">
+        <is>
+          <t>avg.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1241,6 +1276,31 @@
           <t>data-science</t>
         </is>
       </c>
+      <c r="CO3" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="CP3" t="inlineStr">
+        <is>
+          <t>algorithms</t>
+        </is>
+      </c>
+      <c r="CQ3" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="CR3" t="inlineStr">
+        <is>
+          <t>cybersec</t>
+        </is>
+      </c>
+      <c r="CS3" t="inlineStr">
+        <is>
+          <t>data-science</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1568,6 +1628,31 @@
           <t>multi-metric</t>
         </is>
       </c>
+      <c r="CO4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="CP4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="CQ4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="CR4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="CS4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1895,6 +1980,31 @@
           <t>2025-11-09T16:01:38.289528</t>
         </is>
       </c>
+      <c r="CO5" t="inlineStr">
+        <is>
+          <t>2025-11-30T20:18:34.117072</t>
+        </is>
+      </c>
+      <c r="CP5" t="inlineStr">
+        <is>
+          <t>2025-11-30T20:18:34.314666</t>
+        </is>
+      </c>
+      <c r="CQ5" t="inlineStr">
+        <is>
+          <t>2025-11-30T20:18:34.471072</t>
+        </is>
+      </c>
+      <c r="CR5" t="inlineStr">
+        <is>
+          <t>2025-11-30T20:18:34.639656</t>
+        </is>
+      </c>
+      <c r="CS5" t="inlineStr">
+        <is>
+          <t>2025-11-30T20:18:34.787168</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2133,6 +2243,24 @@
       <c r="CM6" s="5" t="n">
         <v>-116.84</v>
       </c>
+      <c r="CO6" s="5" t="n">
+        <v>-61.3</v>
+      </c>
+      <c r="CP6" s="5" t="n">
+        <v>-198.7</v>
+      </c>
+      <c r="CQ6" s="5" t="n">
+        <v>-28.3</v>
+      </c>
+      <c r="CR6" s="5" t="n">
+        <v>-87.09999999999999</v>
+      </c>
+      <c r="CS6" s="5" t="n">
+        <v>-56.3</v>
+      </c>
+      <c r="CT6" s="5" t="n">
+        <v>-86.34</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2332,6 +2460,21 @@
       <c r="CL7" t="n">
         <v>100</v>
       </c>
+      <c r="CO7" t="n">
+        <v>88.23999999999999</v>
+      </c>
+      <c r="CP7" t="n">
+        <v>65.25</v>
+      </c>
+      <c r="CQ7" t="n">
+        <v>100</v>
+      </c>
+      <c r="CR7" t="n">
+        <v>100</v>
+      </c>
+      <c r="CS7" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2531,6 +2674,21 @@
       <c r="CL8" t="n">
         <v>7</v>
       </c>
+      <c r="CO8" t="n">
+        <v>15.87</v>
+      </c>
+      <c r="CP8" t="n">
+        <v>6.13</v>
+      </c>
+      <c r="CQ8" t="n">
+        <v>7</v>
+      </c>
+      <c r="CR8" t="n">
+        <v>18</v>
+      </c>
+      <c r="CS8" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2730,6 +2888,21 @@
       <c r="CL9" s="6" t="n">
         <v>101</v>
       </c>
+      <c r="CO9" t="n">
+        <v>196.06</v>
+      </c>
+      <c r="CP9" t="n">
+        <v>53.64</v>
+      </c>
+      <c r="CQ9" t="n">
+        <v>5</v>
+      </c>
+      <c r="CR9" t="n">
+        <v>91</v>
+      </c>
+      <c r="CS9" t="n">
+        <v>101</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2929,6 +3102,21 @@
       <c r="CL10" s="5" t="n">
         <v>100</v>
       </c>
+      <c r="CO10" t="n">
+        <v>100</v>
+      </c>
+      <c r="CP10" t="n">
+        <v>100</v>
+      </c>
+      <c r="CQ10" t="n">
+        <v>100</v>
+      </c>
+      <c r="CR10" t="n">
+        <v>100</v>
+      </c>
+      <c r="CS10" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3128,6 +3316,21 @@
       <c r="CL11" s="5" t="n">
         <v>86.79000000000001</v>
       </c>
+      <c r="CO11" t="n">
+        <v>99.56999999999999</v>
+      </c>
+      <c r="CP11" t="n">
+        <v>90.84</v>
+      </c>
+      <c r="CQ11" t="n">
+        <v>100</v>
+      </c>
+      <c r="CR11" t="n">
+        <v>100</v>
+      </c>
+      <c r="CS11" t="n">
+        <v>86.79000000000001</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3327,6 +3530,21 @@
       <c r="CL12" t="n">
         <v>130.77</v>
       </c>
+      <c r="CO12" t="n">
+        <v>100</v>
+      </c>
+      <c r="CP12" t="n">
+        <v>118.18</v>
+      </c>
+      <c r="CQ12" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="CR12" t="n">
+        <v>90.48</v>
+      </c>
+      <c r="CS12" t="n">
+        <v>130.77</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3526,6 +3744,21 @@
       <c r="CL13" t="n">
         <v>80</v>
       </c>
+      <c r="CO13" t="n">
+        <v>98.97</v>
+      </c>
+      <c r="CP13" t="n">
+        <v>101.5</v>
+      </c>
+      <c r="CQ13" t="n">
+        <v>92.06</v>
+      </c>
+      <c r="CR13" t="n">
+        <v>83.75</v>
+      </c>
+      <c r="CS13" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3725,6 +3958,21 @@
       <c r="CL14" t="n">
         <v>89.39</v>
       </c>
+      <c r="CO14" t="n">
+        <v>92.59</v>
+      </c>
+      <c r="CP14" t="n">
+        <v>97.62</v>
+      </c>
+      <c r="CQ14" t="n">
+        <v>100</v>
+      </c>
+      <c r="CR14" t="n">
+        <v>97.04000000000001</v>
+      </c>
+      <c r="CS14" t="n">
+        <v>89.39</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3924,6 +4172,21 @@
       <c r="CL15" t="n">
         <v>88.76000000000001</v>
       </c>
+      <c r="CO15" s="6" t="n">
+        <v>86.81</v>
+      </c>
+      <c r="CP15" s="5" t="n">
+        <v>29.91</v>
+      </c>
+      <c r="CQ15" s="6" t="n">
+        <v>106.35</v>
+      </c>
+      <c r="CR15" s="6" t="n">
+        <v>87.56999999999999</v>
+      </c>
+      <c r="CS15" s="5" t="n">
+        <v>91.86</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4123,6 +4386,21 @@
       <c r="CL16" t="n">
         <v>58.11</v>
       </c>
+      <c r="CO16" s="5" t="n">
+        <v>159.38</v>
+      </c>
+      <c r="CP16" s="6" t="n">
+        <v>164.29</v>
+      </c>
+      <c r="CQ16" s="6" t="n">
+        <v>81.09999999999999</v>
+      </c>
+      <c r="CR16" s="6" t="n">
+        <v>224.53</v>
+      </c>
+      <c r="CS16" s="5" t="n">
+        <v>134.38</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4322,6 +4600,21 @@
       <c r="CL17" s="5" t="n">
         <v>99.40000000000001</v>
       </c>
+      <c r="CO17" t="n">
+        <v>99.31999999999999</v>
+      </c>
+      <c r="CP17" t="n">
+        <v>89.02</v>
+      </c>
+      <c r="CQ17" t="n">
+        <v>100.92</v>
+      </c>
+      <c r="CR17" t="n">
+        <v>96</v>
+      </c>
+      <c r="CS17" t="n">
+        <v>99.40000000000001</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4329,7 +4622,7 @@
           <t>------------</t>
         </is>
       </c>
-      <c r="CL18" t="inlineStr"/>
+      <c r="CS18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4337,7 +4630,7 @@
           <t>Score Deductions:</t>
         </is>
       </c>
-      <c r="CL19" t="inlineStr"/>
+      <c r="CS19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4537,6 +4830,21 @@
       <c r="CL20" s="6" t="n">
         <v>5.05</v>
       </c>
+      <c r="CO20" s="6" t="n">
+        <v>11.42</v>
+      </c>
+      <c r="CP20" s="6" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="CQ20" s="6" t="n">
+        <v>12.37</v>
+      </c>
+      <c r="CR20" s="6" t="n">
+        <v>10.33</v>
+      </c>
+      <c r="CS20" s="6" t="n">
+        <v>6.22</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4736,6 +5044,21 @@
       <c r="CL21" s="6" t="n">
         <v>14.57</v>
       </c>
+      <c r="CO21" s="6" t="n">
+        <v>28.22</v>
+      </c>
+      <c r="CP21" s="6" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="CQ21" s="6" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="CR21" s="6" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="CS21" s="6" t="n">
+        <v>17.94</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4935,6 +5258,21 @@
       <c r="CL22" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="CO22" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP22" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ22" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR22" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5134,6 +5472,21 @@
       <c r="CL23" s="6" t="n">
         <v>10.1</v>
       </c>
+      <c r="CO23" s="6" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="CP23" s="6" t="n">
+        <v>20.89</v>
+      </c>
+      <c r="CQ23" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR23" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS23" s="6" t="n">
+        <v>12.43</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5333,6 +5686,21 @@
       <c r="CL24" s="6" t="n">
         <v>2.89</v>
       </c>
+      <c r="CO24" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP24" s="6" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="CQ24" s="6" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="CR24" s="6" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="CS24" s="6" t="n">
+        <v>3.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5532,6 +5900,21 @@
       <c r="CL25" s="6" t="n">
         <v>15.15</v>
       </c>
+      <c r="CO25" s="6" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="CP25" s="6" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="CQ25" s="6" t="n">
+        <v>17.67</v>
+      </c>
+      <c r="CR25" s="6" t="n">
+        <v>7.46</v>
+      </c>
+      <c r="CS25" s="6" t="n">
+        <v>18.65</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -5731,6 +6114,21 @@
       <c r="CL26" s="6" t="n">
         <v>13.71</v>
       </c>
+      <c r="CO26" s="6" t="n">
+        <v>6.53</v>
+      </c>
+      <c r="CP26" s="6" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="CQ26" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR26" s="6" t="n">
+        <v>2.87</v>
+      </c>
+      <c r="CS26" s="6" t="n">
+        <v>16.87</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5930,6 +6328,21 @@
       <c r="CL27" s="6" t="n">
         <v>14.43</v>
       </c>
+      <c r="CO27" s="5" t="n">
+        <v>19.58</v>
+      </c>
+      <c r="CP27" s="5" t="n">
+        <v>37.75</v>
+      </c>
+      <c r="CQ27" s="5" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="CR27" s="5" t="n">
+        <v>12.63</v>
+      </c>
+      <c r="CS27" s="5" t="n">
+        <v>12.43</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6129,6 +6542,21 @@
       <c r="CL28" s="6" t="n">
         <v>22.37</v>
       </c>
+      <c r="CO28" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="CP28" s="5" t="n">
+        <v>6.79</v>
+      </c>
+      <c r="CQ28" s="5" t="n">
+        <v>54.77</v>
+      </c>
+      <c r="CR28" s="6" t="n">
+        <v>37.89</v>
+      </c>
+      <c r="CS28" s="5" t="n">
+        <v>9.77</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6328,6 +6756,21 @@
       <c r="CL29" s="5" t="n">
         <v>1.73</v>
       </c>
+      <c r="CO29" s="6" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="CP29" s="6" t="n">
+        <v>29.29</v>
+      </c>
+      <c r="CQ29" s="6" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="CR29" s="6" t="n">
+        <v>17.22</v>
+      </c>
+      <c r="CS29" s="6" t="n">
+        <v>2.13</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -6527,6 +6970,21 @@
       <c r="CL30" t="n">
         <v>0</v>
       </c>
+      <c r="CO30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ30" s="6" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="CR30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -6534,7 +6992,7 @@
           <t>-----</t>
         </is>
       </c>
-      <c r="CL31" t="inlineStr"/>
+      <c r="CS31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -6734,6 +7192,21 @@
       <c r="CL32" t="n">
         <v>3.5</v>
       </c>
+      <c r="CO32" t="n">
+        <v>7</v>
+      </c>
+      <c r="CP32" t="n">
+        <v>2</v>
+      </c>
+      <c r="CQ32" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="CR32" t="n">
+        <v>9</v>
+      </c>
+      <c r="CS32" t="n">
+        <v>3.5</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -6933,6 +7406,21 @@
       <c r="CL33" s="6" t="n">
         <v>10.1</v>
       </c>
+      <c r="CO33" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="CP33" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="CQ33" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="CR33" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="CS33" s="6" t="n">
+        <v>10.1</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7132,6 +7620,21 @@
       <c r="CL34" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="CO34" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP34" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ34" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR34" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -7331,6 +7834,21 @@
       <c r="CL35" s="6" t="n">
         <v>7</v>
       </c>
+      <c r="CO35" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="CP35" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="CQ35" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR35" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS35" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -7530,6 +8048,21 @@
       <c r="CL36" t="n">
         <v>2</v>
       </c>
+      <c r="CO36" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP36" t="n">
+        <v>2</v>
+      </c>
+      <c r="CQ36" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="CR36" t="n">
+        <v>1</v>
+      </c>
+      <c r="CS36" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -7729,6 +8262,21 @@
       <c r="CL37" t="n">
         <v>10.5</v>
       </c>
+      <c r="CO37" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="CP37" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="CQ37" t="n">
+        <v>5</v>
+      </c>
+      <c r="CR37" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="CS37" t="n">
+        <v>10.5</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -7928,6 +8476,21 @@
       <c r="CL38" t="n">
         <v>9.5</v>
       </c>
+      <c r="CO38" t="n">
+        <v>4</v>
+      </c>
+      <c r="CP38" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="CQ38" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR38" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="CS38" t="n">
+        <v>9.5</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -8127,6 +8690,21 @@
       <c r="CL39" t="n">
         <v>10</v>
       </c>
+      <c r="CO39" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="CP39" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="CQ39" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="CR39" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="CS39" s="5" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -8326,6 +8904,21 @@
       <c r="CL40" t="n">
         <v>15.5</v>
       </c>
+      <c r="CO40" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="CP40" s="5" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="CQ40" s="5" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="CR40" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="CS40" s="5" t="n">
+        <v>5.5</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -8525,6 +9118,21 @@
       <c r="CL41" s="5" t="n">
         <v>1.2</v>
       </c>
+      <c r="CO41" t="n">
+        <v>1</v>
+      </c>
+      <c r="CP41" t="n">
+        <v>58.2</v>
+      </c>
+      <c r="CQ41" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="CR41" t="n">
+        <v>15</v>
+      </c>
+      <c r="CS41" s="6" t="n">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -8724,6 +9332,21 @@
       <c r="CL42" t="n">
         <v>0</v>
       </c>
+      <c r="CO42" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP42" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ42" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="CR42" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS42" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -8731,7 +9354,7 @@
           <t>------------</t>
         </is>
       </c>
-      <c r="CL43" t="inlineStr"/>
+      <c r="CS43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -8931,6 +9554,21 @@
       <c r="CL44" t="n">
         <v>106</v>
       </c>
+      <c r="CO44" t="n">
+        <v>233</v>
+      </c>
+      <c r="CP44" t="n">
+        <v>906</v>
+      </c>
+      <c r="CQ44" t="n">
+        <v>3</v>
+      </c>
+      <c r="CR44" t="n">
+        <v>101</v>
+      </c>
+      <c r="CS44" t="n">
+        <v>106</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -9130,6 +9768,21 @@
       <c r="CL45" s="5" t="n">
         <v>106</v>
       </c>
+      <c r="CO45" t="n">
+        <v>233</v>
+      </c>
+      <c r="CP45" t="n">
+        <v>906</v>
+      </c>
+      <c r="CQ45" t="n">
+        <v>3</v>
+      </c>
+      <c r="CR45" t="n">
+        <v>101</v>
+      </c>
+      <c r="CS45" t="n">
+        <v>106</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -9329,6 +9982,21 @@
       <c r="CL46" s="5" t="n">
         <v>92</v>
       </c>
+      <c r="CO46" t="n">
+        <v>232</v>
+      </c>
+      <c r="CP46" t="n">
+        <v>823</v>
+      </c>
+      <c r="CQ46" t="n">
+        <v>3</v>
+      </c>
+      <c r="CR46" t="n">
+        <v>101</v>
+      </c>
+      <c r="CS46" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -9528,6 +10196,21 @@
       <c r="CL47" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="CO47" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP47" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ47" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR47" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -9727,6 +10410,21 @@
       <c r="CL48" s="6" t="n">
         <v>14</v>
       </c>
+      <c r="CO48" t="n">
+        <v>1</v>
+      </c>
+      <c r="CP48" t="n">
+        <v>83</v>
+      </c>
+      <c r="CQ48" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR48" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS48" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -9926,6 +10624,21 @@
       <c r="CL49" t="n">
         <v>13</v>
       </c>
+      <c r="CO49" t="n">
+        <v>14</v>
+      </c>
+      <c r="CP49" t="n">
+        <v>22</v>
+      </c>
+      <c r="CQ49" t="n">
+        <v>16</v>
+      </c>
+      <c r="CR49" t="n">
+        <v>21</v>
+      </c>
+      <c r="CS49" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -10125,6 +10838,21 @@
       <c r="CL50" t="n">
         <v>17</v>
       </c>
+      <c r="CO50" t="n">
+        <v>14</v>
+      </c>
+      <c r="CP50" t="n">
+        <v>26</v>
+      </c>
+      <c r="CQ50" t="n">
+        <v>15</v>
+      </c>
+      <c r="CR50" t="n">
+        <v>19</v>
+      </c>
+      <c r="CS50" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -10324,6 +11052,21 @@
       <c r="CL51" t="n">
         <v>-4</v>
       </c>
+      <c r="CO51" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP51" t="n">
+        <v>-4</v>
+      </c>
+      <c r="CQ51" t="n">
+        <v>1</v>
+      </c>
+      <c r="CR51" t="n">
+        <v>2</v>
+      </c>
+      <c r="CS51" t="n">
+        <v>-4</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -10523,6 +11266,21 @@
       <c r="CL52" t="n">
         <v>105</v>
       </c>
+      <c r="CO52" t="n">
+        <v>97</v>
+      </c>
+      <c r="CP52" t="n">
+        <v>200</v>
+      </c>
+      <c r="CQ52" t="n">
+        <v>126</v>
+      </c>
+      <c r="CR52" t="n">
+        <v>80</v>
+      </c>
+      <c r="CS52" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -10722,6 +11480,21 @@
       <c r="CL53" t="n">
         <v>84</v>
       </c>
+      <c r="CO53" t="n">
+        <v>96</v>
+      </c>
+      <c r="CP53" t="n">
+        <v>203</v>
+      </c>
+      <c r="CQ53" t="n">
+        <v>116</v>
+      </c>
+      <c r="CR53" t="n">
+        <v>67</v>
+      </c>
+      <c r="CS53" t="n">
+        <v>84</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -10921,6 +11694,21 @@
       <c r="CL54" t="n">
         <v>21</v>
       </c>
+      <c r="CO54" t="n">
+        <v>1</v>
+      </c>
+      <c r="CP54" t="n">
+        <v>-3</v>
+      </c>
+      <c r="CQ54" t="n">
+        <v>10</v>
+      </c>
+      <c r="CR54" t="n">
+        <v>13</v>
+      </c>
+      <c r="CS54" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -11120,6 +11908,21 @@
       <c r="CL55" t="n">
         <v>179</v>
       </c>
+      <c r="CO55" t="n">
+        <v>108</v>
+      </c>
+      <c r="CP55" t="n">
+        <v>126</v>
+      </c>
+      <c r="CQ55" t="n">
+        <v>12</v>
+      </c>
+      <c r="CR55" t="n">
+        <v>169</v>
+      </c>
+      <c r="CS55" t="n">
+        <v>179</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -11319,6 +12122,21 @@
       <c r="CL56" t="n">
         <v>160</v>
       </c>
+      <c r="CO56" t="n">
+        <v>100</v>
+      </c>
+      <c r="CP56" t="n">
+        <v>123</v>
+      </c>
+      <c r="CQ56" t="n">
+        <v>12</v>
+      </c>
+      <c r="CR56" t="n">
+        <v>164</v>
+      </c>
+      <c r="CS56" t="n">
+        <v>160</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -11518,6 +12336,21 @@
       <c r="CL57" t="n">
         <v>19</v>
       </c>
+      <c r="CO57" t="n">
+        <v>8</v>
+      </c>
+      <c r="CP57" t="n">
+        <v>3</v>
+      </c>
+      <c r="CQ57" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR57" t="n">
+        <v>5</v>
+      </c>
+      <c r="CS57" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -11717,6 +12550,21 @@
       <c r="CL58" t="n">
         <v>178</v>
       </c>
+      <c r="CO58" s="5" t="n">
+        <v>182</v>
+      </c>
+      <c r="CP58" s="6" t="n">
+        <v>214</v>
+      </c>
+      <c r="CQ58" s="5" t="n">
+        <v>63</v>
+      </c>
+      <c r="CR58" s="5" t="n">
+        <v>177</v>
+      </c>
+      <c r="CS58" s="6" t="n">
+        <v>172</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -11916,6 +12764,21 @@
       <c r="CL59" t="n">
         <v>158</v>
       </c>
+      <c r="CO59" t="n">
+        <v>158</v>
+      </c>
+      <c r="CP59" t="n">
+        <v>64</v>
+      </c>
+      <c r="CQ59" t="n">
+        <v>67</v>
+      </c>
+      <c r="CR59" t="n">
+        <v>155</v>
+      </c>
+      <c r="CS59" t="n">
+        <v>158</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -12115,6 +12978,21 @@
       <c r="CL60" t="n">
         <v>172</v>
       </c>
+      <c r="CO60" t="n">
+        <v>182</v>
+      </c>
+      <c r="CP60" t="n">
+        <v>68</v>
+      </c>
+      <c r="CQ60" t="n">
+        <v>67</v>
+      </c>
+      <c r="CR60" t="n">
+        <v>156</v>
+      </c>
+      <c r="CS60" t="n">
+        <v>172</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -12314,6 +13192,21 @@
       <c r="CL61" t="n">
         <v>20</v>
       </c>
+      <c r="CO61" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="CP61" s="5" t="n">
+        <v>150</v>
+      </c>
+      <c r="CQ61" s="5" t="n">
+        <v>-4</v>
+      </c>
+      <c r="CR61" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="CS61" s="5" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -12513,6 +13406,21 @@
       <c r="CL62" t="n">
         <v>74</v>
       </c>
+      <c r="CO62" s="6" t="n">
+        <v>64</v>
+      </c>
+      <c r="CP62" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="CQ62" s="5" t="n">
+        <v>164</v>
+      </c>
+      <c r="CR62" s="5" t="n">
+        <v>53</v>
+      </c>
+      <c r="CS62" s="6" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -12712,6 +13620,21 @@
       <c r="CL63" t="n">
         <v>43</v>
       </c>
+      <c r="CO63" t="n">
+        <v>102</v>
+      </c>
+      <c r="CP63" t="n">
+        <v>69</v>
+      </c>
+      <c r="CQ63" t="n">
+        <v>133</v>
+      </c>
+      <c r="CR63" t="n">
+        <v>119</v>
+      </c>
+      <c r="CS63" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -12911,6 +13834,21 @@
       <c r="CL64" t="n">
         <v>31</v>
       </c>
+      <c r="CO64" s="6" t="n">
+        <v>-38</v>
+      </c>
+      <c r="CP64" s="5" t="n">
+        <v>-27</v>
+      </c>
+      <c r="CQ64" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="CR64" s="5" t="n">
+        <v>-66</v>
+      </c>
+      <c r="CS64" s="5" t="n">
+        <v>-11</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -13110,6 +14048,21 @@
       <c r="CL65" t="n">
         <v>1003</v>
       </c>
+      <c r="CO65" t="n">
+        <v>731</v>
+      </c>
+      <c r="CP65" t="n">
+        <v>2651</v>
+      </c>
+      <c r="CQ65" t="n">
+        <v>434</v>
+      </c>
+      <c r="CR65" t="n">
+        <v>1874</v>
+      </c>
+      <c r="CS65" t="n">
+        <v>1003</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -13309,6 +14262,21 @@
       <c r="CL66" s="5" t="n">
         <v>997</v>
       </c>
+      <c r="CO66" t="n">
+        <v>726</v>
+      </c>
+      <c r="CP66" t="n">
+        <v>2360</v>
+      </c>
+      <c r="CQ66" t="n">
+        <v>438</v>
+      </c>
+      <c r="CR66" t="n">
+        <v>1799</v>
+      </c>
+      <c r="CS66" t="n">
+        <v>997</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -13508,6 +14476,21 @@
       <c r="CL67" s="5" t="n">
         <v>6</v>
       </c>
+      <c r="CO67" t="n">
+        <v>5</v>
+      </c>
+      <c r="CP67" t="n">
+        <v>291</v>
+      </c>
+      <c r="CQ67" t="n">
+        <v>-4</v>
+      </c>
+      <c r="CR67" t="n">
+        <v>75</v>
+      </c>
+      <c r="CS67" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -13707,6 +14690,21 @@
       <c r="CL68" t="n">
         <v>566</v>
       </c>
+      <c r="CO68" t="n">
+        <v>611</v>
+      </c>
+      <c r="CP68" t="n">
+        <v>519</v>
+      </c>
+      <c r="CQ68" t="n">
+        <v>831</v>
+      </c>
+      <c r="CR68" t="n">
+        <v>807</v>
+      </c>
+      <c r="CS68" t="n">
+        <v>566</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -13906,6 +14904,21 @@
       <c r="CL69" t="n">
         <v>566</v>
       </c>
+      <c r="CO69" t="n">
+        <v>611</v>
+      </c>
+      <c r="CP69" t="n">
+        <v>519</v>
+      </c>
+      <c r="CQ69" t="n">
+        <v>830</v>
+      </c>
+      <c r="CR69" t="n">
+        <v>807</v>
+      </c>
+      <c r="CS69" t="n">
+        <v>566</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -14105,6 +15118,21 @@
       <c r="CL70" t="n">
         <v>0</v>
       </c>
+      <c r="CO70" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP70" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ70" t="n">
+        <v>1</v>
+      </c>
+      <c r="CR70" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS70" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -14304,6 +15332,21 @@
       <c r="CL71" t="n">
         <v>1</v>
       </c>
+      <c r="CO71" t="n">
+        <v>1</v>
+      </c>
+      <c r="CP71" t="n">
+        <v>1</v>
+      </c>
+      <c r="CQ71" t="n">
+        <v>1</v>
+      </c>
+      <c r="CR71" t="n">
+        <v>1</v>
+      </c>
+      <c r="CS71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -14503,6 +15546,21 @@
       <c r="CL72" t="n">
         <v>1</v>
       </c>
+      <c r="CO72" t="n">
+        <v>1</v>
+      </c>
+      <c r="CP72" t="n">
+        <v>1</v>
+      </c>
+      <c r="CQ72" t="n">
+        <v>1</v>
+      </c>
+      <c r="CR72" t="n">
+        <v>1</v>
+      </c>
+      <c r="CS72" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -14702,6 +15760,21 @@
       <c r="CL73" t="n">
         <v>0</v>
       </c>
+      <c r="CO73" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP73" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ73" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR73" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -14901,6 +15974,21 @@
       <c r="CL74" t="n">
         <v>158</v>
       </c>
+      <c r="CO74" t="n">
+        <v>158</v>
+      </c>
+      <c r="CP74" t="n">
+        <v>64</v>
+      </c>
+      <c r="CQ74" t="n">
+        <v>67</v>
+      </c>
+      <c r="CR74" t="n">
+        <v>155</v>
+      </c>
+      <c r="CS74" t="n">
+        <v>158</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -15100,6 +16188,21 @@
       <c r="CL75" t="n">
         <v>158</v>
       </c>
+      <c r="CO75" t="n">
+        <v>158</v>
+      </c>
+      <c r="CP75" t="n">
+        <v>64</v>
+      </c>
+      <c r="CQ75" t="n">
+        <v>67</v>
+      </c>
+      <c r="CR75" t="n">
+        <v>155</v>
+      </c>
+      <c r="CS75" t="n">
+        <v>158</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -15299,6 +16402,21 @@
       <c r="CL76" t="n">
         <v>0</v>
       </c>
+      <c r="CO76" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP76" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ76" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR76" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS76" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -15498,6 +16616,21 @@
       <c r="CL77" t="n">
         <v>0</v>
       </c>
+      <c r="CO77" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP77" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ77" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR77" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -15697,6 +16830,21 @@
       <c r="CL78" t="n">
         <v>0</v>
       </c>
+      <c r="CO78" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP78" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ78" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR78" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS78" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -15896,6 +17044,21 @@
       <c r="CL79" t="n">
         <v>0</v>
       </c>
+      <c r="CO79" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP79" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ79" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR79" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS79" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -16095,6 +17258,21 @@
       <c r="CL80" t="n">
         <v>43</v>
       </c>
+      <c r="CO80" t="n">
+        <v>102</v>
+      </c>
+      <c r="CP80" t="n">
+        <v>69</v>
+      </c>
+      <c r="CQ80" t="n">
+        <v>133</v>
+      </c>
+      <c r="CR80" t="n">
+        <v>119</v>
+      </c>
+      <c r="CS80" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -16294,6 +17472,21 @@
       <c r="CL81" t="n">
         <v>43</v>
       </c>
+      <c r="CO81" t="n">
+        <v>102</v>
+      </c>
+      <c r="CP81" t="n">
+        <v>69</v>
+      </c>
+      <c r="CQ81" t="n">
+        <v>133</v>
+      </c>
+      <c r="CR81" t="n">
+        <v>119</v>
+      </c>
+      <c r="CS81" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -16493,6 +17686,21 @@
       <c r="CL82" t="n">
         <v>0</v>
       </c>
+      <c r="CO82" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP82" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ82" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR82" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS82" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -16692,6 +17900,21 @@
       <c r="CL83" t="n">
         <v>244</v>
       </c>
+      <c r="CO83" t="n">
+        <v>28</v>
+      </c>
+      <c r="CP83" t="n">
+        <v>114</v>
+      </c>
+      <c r="CQ83" t="n">
+        <v>24</v>
+      </c>
+      <c r="CR83" t="n">
+        <v>265</v>
+      </c>
+      <c r="CS83" t="n">
+        <v>244</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -16891,6 +18114,21 @@
       <c r="CL84" t="n">
         <v>244</v>
       </c>
+      <c r="CO84" t="n">
+        <v>28</v>
+      </c>
+      <c r="CP84" t="n">
+        <v>114</v>
+      </c>
+      <c r="CQ84" t="n">
+        <v>24</v>
+      </c>
+      <c r="CR84" t="n">
+        <v>265</v>
+      </c>
+      <c r="CS84" t="n">
+        <v>244</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -17090,6 +18328,21 @@
       <c r="CL85" t="n">
         <v>0</v>
       </c>
+      <c r="CO85" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP85" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ85" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR85" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -17289,6 +18542,21 @@
       <c r="CL86" t="n">
         <v>1</v>
       </c>
+      <c r="CO86" t="n">
+        <v>9</v>
+      </c>
+      <c r="CP86" t="n">
+        <v>2</v>
+      </c>
+      <c r="CQ86" t="n">
+        <v>38</v>
+      </c>
+      <c r="CR86" t="n">
+        <v>105</v>
+      </c>
+      <c r="CS86" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -17488,6 +18756,21 @@
       <c r="CL87" t="n">
         <v>1</v>
       </c>
+      <c r="CO87" t="n">
+        <v>9</v>
+      </c>
+      <c r="CP87" t="n">
+        <v>2</v>
+      </c>
+      <c r="CQ87" t="n">
+        <v>38</v>
+      </c>
+      <c r="CR87" t="n">
+        <v>105</v>
+      </c>
+      <c r="CS87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -17687,6 +18970,21 @@
       <c r="CL88" t="n">
         <v>0</v>
       </c>
+      <c r="CO88" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP88" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ88" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR88" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -17886,6 +19184,21 @@
       <c r="CL89" t="n">
         <v>0</v>
       </c>
+      <c r="CO89" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP89" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ89" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR89" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS89" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -18085,6 +19398,21 @@
       <c r="CL90" t="n">
         <v>0</v>
       </c>
+      <c r="CO90" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP90" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ90" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR90" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS90" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -18284,6 +19612,21 @@
       <c r="CL91" t="n">
         <v>0</v>
       </c>
+      <c r="CO91" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP91" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ91" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR91" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS91" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -18483,6 +19826,21 @@
       <c r="CL92" t="n">
         <v>4</v>
       </c>
+      <c r="CO92" t="n">
+        <v>68</v>
+      </c>
+      <c r="CP92" t="n">
+        <v>165</v>
+      </c>
+      <c r="CQ92" t="n">
+        <v>459</v>
+      </c>
+      <c r="CR92" t="n">
+        <v>38</v>
+      </c>
+      <c r="CS92" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -18682,6 +20040,21 @@
       <c r="CL93" t="n">
         <v>4</v>
       </c>
+      <c r="CO93" t="n">
+        <v>68</v>
+      </c>
+      <c r="CP93" t="n">
+        <v>165</v>
+      </c>
+      <c r="CQ93" t="n">
+        <v>459</v>
+      </c>
+      <c r="CR93" t="n">
+        <v>38</v>
+      </c>
+      <c r="CS93" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -18881,6 +20254,21 @@
       <c r="CL94" t="n">
         <v>0</v>
       </c>
+      <c r="CO94" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP94" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ94" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR94" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS94" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -19080,6 +20468,21 @@
       <c r="CL95" t="n">
         <v>40</v>
       </c>
+      <c r="CO95" t="n">
+        <v>65</v>
+      </c>
+      <c r="CP95" t="n">
+        <v>36</v>
+      </c>
+      <c r="CQ95" t="n">
+        <v>102</v>
+      </c>
+      <c r="CR95" t="n">
+        <v>83</v>
+      </c>
+      <c r="CS95" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -19279,6 +20682,21 @@
       <c r="CL96" t="n">
         <v>40</v>
       </c>
+      <c r="CO96" t="n">
+        <v>65</v>
+      </c>
+      <c r="CP96" t="n">
+        <v>36</v>
+      </c>
+      <c r="CQ96" t="n">
+        <v>102</v>
+      </c>
+      <c r="CR96" t="n">
+        <v>83</v>
+      </c>
+      <c r="CS96" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -19478,6 +20896,21 @@
       <c r="CL97" t="n">
         <v>0</v>
       </c>
+      <c r="CO97" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP97" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ97" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR97" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -19677,6 +21110,21 @@
       <c r="CL98" t="n">
         <v>0</v>
       </c>
+      <c r="CO98" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP98" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ98" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR98" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS98" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -19876,6 +21324,21 @@
       <c r="CL99" t="n">
         <v>0</v>
       </c>
+      <c r="CO99" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP99" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ99" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR99" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS99" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -20075,6 +21538,21 @@
       <c r="CL100" t="n">
         <v>0</v>
       </c>
+      <c r="CO100" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP100" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ100" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR100" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -20274,6 +21752,21 @@
       <c r="CL101" t="n">
         <v>0</v>
       </c>
+      <c r="CO101" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP101" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ101" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR101" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS101" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -20473,6 +21966,21 @@
       <c r="CL102" t="n">
         <v>0</v>
       </c>
+      <c r="CO102" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP102" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ102" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR102" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS102" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -20672,6 +22180,21 @@
       <c r="CL103" t="n">
         <v>0</v>
       </c>
+      <c r="CO103" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP103" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ103" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR103" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS103" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -20871,6 +22394,21 @@
       <c r="CL104" t="n">
         <v>0</v>
       </c>
+      <c r="CO104" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP104" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ104" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR104" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS104" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -21070,6 +22608,21 @@
       <c r="CL105" t="n">
         <v>0</v>
       </c>
+      <c r="CO105" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP105" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ105" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR105" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS105" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -21269,6 +22822,21 @@
       <c r="CL106" t="n">
         <v>0</v>
       </c>
+      <c r="CO106" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP106" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ106" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR106" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS106" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -21468,6 +23036,21 @@
       <c r="CL107" t="n">
         <v>0</v>
       </c>
+      <c r="CO107" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP107" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ107" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR107" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS107" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -21667,6 +23250,21 @@
       <c r="CL108" t="n">
         <v>0</v>
       </c>
+      <c r="CO108" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP108" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ108" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR108" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS108" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -21866,6 +23464,21 @@
       <c r="CL109" t="n">
         <v>0</v>
       </c>
+      <c r="CO109" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP109" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ109" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR109" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS109" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -22065,6 +23678,21 @@
       <c r="CL110" t="n">
         <v>0</v>
       </c>
+      <c r="CO110" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP110" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ110" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR110" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS110" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -22264,6 +23892,21 @@
       <c r="CL111" t="n">
         <v>0</v>
       </c>
+      <c r="CO111" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP111" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ111" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR111" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS111" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -22463,6 +24106,21 @@
       <c r="CL112" t="n">
         <v>0</v>
       </c>
+      <c r="CO112" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP112" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ112" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR112" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS112" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -22662,6 +24320,21 @@
       <c r="CL113" t="n">
         <v>0</v>
       </c>
+      <c r="CO113" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP113" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ113" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR113" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS113" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -22861,6 +24534,21 @@
       <c r="CL114" t="n">
         <v>0</v>
       </c>
+      <c r="CO114" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP114" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ114" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR114" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS114" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -23060,6 +24748,21 @@
       <c r="CL115" t="n">
         <v>0</v>
       </c>
+      <c r="CO115" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP115" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ115" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR115" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS115" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -23259,6 +24962,21 @@
       <c r="CL116" t="n">
         <v>0</v>
       </c>
+      <c r="CO116" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP116" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ116" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR116" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS116" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -23458,6 +25176,21 @@
       <c r="CL117" t="n">
         <v>0</v>
       </c>
+      <c r="CO117" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP117" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ117" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR117" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS117" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -23657,6 +25390,21 @@
       <c r="CL118" t="n">
         <v>0</v>
       </c>
+      <c r="CO118" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP118" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ118" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR118" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS118" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -23856,6 +25604,21 @@
       <c r="CL119" t="n">
         <v>0</v>
       </c>
+      <c r="CO119" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP119" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ119" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR119" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS119" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -24055,6 +25818,21 @@
       <c r="CL120" t="n">
         <v>0</v>
       </c>
+      <c r="CO120" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP120" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ120" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR120" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS120" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -24254,13 +26032,28 @@
       <c r="CL121" t="n">
         <v>0</v>
       </c>
+      <c r="CO121" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP121" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ121" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR121" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS121" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="BT1:BY1"/>
+    <mergeCell ref="AR1:AW1"/>
+    <mergeCell ref="P1:U1"/>
     <mergeCell ref="AD1:AI1"/>
-    <mergeCell ref="P1:U1"/>
-    <mergeCell ref="AR1:AW1"/>
     <mergeCell ref="CA1:CF1"/>
     <mergeCell ref="BM1:BR1"/>
     <mergeCell ref="W1:AB1"/>
@@ -24270,6 +26063,7 @@
     <mergeCell ref="B1:G1"/>
     <mergeCell ref="I1:N1"/>
     <mergeCell ref="BF1:BK1"/>
+    <mergeCell ref="CO1:CT1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
adding formatting and fixing warnings and errors
</commit_message>
<xml_diff>
--- a/tests/regression_test/results/master_results.xlsx
+++ b/tests/regression_test/results/master_results.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CT121"/>
+  <dimension ref="A1:DA121"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30.33203125" customWidth="1" style="4" min="1" max="1"/>
@@ -522,6 +522,11 @@
           <t>img_fix</t>
         </is>
       </c>
+      <c r="CV1" s="3" t="inlineStr">
+        <is>
+          <t>bold-italic-formatting</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -949,6 +954,36 @@
           <t>avg.</t>
         </is>
       </c>
+      <c r="CV2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="CW2" t="inlineStr">
+        <is>
+          <t>algorithms</t>
+        </is>
+      </c>
+      <c r="CX2" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="CY2" t="inlineStr">
+        <is>
+          <t>cybersec</t>
+        </is>
+      </c>
+      <c r="CZ2" t="inlineStr">
+        <is>
+          <t>data-science</t>
+        </is>
+      </c>
+      <c r="DA2" t="inlineStr">
+        <is>
+          <t>avg.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1301,6 +1336,31 @@
           <t>data-science</t>
         </is>
       </c>
+      <c r="CV3" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="CW3" t="inlineStr">
+        <is>
+          <t>algorithms</t>
+        </is>
+      </c>
+      <c r="CX3" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="CY3" t="inlineStr">
+        <is>
+          <t>cybersec</t>
+        </is>
+      </c>
+      <c r="CZ3" t="inlineStr">
+        <is>
+          <t>data-science</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1653,6 +1713,31 @@
           <t>multi-metric</t>
         </is>
       </c>
+      <c r="CV4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="CW4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="CX4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="CY4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="CZ4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2005,6 +2090,31 @@
           <t>2025-11-30T20:18:34.787168</t>
         </is>
       </c>
+      <c r="CV5" t="inlineStr">
+        <is>
+          <t>2025-12-01T14:00:50.365126</t>
+        </is>
+      </c>
+      <c r="CW5" t="inlineStr">
+        <is>
+          <t>2025-12-01T14:00:50.703490</t>
+        </is>
+      </c>
+      <c r="CX5" t="inlineStr">
+        <is>
+          <t>2025-12-01T14:00:50.587746</t>
+        </is>
+      </c>
+      <c r="CY5" t="inlineStr">
+        <is>
+          <t>2025-12-01T14:00:50.916711</t>
+        </is>
+      </c>
+      <c r="CZ5" t="inlineStr">
+        <is>
+          <t>2025-12-01T14:00:51.042050</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2261,6 +2371,24 @@
       <c r="CT6" s="5" t="n">
         <v>-86.34</v>
       </c>
+      <c r="CV6" s="5" t="n">
+        <v>-46.2</v>
+      </c>
+      <c r="CW6" s="5" t="n">
+        <v>-194.3</v>
+      </c>
+      <c r="CX6" s="5" t="n">
+        <v>-27.1</v>
+      </c>
+      <c r="CY6" s="5" t="n">
+        <v>-80.59999999999999</v>
+      </c>
+      <c r="CZ6" s="5" t="n">
+        <v>-52.5</v>
+      </c>
+      <c r="DA6" s="5" t="n">
+        <v>-80.14</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2475,6 +2603,21 @@
       <c r="CS7" t="n">
         <v>100</v>
       </c>
+      <c r="CV7" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="CW7" s="5" t="n">
+        <v>65.38</v>
+      </c>
+      <c r="CX7" t="n">
+        <v>100</v>
+      </c>
+      <c r="CY7" t="n">
+        <v>100</v>
+      </c>
+      <c r="CZ7" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2689,6 +2832,21 @@
       <c r="CS8" t="n">
         <v>7</v>
       </c>
+      <c r="CV8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW8" s="5" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="CX8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="CY8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="CZ8" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2903,6 +3061,21 @@
       <c r="CS9" t="n">
         <v>101</v>
       </c>
+      <c r="CV9" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="CW9" s="5" t="n">
+        <v>9.18</v>
+      </c>
+      <c r="CX9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="CY9" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="CZ9" s="5" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3117,6 +3290,21 @@
       <c r="CS10" t="n">
         <v>100</v>
       </c>
+      <c r="CV10" t="n">
+        <v>100</v>
+      </c>
+      <c r="CW10" t="n">
+        <v>100</v>
+      </c>
+      <c r="CX10" t="n">
+        <v>100</v>
+      </c>
+      <c r="CY10" t="n">
+        <v>100</v>
+      </c>
+      <c r="CZ10" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3331,6 +3519,21 @@
       <c r="CS11" t="n">
         <v>86.79000000000001</v>
       </c>
+      <c r="CV11" t="n">
+        <v>99.56999999999999</v>
+      </c>
+      <c r="CW11" t="n">
+        <v>90.84</v>
+      </c>
+      <c r="CX11" t="n">
+        <v>100</v>
+      </c>
+      <c r="CY11" s="6" t="n">
+        <v>99.01000000000001</v>
+      </c>
+      <c r="CZ11" t="n">
+        <v>86.79000000000001</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3545,6 +3748,21 @@
       <c r="CS12" t="n">
         <v>130.77</v>
       </c>
+      <c r="CV12" t="n">
+        <v>100</v>
+      </c>
+      <c r="CW12" s="6" t="n">
+        <v>113.64</v>
+      </c>
+      <c r="CX12" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="CY12" t="n">
+        <v>90.48</v>
+      </c>
+      <c r="CZ12" t="n">
+        <v>130.77</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3759,6 +3977,21 @@
       <c r="CS13" t="n">
         <v>80</v>
       </c>
+      <c r="CV13" t="n">
+        <v>98.97</v>
+      </c>
+      <c r="CW13" s="6" t="n">
+        <v>99</v>
+      </c>
+      <c r="CX13" t="n">
+        <v>92.06</v>
+      </c>
+      <c r="CY13" s="6" t="n">
+        <v>81.25</v>
+      </c>
+      <c r="CZ13" s="6" t="n">
+        <v>72.38</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3973,6 +4206,21 @@
       <c r="CS14" t="n">
         <v>89.39</v>
       </c>
+      <c r="CV14" t="n">
+        <v>92.59</v>
+      </c>
+      <c r="CW14" s="6" t="n">
+        <v>96.03</v>
+      </c>
+      <c r="CX14" t="n">
+        <v>100</v>
+      </c>
+      <c r="CY14" s="6" t="n">
+        <v>88.17</v>
+      </c>
+      <c r="CZ14" s="6" t="n">
+        <v>83.23999999999999</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4187,6 +4435,21 @@
       <c r="CS15" s="5" t="n">
         <v>91.86</v>
       </c>
+      <c r="CV15" s="6" t="n">
+        <v>77.47</v>
+      </c>
+      <c r="CW15" t="n">
+        <v>29.91</v>
+      </c>
+      <c r="CX15" t="n">
+        <v>106.35</v>
+      </c>
+      <c r="CY15" s="6" t="n">
+        <v>85.88</v>
+      </c>
+      <c r="CZ15" t="n">
+        <v>91.86</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4401,6 +4664,21 @@
       <c r="CS16" s="5" t="n">
         <v>134.38</v>
       </c>
+      <c r="CV16" t="n">
+        <v>159.38</v>
+      </c>
+      <c r="CW16" t="n">
+        <v>164.29</v>
+      </c>
+      <c r="CX16" t="n">
+        <v>81.09999999999999</v>
+      </c>
+      <c r="CY16" t="n">
+        <v>224.53</v>
+      </c>
+      <c r="CZ16" t="n">
+        <v>134.38</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4615,6 +4893,21 @@
       <c r="CS17" t="n">
         <v>99.40000000000001</v>
       </c>
+      <c r="CV17" t="n">
+        <v>99.31999999999999</v>
+      </c>
+      <c r="CW17" t="n">
+        <v>89.02</v>
+      </c>
+      <c r="CX17" t="n">
+        <v>100.92</v>
+      </c>
+      <c r="CY17" t="n">
+        <v>96</v>
+      </c>
+      <c r="CZ17" t="n">
+        <v>99.40000000000001</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4622,7 +4915,7 @@
           <t>------------</t>
         </is>
       </c>
-      <c r="CS18" t="inlineStr"/>
+      <c r="CZ18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4630,7 +4923,7 @@
           <t>Score Deductions:</t>
         </is>
       </c>
-      <c r="CS19" t="inlineStr"/>
+      <c r="CZ19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4845,6 +5138,21 @@
       <c r="CS20" s="6" t="n">
         <v>6.22</v>
       </c>
+      <c r="CV20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW20" s="5" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="CX20" s="5" t="n">
+        <v>7.38</v>
+      </c>
+      <c r="CY20" s="5" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="CZ20" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5059,6 +5367,21 @@
       <c r="CS21" s="6" t="n">
         <v>17.94</v>
       </c>
+      <c r="CV21" s="5" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="CW21" s="5" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="CX21" s="6" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="CY21" s="5" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="CZ21" s="5" t="n">
+        <v>0.57</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5273,6 +5596,21 @@
       <c r="CS22" t="n">
         <v>0</v>
       </c>
+      <c r="CV22" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW22" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX22" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY22" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5487,6 +5825,21 @@
       <c r="CS23" s="6" t="n">
         <v>12.43</v>
       </c>
+      <c r="CV23" s="6" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="CW23" s="6" t="n">
+        <v>21.36</v>
+      </c>
+      <c r="CX23" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY23" s="6" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="CZ23" s="6" t="n">
+        <v>13.33</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5701,6 +6054,21 @@
       <c r="CS24" s="6" t="n">
         <v>3.55</v>
       </c>
+      <c r="CV24" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW24" s="5" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="CX24" s="6" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="CY24" s="6" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="CZ24" s="6" t="n">
+        <v>3.81</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5915,6 +6283,21 @@
       <c r="CS25" s="6" t="n">
         <v>18.65</v>
       </c>
+      <c r="CV25" s="6" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="CW25" s="5" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="CX25" s="6" t="n">
+        <v>18.45</v>
+      </c>
+      <c r="CY25" s="6" t="n">
+        <v>9.31</v>
+      </c>
+      <c r="CZ25" s="6" t="n">
+        <v>27.62</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6129,6 +6512,21 @@
       <c r="CS26" s="6" t="n">
         <v>16.87</v>
       </c>
+      <c r="CV26" s="6" t="n">
+        <v>8.66</v>
+      </c>
+      <c r="CW26" s="6" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="CX26" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY26" s="6" t="n">
+        <v>12.41</v>
+      </c>
+      <c r="CZ26" s="6" t="n">
+        <v>28.57</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6343,6 +6741,21 @@
       <c r="CS27" s="5" t="n">
         <v>12.43</v>
       </c>
+      <c r="CV27" s="6" t="n">
+        <v>44.37</v>
+      </c>
+      <c r="CW27" s="6" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="CX27" s="6" t="n">
+        <v>7.38</v>
+      </c>
+      <c r="CY27" s="6" t="n">
+        <v>15.51</v>
+      </c>
+      <c r="CZ27" s="6" t="n">
+        <v>13.33</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6557,6 +6970,21 @@
       <c r="CS28" s="5" t="n">
         <v>9.77</v>
       </c>
+      <c r="CV28" s="6" t="n">
+        <v>41.13</v>
+      </c>
+      <c r="CW28" s="6" t="n">
+        <v>6.95</v>
+      </c>
+      <c r="CX28" s="6" t="n">
+        <v>57.2</v>
+      </c>
+      <c r="CY28" s="6" t="n">
+        <v>40.94</v>
+      </c>
+      <c r="CZ28" s="6" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6771,6 +7199,21 @@
       <c r="CS29" s="6" t="n">
         <v>2.13</v>
       </c>
+      <c r="CV29" s="6" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="CW29" s="6" t="n">
+        <v>29.95</v>
+      </c>
+      <c r="CX29" s="6" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="CY29" s="6" t="n">
+        <v>18.61</v>
+      </c>
+      <c r="CZ29" s="6" t="n">
+        <v>2.29</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -6985,6 +7428,21 @@
       <c r="CS30" t="n">
         <v>0</v>
       </c>
+      <c r="CV30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX30" s="6" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="CY30" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -6992,7 +7450,7 @@
           <t>-----</t>
         </is>
       </c>
-      <c r="CS31" t="inlineStr"/>
+      <c r="CZ31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7207,6 +7665,21 @@
       <c r="CS32" t="n">
         <v>3.5</v>
       </c>
+      <c r="CV32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW32" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="CX32" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="CY32" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="CZ32" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7421,6 +7894,21 @@
       <c r="CS33" s="6" t="n">
         <v>10.1</v>
       </c>
+      <c r="CV33" s="5" t="n">
+        <v>0.7000000000000001</v>
+      </c>
+      <c r="CW33" s="5" t="n">
+        <v>0.6000000000000001</v>
+      </c>
+      <c r="CX33" s="6" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="CY33" s="5" t="n">
+        <v>0.6000000000000001</v>
+      </c>
+      <c r="CZ33" s="5" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7635,6 +8123,21 @@
       <c r="CS34" t="n">
         <v>0</v>
       </c>
+      <c r="CV34" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW34" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX34" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY34" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -7849,6 +8352,21 @@
       <c r="CS35" t="n">
         <v>7</v>
       </c>
+      <c r="CV35" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="CW35" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="CX35" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY35" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="CZ35" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -8063,6 +8581,21 @@
       <c r="CS36" t="n">
         <v>2</v>
       </c>
+      <c r="CV36" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW36" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="CX36" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="CY36" t="n">
+        <v>1</v>
+      </c>
+      <c r="CZ36" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -8277,6 +8810,21 @@
       <c r="CS37" t="n">
         <v>10.5</v>
       </c>
+      <c r="CV37" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="CW37" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="CX37" t="n">
+        <v>5</v>
+      </c>
+      <c r="CY37" s="6" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="CZ37" s="6" t="n">
+        <v>14.5</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -8491,6 +9039,21 @@
       <c r="CS38" t="n">
         <v>9.5</v>
       </c>
+      <c r="CV38" t="n">
+        <v>4</v>
+      </c>
+      <c r="CW38" s="6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="CX38" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY38" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="CZ38" s="6" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -8705,6 +9268,21 @@
       <c r="CS39" s="5" t="n">
         <v>7</v>
       </c>
+      <c r="CV39" s="6" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="CW39" t="n">
+        <v>75</v>
+      </c>
+      <c r="CX39" t="n">
+        <v>2</v>
+      </c>
+      <c r="CY39" s="6" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="CZ39" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -8919,6 +9497,21 @@
       <c r="CS40" s="5" t="n">
         <v>5.5</v>
       </c>
+      <c r="CV40" t="n">
+        <v>19</v>
+      </c>
+      <c r="CW40" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="CX40" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="CY40" t="n">
+        <v>33</v>
+      </c>
+      <c r="CZ40" t="n">
+        <v>5.5</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -9133,6 +9726,21 @@
       <c r="CS41" s="6" t="n">
         <v>1.2</v>
       </c>
+      <c r="CV41" t="n">
+        <v>1</v>
+      </c>
+      <c r="CW41" t="n">
+        <v>58.2</v>
+      </c>
+      <c r="CX41" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="CY41" t="n">
+        <v>15</v>
+      </c>
+      <c r="CZ41" s="6" t="n">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -9347,6 +9955,21 @@
       <c r="CS42" t="n">
         <v>0</v>
       </c>
+      <c r="CV42" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW42" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX42" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="CY42" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ42" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -9354,7 +9977,7 @@
           <t>------------</t>
         </is>
       </c>
-      <c r="CS43" t="inlineStr"/>
+      <c r="CZ43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -9569,6 +10192,21 @@
       <c r="CS44" t="n">
         <v>106</v>
       </c>
+      <c r="CV44" t="n">
+        <v>233</v>
+      </c>
+      <c r="CW44" t="n">
+        <v>906</v>
+      </c>
+      <c r="CX44" t="n">
+        <v>3</v>
+      </c>
+      <c r="CY44" t="n">
+        <v>101</v>
+      </c>
+      <c r="CZ44" t="n">
+        <v>106</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -9783,6 +10421,21 @@
       <c r="CS45" t="n">
         <v>106</v>
       </c>
+      <c r="CV45" t="n">
+        <v>233</v>
+      </c>
+      <c r="CW45" t="n">
+        <v>906</v>
+      </c>
+      <c r="CX45" t="n">
+        <v>3</v>
+      </c>
+      <c r="CY45" t="n">
+        <v>101</v>
+      </c>
+      <c r="CZ45" t="n">
+        <v>106</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -9997,6 +10650,21 @@
       <c r="CS46" t="n">
         <v>92</v>
       </c>
+      <c r="CV46" t="n">
+        <v>232</v>
+      </c>
+      <c r="CW46" t="n">
+        <v>823</v>
+      </c>
+      <c r="CX46" t="n">
+        <v>3</v>
+      </c>
+      <c r="CY46" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="CZ46" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -10211,6 +10879,21 @@
       <c r="CS47" t="n">
         <v>0</v>
       </c>
+      <c r="CV47" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW47" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX47" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY47" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -10425,6 +11108,21 @@
       <c r="CS48" t="n">
         <v>14</v>
       </c>
+      <c r="CV48" t="n">
+        <v>1</v>
+      </c>
+      <c r="CW48" t="n">
+        <v>83</v>
+      </c>
+      <c r="CX48" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY48" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CZ48" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -10639,6 +11337,21 @@
       <c r="CS49" t="n">
         <v>13</v>
       </c>
+      <c r="CV49" t="n">
+        <v>14</v>
+      </c>
+      <c r="CW49" t="n">
+        <v>22</v>
+      </c>
+      <c r="CX49" t="n">
+        <v>16</v>
+      </c>
+      <c r="CY49" t="n">
+        <v>21</v>
+      </c>
+      <c r="CZ49" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -10853,6 +11566,21 @@
       <c r="CS50" t="n">
         <v>17</v>
       </c>
+      <c r="CV50" t="n">
+        <v>14</v>
+      </c>
+      <c r="CW50" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="CX50" t="n">
+        <v>15</v>
+      </c>
+      <c r="CY50" t="n">
+        <v>19</v>
+      </c>
+      <c r="CZ50" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -11067,6 +11795,21 @@
       <c r="CS51" t="n">
         <v>-4</v>
       </c>
+      <c r="CV51" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW51" s="5" t="n">
+        <v>-3</v>
+      </c>
+      <c r="CX51" t="n">
+        <v>1</v>
+      </c>
+      <c r="CY51" t="n">
+        <v>2</v>
+      </c>
+      <c r="CZ51" t="n">
+        <v>-4</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -11281,6 +12024,21 @@
       <c r="CS52" t="n">
         <v>105</v>
       </c>
+      <c r="CV52" t="n">
+        <v>97</v>
+      </c>
+      <c r="CW52" t="n">
+        <v>200</v>
+      </c>
+      <c r="CX52" t="n">
+        <v>126</v>
+      </c>
+      <c r="CY52" t="n">
+        <v>80</v>
+      </c>
+      <c r="CZ52" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -11495,6 +12253,21 @@
       <c r="CS53" t="n">
         <v>84</v>
       </c>
+      <c r="CV53" t="n">
+        <v>96</v>
+      </c>
+      <c r="CW53" s="6" t="n">
+        <v>198</v>
+      </c>
+      <c r="CX53" t="n">
+        <v>116</v>
+      </c>
+      <c r="CY53" s="6" t="n">
+        <v>65</v>
+      </c>
+      <c r="CZ53" s="6" t="n">
+        <v>76</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -11709,6 +12482,21 @@
       <c r="CS54" t="n">
         <v>21</v>
       </c>
+      <c r="CV54" t="n">
+        <v>1</v>
+      </c>
+      <c r="CW54" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="CX54" t="n">
+        <v>10</v>
+      </c>
+      <c r="CY54" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="CZ54" s="6" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -11923,6 +12711,21 @@
       <c r="CS55" t="n">
         <v>179</v>
       </c>
+      <c r="CV55" t="n">
+        <v>108</v>
+      </c>
+      <c r="CW55" t="n">
+        <v>126</v>
+      </c>
+      <c r="CX55" t="n">
+        <v>12</v>
+      </c>
+      <c r="CY55" t="n">
+        <v>169</v>
+      </c>
+      <c r="CZ55" t="n">
+        <v>179</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -12137,6 +12940,21 @@
       <c r="CS56" t="n">
         <v>160</v>
       </c>
+      <c r="CV56" t="n">
+        <v>100</v>
+      </c>
+      <c r="CW56" s="6" t="n">
+        <v>121</v>
+      </c>
+      <c r="CX56" t="n">
+        <v>12</v>
+      </c>
+      <c r="CY56" s="6" t="n">
+        <v>149</v>
+      </c>
+      <c r="CZ56" s="6" t="n">
+        <v>149</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -12351,6 +13169,21 @@
       <c r="CS57" t="n">
         <v>19</v>
       </c>
+      <c r="CV57" t="n">
+        <v>8</v>
+      </c>
+      <c r="CW57" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="CX57" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY57" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="CZ57" s="6" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -12565,6 +13398,21 @@
       <c r="CS58" s="6" t="n">
         <v>172</v>
       </c>
+      <c r="CV58" t="n">
+        <v>182</v>
+      </c>
+      <c r="CW58" t="n">
+        <v>214</v>
+      </c>
+      <c r="CX58" t="n">
+        <v>63</v>
+      </c>
+      <c r="CY58" t="n">
+        <v>177</v>
+      </c>
+      <c r="CZ58" t="n">
+        <v>172</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -12779,6 +13627,21 @@
       <c r="CS59" t="n">
         <v>158</v>
       </c>
+      <c r="CV59" s="6" t="n">
+        <v>141</v>
+      </c>
+      <c r="CW59" t="n">
+        <v>64</v>
+      </c>
+      <c r="CX59" t="n">
+        <v>67</v>
+      </c>
+      <c r="CY59" s="6" t="n">
+        <v>152</v>
+      </c>
+      <c r="CZ59" t="n">
+        <v>158</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -12993,6 +13856,21 @@
       <c r="CS60" t="n">
         <v>172</v>
       </c>
+      <c r="CV60" t="n">
+        <v>182</v>
+      </c>
+      <c r="CW60" t="n">
+        <v>68</v>
+      </c>
+      <c r="CX60" t="n">
+        <v>67</v>
+      </c>
+      <c r="CY60" t="n">
+        <v>156</v>
+      </c>
+      <c r="CZ60" t="n">
+        <v>172</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -13207,6 +14085,21 @@
       <c r="CS61" s="5" t="n">
         <v>14</v>
       </c>
+      <c r="CV61" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="CW61" t="n">
+        <v>150</v>
+      </c>
+      <c r="CX61" t="n">
+        <v>-4</v>
+      </c>
+      <c r="CY61" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="CZ61" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -13421,6 +14314,21 @@
       <c r="CS62" s="6" t="n">
         <v>32</v>
       </c>
+      <c r="CV62" t="n">
+        <v>64</v>
+      </c>
+      <c r="CW62" t="n">
+        <v>42</v>
+      </c>
+      <c r="CX62" t="n">
+        <v>164</v>
+      </c>
+      <c r="CY62" t="n">
+        <v>53</v>
+      </c>
+      <c r="CZ62" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -13635,6 +14543,21 @@
       <c r="CS63" t="n">
         <v>43</v>
       </c>
+      <c r="CV63" t="n">
+        <v>102</v>
+      </c>
+      <c r="CW63" t="n">
+        <v>69</v>
+      </c>
+      <c r="CX63" t="n">
+        <v>133</v>
+      </c>
+      <c r="CY63" t="n">
+        <v>119</v>
+      </c>
+      <c r="CZ63" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -13849,6 +14772,21 @@
       <c r="CS64" s="5" t="n">
         <v>-11</v>
       </c>
+      <c r="CV64" t="n">
+        <v>-38</v>
+      </c>
+      <c r="CW64" t="n">
+        <v>-27</v>
+      </c>
+      <c r="CX64" t="n">
+        <v>31</v>
+      </c>
+      <c r="CY64" t="n">
+        <v>-66</v>
+      </c>
+      <c r="CZ64" t="n">
+        <v>-11</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -14063,6 +15001,21 @@
       <c r="CS65" t="n">
         <v>1003</v>
       </c>
+      <c r="CV65" t="n">
+        <v>731</v>
+      </c>
+      <c r="CW65" t="n">
+        <v>2651</v>
+      </c>
+      <c r="CX65" t="n">
+        <v>434</v>
+      </c>
+      <c r="CY65" t="n">
+        <v>1874</v>
+      </c>
+      <c r="CZ65" t="n">
+        <v>1003</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -14277,6 +15230,21 @@
       <c r="CS66" t="n">
         <v>997</v>
       </c>
+      <c r="CV66" t="n">
+        <v>726</v>
+      </c>
+      <c r="CW66" t="n">
+        <v>2360</v>
+      </c>
+      <c r="CX66" t="n">
+        <v>438</v>
+      </c>
+      <c r="CY66" t="n">
+        <v>1799</v>
+      </c>
+      <c r="CZ66" t="n">
+        <v>997</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -14491,6 +15459,21 @@
       <c r="CS67" t="n">
         <v>6</v>
       </c>
+      <c r="CV67" t="n">
+        <v>5</v>
+      </c>
+      <c r="CW67" t="n">
+        <v>291</v>
+      </c>
+      <c r="CX67" t="n">
+        <v>-4</v>
+      </c>
+      <c r="CY67" t="n">
+        <v>75</v>
+      </c>
+      <c r="CZ67" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -14705,6 +15688,21 @@
       <c r="CS68" t="n">
         <v>566</v>
       </c>
+      <c r="CV68" s="6" t="n">
+        <v>595</v>
+      </c>
+      <c r="CW68" s="5" t="n">
+        <v>520</v>
+      </c>
+      <c r="CX68" s="5" t="n">
+        <v>832</v>
+      </c>
+      <c r="CY68" s="6" t="n">
+        <v>805</v>
+      </c>
+      <c r="CZ68" s="5" t="n">
+        <v>567</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -14919,6 +15917,21 @@
       <c r="CS69" t="n">
         <v>566</v>
       </c>
+      <c r="CV69" s="6" t="n">
+        <v>595</v>
+      </c>
+      <c r="CW69" s="5" t="n">
+        <v>520</v>
+      </c>
+      <c r="CX69" s="5" t="n">
+        <v>831</v>
+      </c>
+      <c r="CY69" s="6" t="n">
+        <v>805</v>
+      </c>
+      <c r="CZ69" s="5" t="n">
+        <v>567</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -15133,6 +16146,21 @@
       <c r="CS70" t="n">
         <v>0</v>
       </c>
+      <c r="CV70" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW70" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX70" t="n">
+        <v>1</v>
+      </c>
+      <c r="CY70" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ70" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -15347,6 +16375,21 @@
       <c r="CS71" t="n">
         <v>1</v>
       </c>
+      <c r="CV71" t="n">
+        <v>1</v>
+      </c>
+      <c r="CW71" t="n">
+        <v>1</v>
+      </c>
+      <c r="CX71" t="n">
+        <v>1</v>
+      </c>
+      <c r="CY71" t="n">
+        <v>1</v>
+      </c>
+      <c r="CZ71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -15561,6 +16604,21 @@
       <c r="CS72" t="n">
         <v>1</v>
       </c>
+      <c r="CV72" t="n">
+        <v>1</v>
+      </c>
+      <c r="CW72" t="n">
+        <v>1</v>
+      </c>
+      <c r="CX72" t="n">
+        <v>1</v>
+      </c>
+      <c r="CY72" t="n">
+        <v>1</v>
+      </c>
+      <c r="CZ72" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -15775,6 +16833,21 @@
       <c r="CS73" t="n">
         <v>0</v>
       </c>
+      <c r="CV73" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW73" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX73" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY73" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -15989,6 +17062,21 @@
       <c r="CS74" t="n">
         <v>158</v>
       </c>
+      <c r="CV74" s="6" t="n">
+        <v>141</v>
+      </c>
+      <c r="CW74" t="n">
+        <v>64</v>
+      </c>
+      <c r="CX74" t="n">
+        <v>67</v>
+      </c>
+      <c r="CY74" s="6" t="n">
+        <v>152</v>
+      </c>
+      <c r="CZ74" t="n">
+        <v>158</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -16203,6 +17291,21 @@
       <c r="CS75" t="n">
         <v>158</v>
       </c>
+      <c r="CV75" s="6" t="n">
+        <v>141</v>
+      </c>
+      <c r="CW75" t="n">
+        <v>64</v>
+      </c>
+      <c r="CX75" t="n">
+        <v>67</v>
+      </c>
+      <c r="CY75" s="6" t="n">
+        <v>152</v>
+      </c>
+      <c r="CZ75" t="n">
+        <v>158</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -16417,6 +17520,21 @@
       <c r="CS76" t="n">
         <v>0</v>
       </c>
+      <c r="CV76" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW76" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX76" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY76" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ76" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -16631,6 +17749,21 @@
       <c r="CS77" t="n">
         <v>0</v>
       </c>
+      <c r="CV77" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW77" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX77" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY77" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -16845,6 +17978,21 @@
       <c r="CS78" t="n">
         <v>0</v>
       </c>
+      <c r="CV78" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW78" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX78" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY78" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ78" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -17059,6 +18207,21 @@
       <c r="CS79" t="n">
         <v>0</v>
       </c>
+      <c r="CV79" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW79" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX79" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY79" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ79" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -17273,6 +18436,21 @@
       <c r="CS80" t="n">
         <v>43</v>
       </c>
+      <c r="CV80" t="n">
+        <v>102</v>
+      </c>
+      <c r="CW80" t="n">
+        <v>69</v>
+      </c>
+      <c r="CX80" t="n">
+        <v>133</v>
+      </c>
+      <c r="CY80" t="n">
+        <v>119</v>
+      </c>
+      <c r="CZ80" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -17487,6 +18665,21 @@
       <c r="CS81" t="n">
         <v>43</v>
       </c>
+      <c r="CV81" t="n">
+        <v>102</v>
+      </c>
+      <c r="CW81" t="n">
+        <v>69</v>
+      </c>
+      <c r="CX81" t="n">
+        <v>133</v>
+      </c>
+      <c r="CY81" t="n">
+        <v>119</v>
+      </c>
+      <c r="CZ81" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -17701,6 +18894,21 @@
       <c r="CS82" t="n">
         <v>0</v>
       </c>
+      <c r="CV82" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW82" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX82" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY82" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ82" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -17915,6 +19123,21 @@
       <c r="CS83" t="n">
         <v>244</v>
       </c>
+      <c r="CV83" t="n">
+        <v>28</v>
+      </c>
+      <c r="CW83" t="n">
+        <v>114</v>
+      </c>
+      <c r="CX83" t="n">
+        <v>24</v>
+      </c>
+      <c r="CY83" t="n">
+        <v>265</v>
+      </c>
+      <c r="CZ83" t="n">
+        <v>244</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -18129,6 +19352,21 @@
       <c r="CS84" t="n">
         <v>244</v>
       </c>
+      <c r="CV84" t="n">
+        <v>28</v>
+      </c>
+      <c r="CW84" t="n">
+        <v>114</v>
+      </c>
+      <c r="CX84" t="n">
+        <v>24</v>
+      </c>
+      <c r="CY84" t="n">
+        <v>265</v>
+      </c>
+      <c r="CZ84" t="n">
+        <v>244</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -18343,6 +19581,21 @@
       <c r="CS85" t="n">
         <v>0</v>
       </c>
+      <c r="CV85" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW85" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX85" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY85" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -18557,6 +19810,21 @@
       <c r="CS86" t="n">
         <v>1</v>
       </c>
+      <c r="CV86" t="n">
+        <v>9</v>
+      </c>
+      <c r="CW86" t="n">
+        <v>2</v>
+      </c>
+      <c r="CX86" t="n">
+        <v>38</v>
+      </c>
+      <c r="CY86" t="n">
+        <v>105</v>
+      </c>
+      <c r="CZ86" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -18771,6 +20039,21 @@
       <c r="CS87" t="n">
         <v>1</v>
       </c>
+      <c r="CV87" t="n">
+        <v>9</v>
+      </c>
+      <c r="CW87" t="n">
+        <v>2</v>
+      </c>
+      <c r="CX87" t="n">
+        <v>38</v>
+      </c>
+      <c r="CY87" t="n">
+        <v>105</v>
+      </c>
+      <c r="CZ87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -18985,6 +20268,21 @@
       <c r="CS88" t="n">
         <v>0</v>
       </c>
+      <c r="CV88" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW88" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX88" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY88" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -19199,6 +20497,21 @@
       <c r="CS89" t="n">
         <v>0</v>
       </c>
+      <c r="CV89" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW89" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX89" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY89" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ89" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -19413,6 +20726,21 @@
       <c r="CS90" t="n">
         <v>0</v>
       </c>
+      <c r="CV90" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW90" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX90" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY90" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ90" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -19627,6 +20955,21 @@
       <c r="CS91" t="n">
         <v>0</v>
       </c>
+      <c r="CV91" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW91" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX91" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY91" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ91" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -19841,6 +21184,21 @@
       <c r="CS92" t="n">
         <v>4</v>
       </c>
+      <c r="CV92" t="n">
+        <v>68</v>
+      </c>
+      <c r="CW92" t="n">
+        <v>165</v>
+      </c>
+      <c r="CX92" t="n">
+        <v>459</v>
+      </c>
+      <c r="CY92" t="n">
+        <v>38</v>
+      </c>
+      <c r="CZ92" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -20055,6 +21413,21 @@
       <c r="CS93" t="n">
         <v>4</v>
       </c>
+      <c r="CV93" t="n">
+        <v>68</v>
+      </c>
+      <c r="CW93" t="n">
+        <v>165</v>
+      </c>
+      <c r="CX93" t="n">
+        <v>459</v>
+      </c>
+      <c r="CY93" t="n">
+        <v>38</v>
+      </c>
+      <c r="CZ93" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -20269,6 +21642,21 @@
       <c r="CS94" t="n">
         <v>0</v>
       </c>
+      <c r="CV94" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW94" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX94" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY94" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ94" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -20483,6 +21871,21 @@
       <c r="CS95" t="n">
         <v>40</v>
       </c>
+      <c r="CV95" t="n">
+        <v>65</v>
+      </c>
+      <c r="CW95" t="n">
+        <v>36</v>
+      </c>
+      <c r="CX95" t="n">
+        <v>102</v>
+      </c>
+      <c r="CY95" t="n">
+        <v>83</v>
+      </c>
+      <c r="CZ95" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -20697,6 +22100,21 @@
       <c r="CS96" t="n">
         <v>40</v>
       </c>
+      <c r="CV96" t="n">
+        <v>65</v>
+      </c>
+      <c r="CW96" t="n">
+        <v>36</v>
+      </c>
+      <c r="CX96" t="n">
+        <v>102</v>
+      </c>
+      <c r="CY96" t="n">
+        <v>83</v>
+      </c>
+      <c r="CZ96" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -20911,6 +22329,21 @@
       <c r="CS97" t="n">
         <v>0</v>
       </c>
+      <c r="CV97" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW97" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX97" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY97" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -21125,6 +22558,21 @@
       <c r="CS98" t="n">
         <v>0</v>
       </c>
+      <c r="CV98" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW98" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX98" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY98" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ98" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -21339,6 +22787,21 @@
       <c r="CS99" t="n">
         <v>0</v>
       </c>
+      <c r="CV99" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW99" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX99" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY99" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ99" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -21553,6 +23016,21 @@
       <c r="CS100" t="n">
         <v>0</v>
       </c>
+      <c r="CV100" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW100" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX100" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY100" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -21767,6 +23245,21 @@
       <c r="CS101" t="n">
         <v>0</v>
       </c>
+      <c r="CV101" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW101" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX101" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY101" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ101" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -21981,6 +23474,21 @@
       <c r="CS102" t="n">
         <v>0</v>
       </c>
+      <c r="CV102" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW102" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX102" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY102" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ102" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -22195,6 +23703,21 @@
       <c r="CS103" t="n">
         <v>0</v>
       </c>
+      <c r="CV103" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW103" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX103" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY103" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ103" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -22409,6 +23932,21 @@
       <c r="CS104" t="n">
         <v>0</v>
       </c>
+      <c r="CV104" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW104" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX104" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY104" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ104" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -22623,6 +24161,21 @@
       <c r="CS105" t="n">
         <v>0</v>
       </c>
+      <c r="CV105" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW105" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX105" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY105" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ105" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -22837,6 +24390,21 @@
       <c r="CS106" t="n">
         <v>0</v>
       </c>
+      <c r="CV106" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW106" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX106" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY106" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ106" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -23051,6 +24619,21 @@
       <c r="CS107" t="n">
         <v>0</v>
       </c>
+      <c r="CV107" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW107" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX107" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY107" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ107" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -23265,6 +24848,21 @@
       <c r="CS108" t="n">
         <v>0</v>
       </c>
+      <c r="CV108" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW108" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX108" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY108" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ108" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -23479,6 +25077,21 @@
       <c r="CS109" t="n">
         <v>0</v>
       </c>
+      <c r="CV109" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW109" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX109" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY109" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ109" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -23693,6 +25306,21 @@
       <c r="CS110" t="n">
         <v>0</v>
       </c>
+      <c r="CV110" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW110" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX110" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY110" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ110" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -23907,6 +25535,21 @@
       <c r="CS111" t="n">
         <v>0</v>
       </c>
+      <c r="CV111" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW111" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX111" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY111" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ111" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -24121,6 +25764,21 @@
       <c r="CS112" t="n">
         <v>0</v>
       </c>
+      <c r="CV112" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW112" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX112" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY112" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ112" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -24335,6 +25993,21 @@
       <c r="CS113" t="n">
         <v>0</v>
       </c>
+      <c r="CV113" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW113" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX113" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY113" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ113" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -24549,6 +26222,21 @@
       <c r="CS114" t="n">
         <v>0</v>
       </c>
+      <c r="CV114" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW114" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX114" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY114" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ114" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -24763,6 +26451,21 @@
       <c r="CS115" t="n">
         <v>0</v>
       </c>
+      <c r="CV115" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW115" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX115" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY115" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ115" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -24977,6 +26680,21 @@
       <c r="CS116" t="n">
         <v>0</v>
       </c>
+      <c r="CV116" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW116" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX116" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY116" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ116" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -25191,6 +26909,21 @@
       <c r="CS117" t="n">
         <v>0</v>
       </c>
+      <c r="CV117" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW117" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX117" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY117" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ117" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -25405,6 +27138,21 @@
       <c r="CS118" t="n">
         <v>0</v>
       </c>
+      <c r="CV118" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW118" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX118" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY118" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ118" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -25619,6 +27367,21 @@
       <c r="CS119" t="n">
         <v>0</v>
       </c>
+      <c r="CV119" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW119" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX119" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY119" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ119" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -25833,6 +27596,21 @@
       <c r="CS120" t="n">
         <v>0</v>
       </c>
+      <c r="CV120" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW120" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX120" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY120" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ120" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -26047,13 +27825,28 @@
       <c r="CS121" t="n">
         <v>0</v>
       </c>
+      <c r="CV121" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW121" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX121" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY121" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ121" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="15">
+    <mergeCell ref="AD1:AI1"/>
     <mergeCell ref="BT1:BY1"/>
+    <mergeCell ref="P1:U1"/>
     <mergeCell ref="AR1:AW1"/>
-    <mergeCell ref="P1:U1"/>
-    <mergeCell ref="AD1:AI1"/>
     <mergeCell ref="CA1:CF1"/>
     <mergeCell ref="BM1:BR1"/>
     <mergeCell ref="W1:AB1"/>
@@ -26064,6 +27857,7 @@
     <mergeCell ref="I1:N1"/>
     <mergeCell ref="BF1:BK1"/>
     <mergeCell ref="CO1:CT1"/>
+    <mergeCell ref="CV1:DA1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added PDF extract kit to main pipline + updated algo
</commit_message>
<xml_diff>
--- a/tests/regression_test/results/master_results.xlsx
+++ b/tests/regression_test/results/master_results.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17460" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="AllVersions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AllVersions" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DA121"/>
+  <dimension ref="A1:DO121"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30.33203125" customWidth="1" style="4" min="1" max="1"/>
@@ -527,6 +527,16 @@
           <t>bold-italic-formatting</t>
         </is>
       </c>
+      <c r="DC1" s="3" t="inlineStr">
+        <is>
+          <t>pdfextractkit</t>
+        </is>
+      </c>
+      <c r="DJ1" s="3" t="inlineStr">
+        <is>
+          <t>algo_check</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -984,6 +994,66 @@
           <t>avg.</t>
         </is>
       </c>
+      <c r="DC2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="DD2" t="inlineStr">
+        <is>
+          <t>algorithms</t>
+        </is>
+      </c>
+      <c r="DE2" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="DF2" t="inlineStr">
+        <is>
+          <t>cybersec</t>
+        </is>
+      </c>
+      <c r="DG2" t="inlineStr">
+        <is>
+          <t>data-science</t>
+        </is>
+      </c>
+      <c r="DH2" t="inlineStr">
+        <is>
+          <t>avg.</t>
+        </is>
+      </c>
+      <c r="DJ2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="DK2" t="inlineStr">
+        <is>
+          <t>algorithms</t>
+        </is>
+      </c>
+      <c r="DL2" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="DM2" t="inlineStr">
+        <is>
+          <t>cybersec</t>
+        </is>
+      </c>
+      <c r="DN2" t="inlineStr">
+        <is>
+          <t>data-science</t>
+        </is>
+      </c>
+      <c r="DO2" t="inlineStr">
+        <is>
+          <t>avg.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1361,6 +1431,56 @@
           <t>data-science</t>
         </is>
       </c>
+      <c r="DC3" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="DD3" t="inlineStr">
+        <is>
+          <t>algorithms</t>
+        </is>
+      </c>
+      <c r="DE3" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="DF3" t="inlineStr">
+        <is>
+          <t>cybersec</t>
+        </is>
+      </c>
+      <c r="DG3" t="inlineStr">
+        <is>
+          <t>data-science</t>
+        </is>
+      </c>
+      <c r="DJ3" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="DK3" t="inlineStr">
+        <is>
+          <t>algorithms</t>
+        </is>
+      </c>
+      <c r="DL3" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="DM3" t="inlineStr">
+        <is>
+          <t>cybersec</t>
+        </is>
+      </c>
+      <c r="DN3" t="inlineStr">
+        <is>
+          <t>data-science</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1738,6 +1858,56 @@
           <t>multi-metric</t>
         </is>
       </c>
+      <c r="DC4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="DD4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="DE4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="DF4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="DG4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="DJ4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="DK4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="DL4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="DM4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
+      <c r="DN4" t="inlineStr">
+        <is>
+          <t>multi-metric</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2115,6 +2285,56 @@
           <t>2025-12-01T14:00:51.042050</t>
         </is>
       </c>
+      <c r="DC5" t="inlineStr">
+        <is>
+          <t>2025-12-15T16:10:03.406267</t>
+        </is>
+      </c>
+      <c r="DD5" t="inlineStr">
+        <is>
+          <t>2025-12-15T16:10:03.620470</t>
+        </is>
+      </c>
+      <c r="DE5" t="inlineStr">
+        <is>
+          <t>2025-12-15T16:10:03.798597</t>
+        </is>
+      </c>
+      <c r="DF5" t="inlineStr">
+        <is>
+          <t>2025-12-15T16:10:03.905619</t>
+        </is>
+      </c>
+      <c r="DG5" t="inlineStr">
+        <is>
+          <t>2025-12-15T16:10:04.056492</t>
+        </is>
+      </c>
+      <c r="DJ5" t="inlineStr">
+        <is>
+          <t>2025-12-15T19:20:07.784854</t>
+        </is>
+      </c>
+      <c r="DK5" t="inlineStr">
+        <is>
+          <t>2025-12-15T19:20:07.982985</t>
+        </is>
+      </c>
+      <c r="DL5" t="inlineStr">
+        <is>
+          <t>2025-12-15T19:20:08.169760</t>
+        </is>
+      </c>
+      <c r="DM5" t="inlineStr">
+        <is>
+          <t>2025-12-15T19:20:08.308684</t>
+        </is>
+      </c>
+      <c r="DN5" t="inlineStr">
+        <is>
+          <t>2025-12-15T19:20:08.424451</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2389,6 +2609,42 @@
       <c r="DA6" s="5" t="n">
         <v>-80.14</v>
       </c>
+      <c r="DC6" s="5" t="n">
+        <v>-34.2</v>
+      </c>
+      <c r="DD6" s="5" t="n">
+        <v>-181.8</v>
+      </c>
+      <c r="DE6" s="6" t="n">
+        <v>-31.5</v>
+      </c>
+      <c r="DF6" s="5" t="n">
+        <v>-71.09999999999999</v>
+      </c>
+      <c r="DG6" s="5" t="n">
+        <v>-45.4</v>
+      </c>
+      <c r="DH6" s="5" t="n">
+        <v>-72.8</v>
+      </c>
+      <c r="DJ6" t="n">
+        <v>-34.2</v>
+      </c>
+      <c r="DK6" s="6" t="n">
+        <v>-185.3</v>
+      </c>
+      <c r="DL6" t="n">
+        <v>-31.5</v>
+      </c>
+      <c r="DM6" t="n">
+        <v>-71.09999999999999</v>
+      </c>
+      <c r="DN6" t="n">
+        <v>-45.4</v>
+      </c>
+      <c r="DO6" s="6" t="n">
+        <v>-73.5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2618,6 +2874,36 @@
       <c r="CZ7" t="n">
         <v>100</v>
       </c>
+      <c r="DC7" t="n">
+        <v>100</v>
+      </c>
+      <c r="DD7" s="5" t="n">
+        <v>65.75</v>
+      </c>
+      <c r="DE7" t="n">
+        <v>100</v>
+      </c>
+      <c r="DF7" t="n">
+        <v>100</v>
+      </c>
+      <c r="DG7" t="n">
+        <v>100</v>
+      </c>
+      <c r="DJ7" t="n">
+        <v>100</v>
+      </c>
+      <c r="DK7" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="DL7" t="n">
+        <v>100</v>
+      </c>
+      <c r="DM7" t="n">
+        <v>100</v>
+      </c>
+      <c r="DN7" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2847,6 +3133,36 @@
       <c r="CZ8" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="DC8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD8" s="5" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="DE8" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="DF8" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="DG8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="DL8" t="n">
+        <v>5</v>
+      </c>
+      <c r="DM8" t="n">
+        <v>3</v>
+      </c>
+      <c r="DN8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3076,6 +3392,36 @@
       <c r="CZ9" s="5" t="n">
         <v>3</v>
       </c>
+      <c r="DC9" t="n">
+        <v>7</v>
+      </c>
+      <c r="DD9" s="5" t="n">
+        <v>9.130000000000001</v>
+      </c>
+      <c r="DE9" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="DF9" t="n">
+        <v>6</v>
+      </c>
+      <c r="DG9" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="DJ9" t="n">
+        <v>7</v>
+      </c>
+      <c r="DK9" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="DL9" t="n">
+        <v>7</v>
+      </c>
+      <c r="DM9" t="n">
+        <v>6</v>
+      </c>
+      <c r="DN9" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3305,6 +3651,36 @@
       <c r="CZ10" t="n">
         <v>100</v>
       </c>
+      <c r="DC10" t="n">
+        <v>100</v>
+      </c>
+      <c r="DD10" t="n">
+        <v>100</v>
+      </c>
+      <c r="DE10" t="n">
+        <v>100</v>
+      </c>
+      <c r="DF10" t="n">
+        <v>100</v>
+      </c>
+      <c r="DG10" t="n">
+        <v>100</v>
+      </c>
+      <c r="DJ10" t="n">
+        <v>100</v>
+      </c>
+      <c r="DK10" t="n">
+        <v>100</v>
+      </c>
+      <c r="DL10" t="n">
+        <v>100</v>
+      </c>
+      <c r="DM10" t="n">
+        <v>100</v>
+      </c>
+      <c r="DN10" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3534,6 +3910,36 @@
       <c r="CZ11" t="n">
         <v>86.79000000000001</v>
       </c>
+      <c r="DC11" t="n">
+        <v>99.56999999999999</v>
+      </c>
+      <c r="DD11" t="n">
+        <v>90.84</v>
+      </c>
+      <c r="DE11" t="n">
+        <v>100</v>
+      </c>
+      <c r="DF11" t="n">
+        <v>99.01000000000001</v>
+      </c>
+      <c r="DG11" t="n">
+        <v>86.79000000000001</v>
+      </c>
+      <c r="DJ11" t="n">
+        <v>99.56999999999999</v>
+      </c>
+      <c r="DK11" s="5" t="n">
+        <v>91.17</v>
+      </c>
+      <c r="DL11" t="n">
+        <v>100</v>
+      </c>
+      <c r="DM11" t="n">
+        <v>99.01000000000001</v>
+      </c>
+      <c r="DN11" t="n">
+        <v>86.79000000000001</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3763,6 +4169,36 @@
       <c r="CZ12" t="n">
         <v>130.77</v>
       </c>
+      <c r="DC12" t="n">
+        <v>100</v>
+      </c>
+      <c r="DD12" t="n">
+        <v>113.64</v>
+      </c>
+      <c r="DE12" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="DF12" t="n">
+        <v>90.48</v>
+      </c>
+      <c r="DG12" t="n">
+        <v>130.77</v>
+      </c>
+      <c r="DJ12" t="n">
+        <v>100</v>
+      </c>
+      <c r="DK12" s="5" t="n">
+        <v>118.18</v>
+      </c>
+      <c r="DL12" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="DM12" t="n">
+        <v>90.48</v>
+      </c>
+      <c r="DN12" t="n">
+        <v>130.77</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3992,6 +4428,36 @@
       <c r="CZ13" s="6" t="n">
         <v>72.38</v>
       </c>
+      <c r="DC13" t="n">
+        <v>98.97</v>
+      </c>
+      <c r="DD13" t="n">
+        <v>99</v>
+      </c>
+      <c r="DE13" t="n">
+        <v>92.06</v>
+      </c>
+      <c r="DF13" t="n">
+        <v>81.25</v>
+      </c>
+      <c r="DG13" t="n">
+        <v>72.38</v>
+      </c>
+      <c r="DJ13" t="n">
+        <v>98.97</v>
+      </c>
+      <c r="DK13" s="5" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="DL13" t="n">
+        <v>92.06</v>
+      </c>
+      <c r="DM13" t="n">
+        <v>81.25</v>
+      </c>
+      <c r="DN13" t="n">
+        <v>72.38</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4221,6 +4687,36 @@
       <c r="CZ14" s="6" t="n">
         <v>83.23999999999999</v>
       </c>
+      <c r="DC14" t="n">
+        <v>92.59</v>
+      </c>
+      <c r="DD14" t="n">
+        <v>96.03</v>
+      </c>
+      <c r="DE14" t="n">
+        <v>100</v>
+      </c>
+      <c r="DF14" t="n">
+        <v>88.17</v>
+      </c>
+      <c r="DG14" t="n">
+        <v>83.23999999999999</v>
+      </c>
+      <c r="DJ14" t="n">
+        <v>92.59</v>
+      </c>
+      <c r="DK14" s="5" t="n">
+        <v>97.62</v>
+      </c>
+      <c r="DL14" t="n">
+        <v>100</v>
+      </c>
+      <c r="DM14" t="n">
+        <v>88.17</v>
+      </c>
+      <c r="DN14" t="n">
+        <v>83.23999999999999</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4450,6 +4946,36 @@
       <c r="CZ15" t="n">
         <v>91.86</v>
       </c>
+      <c r="DC15" s="5" t="n">
+        <v>90.66</v>
+      </c>
+      <c r="DD15" s="5" t="n">
+        <v>41.59</v>
+      </c>
+      <c r="DE15" s="5" t="n">
+        <v>119.05</v>
+      </c>
+      <c r="DF15" s="5" t="n">
+        <v>102.26</v>
+      </c>
+      <c r="DG15" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="DJ15" t="n">
+        <v>90.66</v>
+      </c>
+      <c r="DK15" s="5" t="n">
+        <v>148.6</v>
+      </c>
+      <c r="DL15" t="n">
+        <v>119.05</v>
+      </c>
+      <c r="DM15" t="n">
+        <v>102.26</v>
+      </c>
+      <c r="DN15" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4679,6 +5205,36 @@
       <c r="CZ16" t="n">
         <v>134.38</v>
       </c>
+      <c r="DC16" t="n">
+        <v>159.38</v>
+      </c>
+      <c r="DD16" t="n">
+        <v>164.29</v>
+      </c>
+      <c r="DE16" t="n">
+        <v>81.09999999999999</v>
+      </c>
+      <c r="DF16" t="n">
+        <v>224.53</v>
+      </c>
+      <c r="DG16" t="n">
+        <v>134.38</v>
+      </c>
+      <c r="DJ16" t="n">
+        <v>159.38</v>
+      </c>
+      <c r="DK16" s="5" t="n">
+        <v>238.1</v>
+      </c>
+      <c r="DL16" t="n">
+        <v>81.09999999999999</v>
+      </c>
+      <c r="DM16" t="n">
+        <v>224.53</v>
+      </c>
+      <c r="DN16" t="n">
+        <v>134.38</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4908,6 +5464,36 @@
       <c r="CZ17" t="n">
         <v>99.40000000000001</v>
       </c>
+      <c r="DC17" t="n">
+        <v>99.31999999999999</v>
+      </c>
+      <c r="DD17" t="n">
+        <v>89.02</v>
+      </c>
+      <c r="DE17" t="n">
+        <v>100.92</v>
+      </c>
+      <c r="DF17" t="n">
+        <v>96</v>
+      </c>
+      <c r="DG17" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="DJ17" t="n">
+        <v>99.31999999999999</v>
+      </c>
+      <c r="DK17" s="5" t="n">
+        <v>89.25</v>
+      </c>
+      <c r="DL17" t="n">
+        <v>100.92</v>
+      </c>
+      <c r="DM17" t="n">
+        <v>96</v>
+      </c>
+      <c r="DN17" t="n">
+        <v>99.40000000000001</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4915,7 +5501,7 @@
           <t>------------</t>
         </is>
       </c>
-      <c r="CZ18" t="inlineStr"/>
+      <c r="DN18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4923,7 +5509,7 @@
           <t>Score Deductions:</t>
         </is>
       </c>
-      <c r="CZ19" t="inlineStr"/>
+      <c r="DN19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5153,6 +5739,36 @@
       <c r="CZ20" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="DC20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD20" s="6" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="DE20" s="6" t="n">
+        <v>7.94</v>
+      </c>
+      <c r="DF20" s="6" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="DG20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ20" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK20" s="5" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="DL20" t="n">
+        <v>7.94</v>
+      </c>
+      <c r="DM20" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="DN20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5382,6 +5998,36 @@
       <c r="CZ21" s="5" t="n">
         <v>0.57</v>
       </c>
+      <c r="DC21" s="6" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="DD21" s="6" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="DE21" s="5" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="DF21" s="6" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="DG21" s="5" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="DJ21" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="DK21" s="6" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="DL21" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="DM21" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="DN21" t="n">
+        <v>0.44</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5611,6 +6257,36 @@
       <c r="CZ22" t="n">
         <v>0</v>
       </c>
+      <c r="DC22" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD22" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE22" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF22" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG22" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ22" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK22" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL22" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM22" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5840,6 +6516,36 @@
       <c r="CZ23" s="6" t="n">
         <v>13.33</v>
       </c>
+      <c r="DC23" s="6" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="DD23" s="6" t="n">
+        <v>22.83</v>
+      </c>
+      <c r="DE23" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF23" s="6" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="DG23" s="6" t="n">
+        <v>15.42</v>
+      </c>
+      <c r="DJ23" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="DK23" s="5" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="DL23" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM23" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="DN23" t="n">
+        <v>15.42</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6069,6 +6775,36 @@
       <c r="CZ24" s="6" t="n">
         <v>3.81</v>
       </c>
+      <c r="DC24" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD24" s="6" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="DE24" s="5" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="DF24" s="6" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="DG24" s="6" t="n">
+        <v>4.41</v>
+      </c>
+      <c r="DJ24" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK24" s="6" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="DL24" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="DM24" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="DN24" t="n">
+        <v>4.41</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6298,6 +7034,36 @@
       <c r="CZ25" s="6" t="n">
         <v>27.62</v>
       </c>
+      <c r="DC25" s="6" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="DD25" s="6" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="DE25" s="5" t="n">
+        <v>15.87</v>
+      </c>
+      <c r="DF25" s="6" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="DG25" s="6" t="n">
+        <v>31.94</v>
+      </c>
+      <c r="DJ25" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="DK25" s="6" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="DL25" t="n">
+        <v>15.87</v>
+      </c>
+      <c r="DM25" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="DN25" t="n">
+        <v>31.94</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6527,6 +7293,36 @@
       <c r="CZ26" s="6" t="n">
         <v>28.57</v>
       </c>
+      <c r="DC26" s="6" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="DD26" s="6" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="DE26" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF26" s="6" t="n">
+        <v>14.06</v>
+      </c>
+      <c r="DG26" s="6" t="n">
+        <v>33.04</v>
+      </c>
+      <c r="DJ26" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="DK26" s="5" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="DL26" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM26" t="n">
+        <v>14.06</v>
+      </c>
+      <c r="DN26" t="n">
+        <v>33.04</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6756,6 +7552,36 @@
       <c r="CZ27" s="6" t="n">
         <v>13.33</v>
       </c>
+      <c r="DC27" s="5" t="n">
+        <v>24.85</v>
+      </c>
+      <c r="DD27" s="5" t="n">
+        <v>34.38</v>
+      </c>
+      <c r="DE27" s="6" t="n">
+        <v>19.05</v>
+      </c>
+      <c r="DF27" s="5" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="DG27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ27" t="n">
+        <v>24.85</v>
+      </c>
+      <c r="DK27" s="5" t="n">
+        <v>28.06</v>
+      </c>
+      <c r="DL27" t="n">
+        <v>19.05</v>
+      </c>
+      <c r="DM27" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="DN27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6985,6 +7811,36 @@
       <c r="CZ28" s="6" t="n">
         <v>10.48</v>
       </c>
+      <c r="DC28" s="6" t="n">
+        <v>55.56</v>
+      </c>
+      <c r="DD28" s="6" t="n">
+        <v>7.43</v>
+      </c>
+      <c r="DE28" s="5" t="n">
+        <v>49.21</v>
+      </c>
+      <c r="DF28" s="6" t="n">
+        <v>46.41</v>
+      </c>
+      <c r="DG28" s="6" t="n">
+        <v>12.11</v>
+      </c>
+      <c r="DJ28" t="n">
+        <v>55.56</v>
+      </c>
+      <c r="DK28" s="6" t="n">
+        <v>15.65</v>
+      </c>
+      <c r="DL28" t="n">
+        <v>49.21</v>
+      </c>
+      <c r="DM28" t="n">
+        <v>46.41</v>
+      </c>
+      <c r="DN28" t="n">
+        <v>12.11</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -7214,6 +8070,36 @@
       <c r="CZ29" s="6" t="n">
         <v>2.29</v>
       </c>
+      <c r="DC29" s="6" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="DD29" s="6" t="n">
+        <v>32.01</v>
+      </c>
+      <c r="DE29" s="5" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="DF29" s="6" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="DG29" s="6" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="DJ29" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="DK29" s="5" t="n">
+        <v>30.76</v>
+      </c>
+      <c r="DL29" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="DM29" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="DN29" t="n">
+        <v>2.64</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -7443,6 +8329,36 @@
       <c r="CZ30" t="n">
         <v>0</v>
       </c>
+      <c r="DC30" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD30" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE30" s="5" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="DF30" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG30" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ30" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK30" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL30" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="DM30" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -7450,7 +8366,7 @@
           <t>-----</t>
         </is>
       </c>
-      <c r="CZ31" t="inlineStr"/>
+      <c r="DN31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7680,6 +8596,36 @@
       <c r="CZ32" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="DC32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD32" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="DE32" s="6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="DF32" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="DG32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ32" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="DL32" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="DM32" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="DN32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7909,6 +8855,36 @@
       <c r="CZ33" s="5" t="n">
         <v>0.3</v>
       </c>
+      <c r="DC33" t="n">
+        <v>0.7000000000000001</v>
+      </c>
+      <c r="DD33" t="n">
+        <v>0.6000000000000001</v>
+      </c>
+      <c r="DE33" s="5" t="n">
+        <v>0.7000000000000001</v>
+      </c>
+      <c r="DF33" t="n">
+        <v>0.6000000000000001</v>
+      </c>
+      <c r="DG33" s="5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="DJ33" t="n">
+        <v>0.7000000000000001</v>
+      </c>
+      <c r="DK33" s="6" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="DL33" t="n">
+        <v>0.7000000000000001</v>
+      </c>
+      <c r="DM33" t="n">
+        <v>0.6000000000000001</v>
+      </c>
+      <c r="DN33" t="n">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -8138,6 +9114,36 @@
       <c r="CZ34" t="n">
         <v>0</v>
       </c>
+      <c r="DC34" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD34" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE34" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF34" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG34" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ34" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK34" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL34" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM34" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -8367,6 +9373,36 @@
       <c r="CZ35" t="n">
         <v>7</v>
       </c>
+      <c r="DC35" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="DD35" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="DE35" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF35" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="DG35" t="n">
+        <v>7</v>
+      </c>
+      <c r="DJ35" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="DK35" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="DL35" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM35" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="DN35" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -8596,6 +9632,36 @@
       <c r="CZ36" t="n">
         <v>2</v>
       </c>
+      <c r="DC36" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD36" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="DE36" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="DF36" t="n">
+        <v>1</v>
+      </c>
+      <c r="DG36" t="n">
+        <v>2</v>
+      </c>
+      <c r="DJ36" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK36" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="DL36" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="DM36" t="n">
+        <v>1</v>
+      </c>
+      <c r="DN36" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -8825,6 +9891,36 @@
       <c r="CZ37" s="6" t="n">
         <v>14.5</v>
       </c>
+      <c r="DC37" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="DD37" t="n">
+        <v>1</v>
+      </c>
+      <c r="DE37" t="n">
+        <v>5</v>
+      </c>
+      <c r="DF37" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="DG37" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="DJ37" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="DK37" s="6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="DL37" t="n">
+        <v>5</v>
+      </c>
+      <c r="DM37" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="DN37" t="n">
+        <v>14.5</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -9054,6 +10150,36 @@
       <c r="CZ38" s="6" t="n">
         <v>15</v>
       </c>
+      <c r="DC38" t="n">
+        <v>4</v>
+      </c>
+      <c r="DD38" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="DE38" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF38" t="n">
+        <v>10</v>
+      </c>
+      <c r="DG38" t="n">
+        <v>15</v>
+      </c>
+      <c r="DJ38" t="n">
+        <v>4</v>
+      </c>
+      <c r="DK38" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="DL38" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM38" t="n">
+        <v>10</v>
+      </c>
+      <c r="DN38" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -9283,6 +10409,36 @@
       <c r="CZ39" t="n">
         <v>7</v>
       </c>
+      <c r="DC39" s="5" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="DD39" s="5" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="DE39" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="DF39" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="DG39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ39" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="DK39" s="5" t="n">
+        <v>52</v>
+      </c>
+      <c r="DL39" t="n">
+        <v>6</v>
+      </c>
+      <c r="DM39" t="n">
+        <v>2</v>
+      </c>
+      <c r="DN39" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -9512,6 +10668,36 @@
       <c r="CZ40" t="n">
         <v>5.5</v>
       </c>
+      <c r="DC40" t="n">
+        <v>19</v>
+      </c>
+      <c r="DD40" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="DE40" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="DF40" t="n">
+        <v>33</v>
+      </c>
+      <c r="DG40" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="DJ40" t="n">
+        <v>19</v>
+      </c>
+      <c r="DK40" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="DL40" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="DM40" t="n">
+        <v>33</v>
+      </c>
+      <c r="DN40" t="n">
+        <v>5.5</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -9741,6 +10927,36 @@
       <c r="CZ41" s="6" t="n">
         <v>1.2</v>
       </c>
+      <c r="DC41" t="n">
+        <v>1</v>
+      </c>
+      <c r="DD41" t="n">
+        <v>58.2</v>
+      </c>
+      <c r="DE41" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="DF41" t="n">
+        <v>15</v>
+      </c>
+      <c r="DG41" s="6" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="DJ41" t="n">
+        <v>1</v>
+      </c>
+      <c r="DK41" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="DL41" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="DM41" t="n">
+        <v>15</v>
+      </c>
+      <c r="DN41" s="6" t="n">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -9970,6 +11186,36 @@
       <c r="CZ42" t="n">
         <v>0</v>
       </c>
+      <c r="DC42" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD42" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE42" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="DF42" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG42" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ42" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK42" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL42" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="DM42" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN42" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -9977,7 +11223,7 @@
           <t>------------</t>
         </is>
       </c>
-      <c r="CZ43" t="inlineStr"/>
+      <c r="DN43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -10207,6 +11453,36 @@
       <c r="CZ44" t="n">
         <v>106</v>
       </c>
+      <c r="DC44" t="n">
+        <v>233</v>
+      </c>
+      <c r="DD44" t="n">
+        <v>906</v>
+      </c>
+      <c r="DE44" t="n">
+        <v>3</v>
+      </c>
+      <c r="DF44" t="n">
+        <v>101</v>
+      </c>
+      <c r="DG44" t="n">
+        <v>106</v>
+      </c>
+      <c r="DJ44" t="n">
+        <v>233</v>
+      </c>
+      <c r="DK44" t="n">
+        <v>906</v>
+      </c>
+      <c r="DL44" t="n">
+        <v>3</v>
+      </c>
+      <c r="DM44" t="n">
+        <v>101</v>
+      </c>
+      <c r="DN44" t="n">
+        <v>106</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -10436,6 +11712,36 @@
       <c r="CZ45" t="n">
         <v>106</v>
       </c>
+      <c r="DC45" t="n">
+        <v>233</v>
+      </c>
+      <c r="DD45" t="n">
+        <v>906</v>
+      </c>
+      <c r="DE45" t="n">
+        <v>3</v>
+      </c>
+      <c r="DF45" t="n">
+        <v>101</v>
+      </c>
+      <c r="DG45" t="n">
+        <v>106</v>
+      </c>
+      <c r="DJ45" t="n">
+        <v>233</v>
+      </c>
+      <c r="DK45" t="n">
+        <v>906</v>
+      </c>
+      <c r="DL45" t="n">
+        <v>3</v>
+      </c>
+      <c r="DM45" t="n">
+        <v>101</v>
+      </c>
+      <c r="DN45" t="n">
+        <v>106</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -10665,6 +11971,36 @@
       <c r="CZ46" t="n">
         <v>92</v>
       </c>
+      <c r="DC46" t="n">
+        <v>232</v>
+      </c>
+      <c r="DD46" t="n">
+        <v>823</v>
+      </c>
+      <c r="DE46" t="n">
+        <v>3</v>
+      </c>
+      <c r="DF46" t="n">
+        <v>100</v>
+      </c>
+      <c r="DG46" t="n">
+        <v>92</v>
+      </c>
+      <c r="DJ46" t="n">
+        <v>232</v>
+      </c>
+      <c r="DK46" s="5" t="n">
+        <v>826</v>
+      </c>
+      <c r="DL46" t="n">
+        <v>3</v>
+      </c>
+      <c r="DM46" t="n">
+        <v>100</v>
+      </c>
+      <c r="DN46" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -10894,6 +12230,36 @@
       <c r="CZ47" t="n">
         <v>0</v>
       </c>
+      <c r="DC47" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD47" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE47" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF47" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG47" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ47" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK47" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL47" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM47" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -11123,6 +12489,36 @@
       <c r="CZ48" t="n">
         <v>14</v>
       </c>
+      <c r="DC48" t="n">
+        <v>1</v>
+      </c>
+      <c r="DD48" t="n">
+        <v>83</v>
+      </c>
+      <c r="DE48" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF48" t="n">
+        <v>1</v>
+      </c>
+      <c r="DG48" t="n">
+        <v>14</v>
+      </c>
+      <c r="DJ48" t="n">
+        <v>1</v>
+      </c>
+      <c r="DK48" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="DL48" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM48" t="n">
+        <v>1</v>
+      </c>
+      <c r="DN48" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -11352,6 +12748,36 @@
       <c r="CZ49" t="n">
         <v>13</v>
       </c>
+      <c r="DC49" t="n">
+        <v>14</v>
+      </c>
+      <c r="DD49" t="n">
+        <v>22</v>
+      </c>
+      <c r="DE49" t="n">
+        <v>16</v>
+      </c>
+      <c r="DF49" t="n">
+        <v>21</v>
+      </c>
+      <c r="DG49" t="n">
+        <v>13</v>
+      </c>
+      <c r="DJ49" t="n">
+        <v>14</v>
+      </c>
+      <c r="DK49" t="n">
+        <v>22</v>
+      </c>
+      <c r="DL49" t="n">
+        <v>16</v>
+      </c>
+      <c r="DM49" t="n">
+        <v>21</v>
+      </c>
+      <c r="DN49" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -11581,6 +13007,36 @@
       <c r="CZ50" t="n">
         <v>17</v>
       </c>
+      <c r="DC50" t="n">
+        <v>14</v>
+      </c>
+      <c r="DD50" t="n">
+        <v>25</v>
+      </c>
+      <c r="DE50" t="n">
+        <v>15</v>
+      </c>
+      <c r="DF50" t="n">
+        <v>19</v>
+      </c>
+      <c r="DG50" t="n">
+        <v>17</v>
+      </c>
+      <c r="DJ50" t="n">
+        <v>14</v>
+      </c>
+      <c r="DK50" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="DL50" t="n">
+        <v>15</v>
+      </c>
+      <c r="DM50" t="n">
+        <v>19</v>
+      </c>
+      <c r="DN50" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -11810,6 +13266,36 @@
       <c r="CZ51" t="n">
         <v>-4</v>
       </c>
+      <c r="DC51" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD51" t="n">
+        <v>-3</v>
+      </c>
+      <c r="DE51" t="n">
+        <v>1</v>
+      </c>
+      <c r="DF51" t="n">
+        <v>2</v>
+      </c>
+      <c r="DG51" t="n">
+        <v>-4</v>
+      </c>
+      <c r="DJ51" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK51" s="6" t="n">
+        <v>-4</v>
+      </c>
+      <c r="DL51" t="n">
+        <v>1</v>
+      </c>
+      <c r="DM51" t="n">
+        <v>2</v>
+      </c>
+      <c r="DN51" t="n">
+        <v>-4</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -12039,6 +13525,36 @@
       <c r="CZ52" t="n">
         <v>105</v>
       </c>
+      <c r="DC52" t="n">
+        <v>97</v>
+      </c>
+      <c r="DD52" t="n">
+        <v>200</v>
+      </c>
+      <c r="DE52" t="n">
+        <v>126</v>
+      </c>
+      <c r="DF52" t="n">
+        <v>80</v>
+      </c>
+      <c r="DG52" t="n">
+        <v>105</v>
+      </c>
+      <c r="DJ52" t="n">
+        <v>97</v>
+      </c>
+      <c r="DK52" t="n">
+        <v>200</v>
+      </c>
+      <c r="DL52" t="n">
+        <v>126</v>
+      </c>
+      <c r="DM52" t="n">
+        <v>80</v>
+      </c>
+      <c r="DN52" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -12268,6 +13784,36 @@
       <c r="CZ53" s="6" t="n">
         <v>76</v>
       </c>
+      <c r="DC53" t="n">
+        <v>96</v>
+      </c>
+      <c r="DD53" t="n">
+        <v>198</v>
+      </c>
+      <c r="DE53" t="n">
+        <v>116</v>
+      </c>
+      <c r="DF53" t="n">
+        <v>65</v>
+      </c>
+      <c r="DG53" t="n">
+        <v>76</v>
+      </c>
+      <c r="DJ53" t="n">
+        <v>96</v>
+      </c>
+      <c r="DK53" s="5" t="n">
+        <v>205</v>
+      </c>
+      <c r="DL53" t="n">
+        <v>116</v>
+      </c>
+      <c r="DM53" t="n">
+        <v>65</v>
+      </c>
+      <c r="DN53" t="n">
+        <v>76</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -12497,6 +14043,36 @@
       <c r="CZ54" s="6" t="n">
         <v>29</v>
       </c>
+      <c r="DC54" t="n">
+        <v>1</v>
+      </c>
+      <c r="DD54" t="n">
+        <v>2</v>
+      </c>
+      <c r="DE54" t="n">
+        <v>10</v>
+      </c>
+      <c r="DF54" t="n">
+        <v>15</v>
+      </c>
+      <c r="DG54" t="n">
+        <v>29</v>
+      </c>
+      <c r="DJ54" t="n">
+        <v>1</v>
+      </c>
+      <c r="DK54" s="6" t="n">
+        <v>-5</v>
+      </c>
+      <c r="DL54" t="n">
+        <v>10</v>
+      </c>
+      <c r="DM54" t="n">
+        <v>15</v>
+      </c>
+      <c r="DN54" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -12726,6 +14302,36 @@
       <c r="CZ55" t="n">
         <v>179</v>
       </c>
+      <c r="DC55" t="n">
+        <v>108</v>
+      </c>
+      <c r="DD55" t="n">
+        <v>126</v>
+      </c>
+      <c r="DE55" t="n">
+        <v>12</v>
+      </c>
+      <c r="DF55" t="n">
+        <v>169</v>
+      </c>
+      <c r="DG55" t="n">
+        <v>179</v>
+      </c>
+      <c r="DJ55" t="n">
+        <v>108</v>
+      </c>
+      <c r="DK55" t="n">
+        <v>126</v>
+      </c>
+      <c r="DL55" t="n">
+        <v>12</v>
+      </c>
+      <c r="DM55" t="n">
+        <v>169</v>
+      </c>
+      <c r="DN55" t="n">
+        <v>179</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -12955,6 +14561,36 @@
       <c r="CZ56" s="6" t="n">
         <v>149</v>
       </c>
+      <c r="DC56" t="n">
+        <v>100</v>
+      </c>
+      <c r="DD56" t="n">
+        <v>121</v>
+      </c>
+      <c r="DE56" t="n">
+        <v>12</v>
+      </c>
+      <c r="DF56" t="n">
+        <v>149</v>
+      </c>
+      <c r="DG56" t="n">
+        <v>149</v>
+      </c>
+      <c r="DJ56" t="n">
+        <v>100</v>
+      </c>
+      <c r="DK56" s="5" t="n">
+        <v>123</v>
+      </c>
+      <c r="DL56" t="n">
+        <v>12</v>
+      </c>
+      <c r="DM56" t="n">
+        <v>149</v>
+      </c>
+      <c r="DN56" t="n">
+        <v>149</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -13184,6 +14820,36 @@
       <c r="CZ57" s="6" t="n">
         <v>30</v>
       </c>
+      <c r="DC57" t="n">
+        <v>8</v>
+      </c>
+      <c r="DD57" t="n">
+        <v>5</v>
+      </c>
+      <c r="DE57" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF57" t="n">
+        <v>20</v>
+      </c>
+      <c r="DG57" t="n">
+        <v>30</v>
+      </c>
+      <c r="DJ57" t="n">
+        <v>8</v>
+      </c>
+      <c r="DK57" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="DL57" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM57" t="n">
+        <v>20</v>
+      </c>
+      <c r="DN57" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -13413,6 +15079,36 @@
       <c r="CZ58" t="n">
         <v>172</v>
       </c>
+      <c r="DC58" t="n">
+        <v>182</v>
+      </c>
+      <c r="DD58" t="n">
+        <v>214</v>
+      </c>
+      <c r="DE58" t="n">
+        <v>63</v>
+      </c>
+      <c r="DF58" t="n">
+        <v>177</v>
+      </c>
+      <c r="DG58" t="n">
+        <v>172</v>
+      </c>
+      <c r="DJ58" t="n">
+        <v>182</v>
+      </c>
+      <c r="DK58" t="n">
+        <v>214</v>
+      </c>
+      <c r="DL58" t="n">
+        <v>63</v>
+      </c>
+      <c r="DM58" t="n">
+        <v>177</v>
+      </c>
+      <c r="DN58" t="n">
+        <v>172</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -13642,6 +15338,36 @@
       <c r="CZ59" t="n">
         <v>158</v>
       </c>
+      <c r="DC59" s="5" t="n">
+        <v>165</v>
+      </c>
+      <c r="DD59" s="5" t="n">
+        <v>89</v>
+      </c>
+      <c r="DE59" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="DF59" s="5" t="n">
+        <v>181</v>
+      </c>
+      <c r="DG59" s="5" t="n">
+        <v>172</v>
+      </c>
+      <c r="DJ59" t="n">
+        <v>165</v>
+      </c>
+      <c r="DK59" s="5" t="n">
+        <v>318</v>
+      </c>
+      <c r="DL59" t="n">
+        <v>75</v>
+      </c>
+      <c r="DM59" t="n">
+        <v>181</v>
+      </c>
+      <c r="DN59" t="n">
+        <v>172</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -13871,6 +15597,36 @@
       <c r="CZ60" t="n">
         <v>172</v>
       </c>
+      <c r="DC60" s="5" t="n">
+        <v>206</v>
+      </c>
+      <c r="DD60" s="5" t="n">
+        <v>93</v>
+      </c>
+      <c r="DE60" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="DF60" s="5" t="n">
+        <v>185</v>
+      </c>
+      <c r="DG60" s="5" t="n">
+        <v>186</v>
+      </c>
+      <c r="DJ60" t="n">
+        <v>206</v>
+      </c>
+      <c r="DK60" s="5" t="n">
+        <v>385</v>
+      </c>
+      <c r="DL60" t="n">
+        <v>75</v>
+      </c>
+      <c r="DM60" t="n">
+        <v>185</v>
+      </c>
+      <c r="DN60" t="n">
+        <v>186</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -14100,6 +15856,36 @@
       <c r="CZ61" t="n">
         <v>14</v>
       </c>
+      <c r="DC61" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="DD61" s="5" t="n">
+        <v>125</v>
+      </c>
+      <c r="DE61" s="6" t="n">
+        <v>-12</v>
+      </c>
+      <c r="DF61" s="5" t="n">
+        <v>-4</v>
+      </c>
+      <c r="DG61" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ61" t="n">
+        <v>17</v>
+      </c>
+      <c r="DK61" s="5" t="n">
+        <v>-104</v>
+      </c>
+      <c r="DL61" t="n">
+        <v>-12</v>
+      </c>
+      <c r="DM61" t="n">
+        <v>-4</v>
+      </c>
+      <c r="DN61" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -14329,6 +16115,36 @@
       <c r="CZ62" t="n">
         <v>32</v>
       </c>
+      <c r="DC62" t="n">
+        <v>64</v>
+      </c>
+      <c r="DD62" t="n">
+        <v>42</v>
+      </c>
+      <c r="DE62" t="n">
+        <v>164</v>
+      </c>
+      <c r="DF62" t="n">
+        <v>53</v>
+      </c>
+      <c r="DG62" t="n">
+        <v>32</v>
+      </c>
+      <c r="DJ62" t="n">
+        <v>64</v>
+      </c>
+      <c r="DK62" t="n">
+        <v>42</v>
+      </c>
+      <c r="DL62" t="n">
+        <v>164</v>
+      </c>
+      <c r="DM62" t="n">
+        <v>53</v>
+      </c>
+      <c r="DN62" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -14558,6 +16374,36 @@
       <c r="CZ63" t="n">
         <v>43</v>
       </c>
+      <c r="DC63" t="n">
+        <v>102</v>
+      </c>
+      <c r="DD63" t="n">
+        <v>69</v>
+      </c>
+      <c r="DE63" t="n">
+        <v>133</v>
+      </c>
+      <c r="DF63" t="n">
+        <v>119</v>
+      </c>
+      <c r="DG63" t="n">
+        <v>43</v>
+      </c>
+      <c r="DJ63" t="n">
+        <v>102</v>
+      </c>
+      <c r="DK63" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="DL63" t="n">
+        <v>133</v>
+      </c>
+      <c r="DM63" t="n">
+        <v>119</v>
+      </c>
+      <c r="DN63" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -14787,6 +16633,36 @@
       <c r="CZ64" t="n">
         <v>-11</v>
       </c>
+      <c r="DC64" t="n">
+        <v>-38</v>
+      </c>
+      <c r="DD64" t="n">
+        <v>-27</v>
+      </c>
+      <c r="DE64" t="n">
+        <v>31</v>
+      </c>
+      <c r="DF64" t="n">
+        <v>-66</v>
+      </c>
+      <c r="DG64" t="n">
+        <v>-11</v>
+      </c>
+      <c r="DJ64" t="n">
+        <v>-38</v>
+      </c>
+      <c r="DK64" s="6" t="n">
+        <v>-58</v>
+      </c>
+      <c r="DL64" t="n">
+        <v>31</v>
+      </c>
+      <c r="DM64" t="n">
+        <v>-66</v>
+      </c>
+      <c r="DN64" t="n">
+        <v>-11</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -15016,6 +16892,36 @@
       <c r="CZ65" t="n">
         <v>1003</v>
       </c>
+      <c r="DC65" t="n">
+        <v>731</v>
+      </c>
+      <c r="DD65" t="n">
+        <v>2651</v>
+      </c>
+      <c r="DE65" t="n">
+        <v>434</v>
+      </c>
+      <c r="DF65" t="n">
+        <v>1874</v>
+      </c>
+      <c r="DG65" t="n">
+        <v>1003</v>
+      </c>
+      <c r="DJ65" t="n">
+        <v>731</v>
+      </c>
+      <c r="DK65" t="n">
+        <v>2651</v>
+      </c>
+      <c r="DL65" t="n">
+        <v>434</v>
+      </c>
+      <c r="DM65" t="n">
+        <v>1874</v>
+      </c>
+      <c r="DN65" t="n">
+        <v>1003</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -15245,6 +17151,36 @@
       <c r="CZ66" t="n">
         <v>997</v>
       </c>
+      <c r="DC66" t="n">
+        <v>726</v>
+      </c>
+      <c r="DD66" t="n">
+        <v>2360</v>
+      </c>
+      <c r="DE66" t="n">
+        <v>438</v>
+      </c>
+      <c r="DF66" t="n">
+        <v>1799</v>
+      </c>
+      <c r="DG66" t="n">
+        <v>997</v>
+      </c>
+      <c r="DJ66" t="n">
+        <v>726</v>
+      </c>
+      <c r="DK66" s="5" t="n">
+        <v>2366</v>
+      </c>
+      <c r="DL66" t="n">
+        <v>438</v>
+      </c>
+      <c r="DM66" t="n">
+        <v>1799</v>
+      </c>
+      <c r="DN66" t="n">
+        <v>997</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -15474,6 +17410,36 @@
       <c r="CZ67" t="n">
         <v>6</v>
       </c>
+      <c r="DC67" t="n">
+        <v>5</v>
+      </c>
+      <c r="DD67" t="n">
+        <v>291</v>
+      </c>
+      <c r="DE67" t="n">
+        <v>-4</v>
+      </c>
+      <c r="DF67" t="n">
+        <v>75</v>
+      </c>
+      <c r="DG67" t="n">
+        <v>6</v>
+      </c>
+      <c r="DJ67" t="n">
+        <v>5</v>
+      </c>
+      <c r="DK67" s="5" t="n">
+        <v>285</v>
+      </c>
+      <c r="DL67" t="n">
+        <v>-4</v>
+      </c>
+      <c r="DM67" t="n">
+        <v>75</v>
+      </c>
+      <c r="DN67" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -15703,6 +17669,36 @@
       <c r="CZ68" s="5" t="n">
         <v>567</v>
       </c>
+      <c r="DC68" s="5" t="n">
+        <v>619</v>
+      </c>
+      <c r="DD68" s="5" t="n">
+        <v>545</v>
+      </c>
+      <c r="DE68" s="5" t="n">
+        <v>840</v>
+      </c>
+      <c r="DF68" s="5" t="n">
+        <v>834</v>
+      </c>
+      <c r="DG68" s="5" t="n">
+        <v>581</v>
+      </c>
+      <c r="DJ68" t="n">
+        <v>619</v>
+      </c>
+      <c r="DK68" s="5" t="n">
+        <v>1175</v>
+      </c>
+      <c r="DL68" t="n">
+        <v>840</v>
+      </c>
+      <c r="DM68" t="n">
+        <v>834</v>
+      </c>
+      <c r="DN68" t="n">
+        <v>581</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -15932,6 +17928,36 @@
       <c r="CZ69" s="5" t="n">
         <v>567</v>
       </c>
+      <c r="DC69" s="5" t="n">
+        <v>619</v>
+      </c>
+      <c r="DD69" s="5" t="n">
+        <v>545</v>
+      </c>
+      <c r="DE69" s="5" t="n">
+        <v>839</v>
+      </c>
+      <c r="DF69" s="5" t="n">
+        <v>834</v>
+      </c>
+      <c r="DG69" s="5" t="n">
+        <v>581</v>
+      </c>
+      <c r="DJ69" t="n">
+        <v>619</v>
+      </c>
+      <c r="DK69" s="5" t="n">
+        <v>1175</v>
+      </c>
+      <c r="DL69" t="n">
+        <v>839</v>
+      </c>
+      <c r="DM69" t="n">
+        <v>834</v>
+      </c>
+      <c r="DN69" t="n">
+        <v>581</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -16161,6 +18187,36 @@
       <c r="CZ70" t="n">
         <v>0</v>
       </c>
+      <c r="DC70" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD70" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE70" t="n">
+        <v>1</v>
+      </c>
+      <c r="DF70" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG70" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ70" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK70" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL70" t="n">
+        <v>1</v>
+      </c>
+      <c r="DM70" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN70" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -16390,6 +18446,36 @@
       <c r="CZ71" t="n">
         <v>1</v>
       </c>
+      <c r="DC71" t="n">
+        <v>1</v>
+      </c>
+      <c r="DD71" t="n">
+        <v>1</v>
+      </c>
+      <c r="DE71" t="n">
+        <v>1</v>
+      </c>
+      <c r="DF71" t="n">
+        <v>1</v>
+      </c>
+      <c r="DG71" t="n">
+        <v>1</v>
+      </c>
+      <c r="DJ71" t="n">
+        <v>1</v>
+      </c>
+      <c r="DK71" t="n">
+        <v>1</v>
+      </c>
+      <c r="DL71" t="n">
+        <v>1</v>
+      </c>
+      <c r="DM71" t="n">
+        <v>1</v>
+      </c>
+      <c r="DN71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -16619,6 +18705,36 @@
       <c r="CZ72" t="n">
         <v>1</v>
       </c>
+      <c r="DC72" t="n">
+        <v>1</v>
+      </c>
+      <c r="DD72" t="n">
+        <v>1</v>
+      </c>
+      <c r="DE72" t="n">
+        <v>1</v>
+      </c>
+      <c r="DF72" t="n">
+        <v>1</v>
+      </c>
+      <c r="DG72" t="n">
+        <v>1</v>
+      </c>
+      <c r="DJ72" t="n">
+        <v>1</v>
+      </c>
+      <c r="DK72" t="n">
+        <v>1</v>
+      </c>
+      <c r="DL72" t="n">
+        <v>1</v>
+      </c>
+      <c r="DM72" t="n">
+        <v>1</v>
+      </c>
+      <c r="DN72" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -16848,6 +18964,36 @@
       <c r="CZ73" t="n">
         <v>0</v>
       </c>
+      <c r="DC73" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD73" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE73" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF73" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG73" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ73" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK73" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL73" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM73" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -17077,6 +19223,36 @@
       <c r="CZ74" t="n">
         <v>158</v>
       </c>
+      <c r="DC74" s="5" t="n">
+        <v>165</v>
+      </c>
+      <c r="DD74" s="5" t="n">
+        <v>89</v>
+      </c>
+      <c r="DE74" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="DF74" s="5" t="n">
+        <v>181</v>
+      </c>
+      <c r="DG74" s="5" t="n">
+        <v>172</v>
+      </c>
+      <c r="DJ74" t="n">
+        <v>165</v>
+      </c>
+      <c r="DK74" s="5" t="n">
+        <v>318</v>
+      </c>
+      <c r="DL74" t="n">
+        <v>75</v>
+      </c>
+      <c r="DM74" t="n">
+        <v>181</v>
+      </c>
+      <c r="DN74" t="n">
+        <v>172</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -17306,6 +19482,36 @@
       <c r="CZ75" t="n">
         <v>158</v>
       </c>
+      <c r="DC75" s="5" t="n">
+        <v>165</v>
+      </c>
+      <c r="DD75" s="5" t="n">
+        <v>89</v>
+      </c>
+      <c r="DE75" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="DF75" s="5" t="n">
+        <v>181</v>
+      </c>
+      <c r="DG75" s="5" t="n">
+        <v>172</v>
+      </c>
+      <c r="DJ75" t="n">
+        <v>165</v>
+      </c>
+      <c r="DK75" s="5" t="n">
+        <v>318</v>
+      </c>
+      <c r="DL75" t="n">
+        <v>75</v>
+      </c>
+      <c r="DM75" t="n">
+        <v>181</v>
+      </c>
+      <c r="DN75" t="n">
+        <v>172</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -17535,6 +19741,36 @@
       <c r="CZ76" t="n">
         <v>0</v>
       </c>
+      <c r="DC76" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD76" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE76" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF76" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG76" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ76" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK76" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL76" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM76" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN76" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -17764,6 +20000,36 @@
       <c r="CZ77" t="n">
         <v>0</v>
       </c>
+      <c r="DC77" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD77" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE77" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF77" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG77" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ77" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK77" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="DL77" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM77" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -17993,6 +20259,36 @@
       <c r="CZ78" t="n">
         <v>0</v>
       </c>
+      <c r="DC78" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD78" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE78" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF78" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG78" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ78" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK78" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="DL78" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM78" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN78" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -18222,6 +20518,36 @@
       <c r="CZ79" t="n">
         <v>0</v>
       </c>
+      <c r="DC79" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD79" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE79" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF79" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG79" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ79" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK79" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL79" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM79" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN79" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -18451,6 +20777,36 @@
       <c r="CZ80" t="n">
         <v>43</v>
       </c>
+      <c r="DC80" t="n">
+        <v>102</v>
+      </c>
+      <c r="DD80" t="n">
+        <v>69</v>
+      </c>
+      <c r="DE80" t="n">
+        <v>133</v>
+      </c>
+      <c r="DF80" t="n">
+        <v>119</v>
+      </c>
+      <c r="DG80" t="n">
+        <v>43</v>
+      </c>
+      <c r="DJ80" t="n">
+        <v>102</v>
+      </c>
+      <c r="DK80" s="5" t="n">
+        <v>78</v>
+      </c>
+      <c r="DL80" t="n">
+        <v>133</v>
+      </c>
+      <c r="DM80" t="n">
+        <v>119</v>
+      </c>
+      <c r="DN80" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -18680,6 +21036,36 @@
       <c r="CZ81" t="n">
         <v>43</v>
       </c>
+      <c r="DC81" t="n">
+        <v>102</v>
+      </c>
+      <c r="DD81" t="n">
+        <v>69</v>
+      </c>
+      <c r="DE81" t="n">
+        <v>133</v>
+      </c>
+      <c r="DF81" t="n">
+        <v>119</v>
+      </c>
+      <c r="DG81" t="n">
+        <v>43</v>
+      </c>
+      <c r="DJ81" t="n">
+        <v>102</v>
+      </c>
+      <c r="DK81" s="5" t="n">
+        <v>78</v>
+      </c>
+      <c r="DL81" t="n">
+        <v>133</v>
+      </c>
+      <c r="DM81" t="n">
+        <v>119</v>
+      </c>
+      <c r="DN81" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -18909,6 +21295,36 @@
       <c r="CZ82" t="n">
         <v>0</v>
       </c>
+      <c r="DC82" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD82" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE82" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF82" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG82" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ82" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK82" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL82" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM82" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN82" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -19138,6 +21554,36 @@
       <c r="CZ83" t="n">
         <v>244</v>
       </c>
+      <c r="DC83" t="n">
+        <v>28</v>
+      </c>
+      <c r="DD83" t="n">
+        <v>114</v>
+      </c>
+      <c r="DE83" t="n">
+        <v>24</v>
+      </c>
+      <c r="DF83" t="n">
+        <v>265</v>
+      </c>
+      <c r="DG83" t="n">
+        <v>244</v>
+      </c>
+      <c r="DJ83" t="n">
+        <v>28</v>
+      </c>
+      <c r="DK83" s="5" t="n">
+        <v>325</v>
+      </c>
+      <c r="DL83" t="n">
+        <v>24</v>
+      </c>
+      <c r="DM83" t="n">
+        <v>265</v>
+      </c>
+      <c r="DN83" t="n">
+        <v>244</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -19367,6 +21813,36 @@
       <c r="CZ84" t="n">
         <v>244</v>
       </c>
+      <c r="DC84" t="n">
+        <v>28</v>
+      </c>
+      <c r="DD84" t="n">
+        <v>114</v>
+      </c>
+      <c r="DE84" t="n">
+        <v>24</v>
+      </c>
+      <c r="DF84" t="n">
+        <v>265</v>
+      </c>
+      <c r="DG84" t="n">
+        <v>244</v>
+      </c>
+      <c r="DJ84" t="n">
+        <v>28</v>
+      </c>
+      <c r="DK84" s="5" t="n">
+        <v>325</v>
+      </c>
+      <c r="DL84" t="n">
+        <v>24</v>
+      </c>
+      <c r="DM84" t="n">
+        <v>265</v>
+      </c>
+      <c r="DN84" t="n">
+        <v>244</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -19596,6 +22072,36 @@
       <c r="CZ85" t="n">
         <v>0</v>
       </c>
+      <c r="DC85" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD85" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE85" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF85" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG85" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ85" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK85" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL85" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM85" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -19825,6 +22331,36 @@
       <c r="CZ86" t="n">
         <v>1</v>
       </c>
+      <c r="DC86" t="n">
+        <v>9</v>
+      </c>
+      <c r="DD86" t="n">
+        <v>2</v>
+      </c>
+      <c r="DE86" t="n">
+        <v>38</v>
+      </c>
+      <c r="DF86" t="n">
+        <v>105</v>
+      </c>
+      <c r="DG86" t="n">
+        <v>1</v>
+      </c>
+      <c r="DJ86" t="n">
+        <v>9</v>
+      </c>
+      <c r="DK86" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="DL86" t="n">
+        <v>38</v>
+      </c>
+      <c r="DM86" t="n">
+        <v>105</v>
+      </c>
+      <c r="DN86" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -20054,6 +22590,36 @@
       <c r="CZ87" t="n">
         <v>1</v>
       </c>
+      <c r="DC87" t="n">
+        <v>9</v>
+      </c>
+      <c r="DD87" t="n">
+        <v>2</v>
+      </c>
+      <c r="DE87" t="n">
+        <v>38</v>
+      </c>
+      <c r="DF87" t="n">
+        <v>105</v>
+      </c>
+      <c r="DG87" t="n">
+        <v>1</v>
+      </c>
+      <c r="DJ87" t="n">
+        <v>9</v>
+      </c>
+      <c r="DK87" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="DL87" t="n">
+        <v>38</v>
+      </c>
+      <c r="DM87" t="n">
+        <v>105</v>
+      </c>
+      <c r="DN87" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -20283,6 +22849,36 @@
       <c r="CZ88" t="n">
         <v>0</v>
       </c>
+      <c r="DC88" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD88" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE88" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF88" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG88" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ88" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK88" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL88" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM88" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -20512,6 +23108,36 @@
       <c r="CZ89" t="n">
         <v>0</v>
       </c>
+      <c r="DC89" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD89" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE89" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF89" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG89" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ89" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK89" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL89" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM89" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN89" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -20741,6 +23367,36 @@
       <c r="CZ90" t="n">
         <v>0</v>
       </c>
+      <c r="DC90" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD90" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE90" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF90" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG90" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ90" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK90" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL90" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM90" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN90" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -20970,6 +23626,36 @@
       <c r="CZ91" t="n">
         <v>0</v>
       </c>
+      <c r="DC91" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD91" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE91" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF91" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG91" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ91" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK91" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL91" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM91" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN91" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -21199,6 +23885,36 @@
       <c r="CZ92" t="n">
         <v>4</v>
       </c>
+      <c r="DC92" t="n">
+        <v>68</v>
+      </c>
+      <c r="DD92" t="n">
+        <v>165</v>
+      </c>
+      <c r="DE92" t="n">
+        <v>459</v>
+      </c>
+      <c r="DF92" t="n">
+        <v>38</v>
+      </c>
+      <c r="DG92" t="n">
+        <v>4</v>
+      </c>
+      <c r="DJ92" t="n">
+        <v>68</v>
+      </c>
+      <c r="DK92" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="DL92" t="n">
+        <v>459</v>
+      </c>
+      <c r="DM92" t="n">
+        <v>38</v>
+      </c>
+      <c r="DN92" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -21428,6 +24144,36 @@
       <c r="CZ93" t="n">
         <v>4</v>
       </c>
+      <c r="DC93" t="n">
+        <v>68</v>
+      </c>
+      <c r="DD93" t="n">
+        <v>165</v>
+      </c>
+      <c r="DE93" t="n">
+        <v>459</v>
+      </c>
+      <c r="DF93" t="n">
+        <v>38</v>
+      </c>
+      <c r="DG93" t="n">
+        <v>4</v>
+      </c>
+      <c r="DJ93" t="n">
+        <v>68</v>
+      </c>
+      <c r="DK93" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="DL93" t="n">
+        <v>459</v>
+      </c>
+      <c r="DM93" t="n">
+        <v>38</v>
+      </c>
+      <c r="DN93" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -21657,6 +24403,36 @@
       <c r="CZ94" t="n">
         <v>0</v>
       </c>
+      <c r="DC94" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD94" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE94" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF94" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG94" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ94" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK94" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL94" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM94" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN94" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -21886,6 +24662,36 @@
       <c r="CZ95" t="n">
         <v>40</v>
       </c>
+      <c r="DC95" t="n">
+        <v>65</v>
+      </c>
+      <c r="DD95" t="n">
+        <v>36</v>
+      </c>
+      <c r="DE95" t="n">
+        <v>102</v>
+      </c>
+      <c r="DF95" t="n">
+        <v>83</v>
+      </c>
+      <c r="DG95" t="n">
+        <v>40</v>
+      </c>
+      <c r="DJ95" t="n">
+        <v>65</v>
+      </c>
+      <c r="DK95" s="5" t="n">
+        <v>193</v>
+      </c>
+      <c r="DL95" t="n">
+        <v>102</v>
+      </c>
+      <c r="DM95" t="n">
+        <v>83</v>
+      </c>
+      <c r="DN95" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -22115,6 +24921,36 @@
       <c r="CZ96" t="n">
         <v>40</v>
       </c>
+      <c r="DC96" t="n">
+        <v>65</v>
+      </c>
+      <c r="DD96" t="n">
+        <v>36</v>
+      </c>
+      <c r="DE96" t="n">
+        <v>102</v>
+      </c>
+      <c r="DF96" t="n">
+        <v>83</v>
+      </c>
+      <c r="DG96" t="n">
+        <v>40</v>
+      </c>
+      <c r="DJ96" t="n">
+        <v>65</v>
+      </c>
+      <c r="DK96" s="5" t="n">
+        <v>193</v>
+      </c>
+      <c r="DL96" t="n">
+        <v>102</v>
+      </c>
+      <c r="DM96" t="n">
+        <v>83</v>
+      </c>
+      <c r="DN96" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -22344,6 +25180,36 @@
       <c r="CZ97" t="n">
         <v>0</v>
       </c>
+      <c r="DC97" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD97" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE97" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF97" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG97" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ97" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK97" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL97" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM97" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -22573,6 +25439,36 @@
       <c r="CZ98" t="n">
         <v>0</v>
       </c>
+      <c r="DC98" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD98" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE98" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF98" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG98" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ98" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK98" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL98" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM98" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN98" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -22802,6 +25698,36 @@
       <c r="CZ99" t="n">
         <v>0</v>
       </c>
+      <c r="DC99" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD99" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE99" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF99" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG99" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ99" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK99" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL99" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM99" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN99" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -23031,6 +25957,36 @@
       <c r="CZ100" t="n">
         <v>0</v>
       </c>
+      <c r="DC100" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD100" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE100" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF100" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG100" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ100" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK100" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL100" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM100" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -23260,6 +26216,36 @@
       <c r="CZ101" t="n">
         <v>0</v>
       </c>
+      <c r="DC101" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD101" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE101" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF101" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG101" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ101" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK101" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL101" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM101" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN101" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -23489,6 +26475,36 @@
       <c r="CZ102" t="n">
         <v>0</v>
       </c>
+      <c r="DC102" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD102" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE102" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF102" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG102" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ102" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK102" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL102" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM102" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN102" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -23718,6 +26734,36 @@
       <c r="CZ103" t="n">
         <v>0</v>
       </c>
+      <c r="DC103" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD103" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE103" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF103" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG103" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ103" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK103" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL103" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM103" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN103" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -23947,6 +26993,36 @@
       <c r="CZ104" t="n">
         <v>0</v>
       </c>
+      <c r="DC104" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD104" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE104" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF104" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG104" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ104" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK104" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL104" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM104" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN104" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -24176,6 +27252,36 @@
       <c r="CZ105" t="n">
         <v>0</v>
       </c>
+      <c r="DC105" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD105" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE105" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF105" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG105" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ105" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK105" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL105" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM105" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN105" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -24405,6 +27511,36 @@
       <c r="CZ106" t="n">
         <v>0</v>
       </c>
+      <c r="DC106" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD106" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE106" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF106" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG106" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ106" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK106" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL106" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM106" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN106" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -24634,6 +27770,36 @@
       <c r="CZ107" t="n">
         <v>0</v>
       </c>
+      <c r="DC107" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD107" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE107" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF107" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG107" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ107" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK107" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL107" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM107" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN107" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -24863,6 +28029,36 @@
       <c r="CZ108" t="n">
         <v>0</v>
       </c>
+      <c r="DC108" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD108" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE108" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF108" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG108" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ108" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK108" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL108" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM108" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN108" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -25092,6 +28288,36 @@
       <c r="CZ109" t="n">
         <v>0</v>
       </c>
+      <c r="DC109" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD109" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE109" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF109" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG109" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ109" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK109" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL109" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM109" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN109" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -25321,6 +28547,36 @@
       <c r="CZ110" t="n">
         <v>0</v>
       </c>
+      <c r="DC110" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD110" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE110" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF110" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG110" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ110" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK110" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL110" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM110" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN110" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -25550,6 +28806,36 @@
       <c r="CZ111" t="n">
         <v>0</v>
       </c>
+      <c r="DC111" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD111" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE111" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF111" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG111" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ111" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK111" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL111" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM111" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN111" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -25779,6 +29065,36 @@
       <c r="CZ112" t="n">
         <v>0</v>
       </c>
+      <c r="DC112" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD112" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE112" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF112" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG112" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ112" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK112" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL112" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM112" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN112" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -26008,6 +29324,36 @@
       <c r="CZ113" t="n">
         <v>0</v>
       </c>
+      <c r="DC113" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD113" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE113" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF113" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG113" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ113" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK113" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL113" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM113" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN113" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -26237,6 +29583,36 @@
       <c r="CZ114" t="n">
         <v>0</v>
       </c>
+      <c r="DC114" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD114" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE114" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF114" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG114" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ114" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK114" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL114" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM114" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN114" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -26466,6 +29842,36 @@
       <c r="CZ115" t="n">
         <v>0</v>
       </c>
+      <c r="DC115" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD115" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE115" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF115" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG115" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ115" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK115" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL115" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM115" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN115" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -26695,6 +30101,36 @@
       <c r="CZ116" t="n">
         <v>0</v>
       </c>
+      <c r="DC116" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD116" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE116" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF116" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG116" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ116" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK116" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL116" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM116" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN116" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -26924,6 +30360,36 @@
       <c r="CZ117" t="n">
         <v>0</v>
       </c>
+      <c r="DC117" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD117" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE117" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF117" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG117" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ117" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK117" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL117" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM117" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN117" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -27153,6 +30619,36 @@
       <c r="CZ118" t="n">
         <v>0</v>
       </c>
+      <c r="DC118" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD118" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE118" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF118" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG118" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ118" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK118" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL118" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM118" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN118" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -27382,6 +30878,36 @@
       <c r="CZ119" t="n">
         <v>0</v>
       </c>
+      <c r="DC119" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD119" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE119" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF119" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG119" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ119" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK119" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL119" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM119" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN119" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -27611,6 +31137,36 @@
       <c r="CZ120" t="n">
         <v>0</v>
       </c>
+      <c r="DC120" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD120" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE120" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF120" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG120" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ120" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK120" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL120" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM120" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN120" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -27840,13 +31396,43 @@
       <c r="CZ121" t="n">
         <v>0</v>
       </c>
+      <c r="DC121" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD121" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE121" t="n">
+        <v>0</v>
+      </c>
+      <c r="DF121" t="n">
+        <v>0</v>
+      </c>
+      <c r="DG121" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ121" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK121" t="n">
+        <v>0</v>
+      </c>
+      <c r="DL121" t="n">
+        <v>0</v>
+      </c>
+      <c r="DM121" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN121" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="17">
+    <mergeCell ref="BT1:BY1"/>
+    <mergeCell ref="AR1:AW1"/>
+    <mergeCell ref="P1:U1"/>
     <mergeCell ref="AD1:AI1"/>
-    <mergeCell ref="BT1:BY1"/>
-    <mergeCell ref="P1:U1"/>
-    <mergeCell ref="AR1:AW1"/>
     <mergeCell ref="CA1:CF1"/>
     <mergeCell ref="BM1:BR1"/>
     <mergeCell ref="W1:AB1"/>
@@ -27854,6 +31440,8 @@
     <mergeCell ref="CH1:CM1"/>
     <mergeCell ref="AY1:BD1"/>
     <mergeCell ref="B1:G1"/>
+    <mergeCell ref="DC1:DH1"/>
+    <mergeCell ref="DJ1:DO1"/>
     <mergeCell ref="I1:N1"/>
     <mergeCell ref="BF1:BK1"/>
     <mergeCell ref="CO1:CT1"/>

</xml_diff>